<commit_message>
New Years step-up banner summons
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5.133629820345758</t>
+          <t>5.106760855733459</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.311965175196768</t>
+          <t>6.3034485578175605</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>18.63423667815604</t>
+          <t>2.2898346271860213</t>
         </is>
       </c>
     </row>
@@ -595,12 +595,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.53535234265245</t>
+          <t>0.8509043556650404</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.0408539720695054</t>
+          <t>1.1406434434506174</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.8509131546954856</t>
+          <t>3.9193830948577286</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3.290185032381231</t>
+          <t>3.605623925768521</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>5.050299810830412</t>
+          <t>4.942710365200972</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1.7113917697967995</t>
+          <t>1.710213706139319</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2.7396817278381107</t>
+          <t>3.002342387940007</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>10.77020820601579</t>
+          <t>10.80716535705717</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -820,7 +820,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.9436161385808894</t>
+          <t>1.9636098969079292</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>6.446747524345021</t>
+          <t>6.422778228607779</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.4812344024448405</t>
+          <t>1.2873746001238011</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>23.031295226668618</t>
+          <t>25.23936748037964</t>
         </is>
       </c>
     </row>
@@ -903,12 +903,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>8.548627021991578</t>
+          <t>4.5283260867300825</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>5.883739351590575</t>
+          <t>5.898390779319075</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>4.733804726662532</t>
+          <t>4.7377401587601735</t>
         </is>
       </c>
     </row>
@@ -969,12 +969,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>7.940115468734638</t>
+          <t>6.403559714390065</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>4.0275482685158925</t>
+          <t>3.9993274178410205</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>1.057076985958365</t>
+          <t>1.075278946048834</t>
         </is>
       </c>
     </row>
@@ -1057,12 +1057,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>6.121311684243718</t>
+          <t>5.079492758476391</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>1.646948633257536</t>
+          <t>1.6357838934475382</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3.2974398465700556</t>
+          <t>3.3154010358208756</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.5483641720635385</t>
+          <t>0.6009373209614203</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>4.62498467374853</t>
+          <t>4.6067889422623995</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>0.9497946070644906</t>
+          <t>1.0408539720695054</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10.270649215942775</t>
+          <t>10.254860336918142</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>7.056112711267345</t>
+          <t>7.013988726245884</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>3.7674583264236645</t>
+          <t>3.763595432749121</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>1.846563586895664</t>
+          <t>1.8995892141289812</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>0.9497946070644906</t>
+          <t>1.0408539720695054</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>8.219045183514332</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>5.98791648785982</t>
+          <t>5.998875707712465</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>13.33454837764203</t>
+          <t>13.34544908976272</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2.102264387794558</t>
+          <t>2.09547389220487</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>0.9497946070644906</t>
+          <t>1.0408539720695054</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>3.75</t>
+          <t>4.109522591757166</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>5.373745799717781</t>
+          <t>5.353240576361516</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>3.9331089352926814</t>
+          <t>3.9151307467612106</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>4.735790517442211</t>
+          <t>4.745322983057517</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>10.905083784457336</t>
+          <t>10.853545010989887</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>4.224085265782004</t>
+          <t>4.525259970323061</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>1.5941958216236358</t>
+          <t>1.5471527008601313</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>3.8582543803639955</t>
+          <t>3.8568586918725742</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>20.183131593989238</t>
+          <t>20.106848935985056</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>16.7361406519366</t>
+          <t>16.70593453430589</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4.209236597147822</t>
+          <t>4.240025259904726</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>4.043133674665377</t>
+          <t>4.057366480645557</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>5.2744189091902225</t>
+          <t>5.289165677193682</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>4.159803195494077</t>
+          <t>4.317723948459807</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>5.081279659511366</t>
+          <t>5.092632848742794</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>6.105435629983042</t>
+          <t>6.1045025423440435</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>5.265024340549225</t>
+          <t>5.27391962299201</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>3.8584742389077356</t>
+          <t>3.871483908100057</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>5.816536158485467</t>
+          <t>5.826855101739504</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>6.438632356338654</t>
+          <t>6.434572116543064</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>4.91013918804361</t>
+          <t>5.090705543188559</t>
         </is>
       </c>
     </row>
@@ -2162,7 +2162,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>0.3823555783665645</t>
+          <t>0.3907698589301063</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>11.00671732931579</t>
+          <t>10.65405371412179</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>4.724971371128469</t>
+          <t>4.706748311059482</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>3.3267279851573472</t>
+          <t>3.369981125231632</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>14.582615788593614</t>
+          <t>14.55770449228303</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>7.2074459858020035</t>
+          <t>7.591381556604848</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>3.987225432010584</t>
+          <t>3.9938398055501105</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>1.8715331106811814</t>
+          <t>1.865205404095235</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>0.41006106261296704</t>
+          <t>0.4094741841668128</t>
         </is>
       </c>
     </row>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>2.1134618317034324</t>
+          <t>2.0967726545419723</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>1.1637584361929352</t>
+          <t>1.1619195325231022</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>4.273655406940542</t>
+          <t>4.271870949755012</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>2.54694185254745</t>
+          <t>2.537679162941929</t>
         </is>
       </c>
     </row>
@@ -2575,12 +2575,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>20.79540373807589</t>
+          <t>4.061664223324982</t>
         </is>
       </c>
     </row>
@@ -2624,7 +2624,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>1.7649304822825407</t>
+          <t>1.7263891097903787</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>10.909182199510326</t>
+          <t>11.72205959142498</t>
         </is>
       </c>
     </row>
@@ -2663,12 +2663,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>5.0184165247225465</t>
+          <t>2.2894298861818627</t>
         </is>
       </c>
     </row>
@@ -2685,12 +2685,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>20.770251757696677</t>
+          <t>4.417216300121261</t>
         </is>
       </c>
     </row>
@@ -2751,12 +2751,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>2.631716901415027</t>
+          <t>1.02311457587186</t>
         </is>
       </c>
     </row>
@@ -2839,12 +2839,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>5.038437158956202</t>
+          <t>1.666179903653175</t>
         </is>
       </c>
     </row>
@@ -2861,12 +2861,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>13.39169307044152</t>
+          <t>13.46711058678533</t>
         </is>
       </c>
     </row>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>1.693112981690161</t>
+          <t>1.702620618192863</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>1.6450925161906156</t>
+          <t>1.8028119628842605</t>
         </is>
       </c>
     </row>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>0.27103930228763695</t>
+          <t>0.6417733367788604</t>
         </is>
       </c>
     </row>
@@ -3020,7 +3020,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>1.6080360299086003</t>
+          <t>1.6087972667815311</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>3.881494363024722</t>
+          <t>3.8585139043854424</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>6.746909173979117</t>
+          <t>6.722389146749922</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>1.3688619479542474</t>
+          <t>1.3685276335420795</t>
         </is>
       </c>
     </row>
@@ -3147,12 +3147,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>0.2597371646463313</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>3.291386803864336</t>
+          <t>3.283388614725382</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>2.178854658996549</t>
+          <t>2.1716975202363002</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>1.5011711939700034</t>
+          <t>1.6450925161906156</t>
         </is>
       </c>
     </row>
@@ -3614,7 +3614,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>1.348498530131189</t>
+          <t>1.345896568004517</t>
         </is>
       </c>
     </row>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>1.5946255641519465</t>
+          <t>1.5911403726015974</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>3.802096685352211</t>
+          <t>3.7869757366020487</t>
         </is>
       </c>
     </row>
@@ -3741,12 +3741,12 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>2.7294066999974573</t>
+          <t>3.1980268189557073</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>1.9631134912983494</t>
+          <t>1.9418391658543042</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>2.041427081834195</t>
+          <t>2.0295968474360158</t>
         </is>
       </c>
     </row>
@@ -3895,12 +3895,12 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>15.605223720903039</t>
+          <t>8.771631716820409</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>2.4929233969313813</t>
+          <t>2.4968155834561685</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>10.472427296448066</t>
+          <t>10.506442875864757</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>7.983781354105177</t>
+          <t>7.917247916334581</t>
         </is>
       </c>
     </row>
@@ -4005,12 +4005,12 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>11.04946658485552</t>
+          <t>9.30045711428055</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>11.6682784237647</t>
+          <t>12.045081018239562</t>
         </is>
       </c>
     </row>
@@ -4181,12 +4181,12 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>2.7701506341537043</t>
+          <t>4.952928154885152</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>4.199510984798888</t>
+          <t>4.175098205808009</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>0.7845459579504102</t>
+          <t>0.7853750537906965</t>
         </is>
       </c>
     </row>
@@ -4494,7 +4494,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>1.8790564119467172</t>
+          <t>1.8697348939400107</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>1.997477213295575</t>
+          <t>1.8510659297872039</t>
         </is>
       </c>
     </row>
@@ -4604,7 +4604,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>0.35169694648809013</t>
+          <t>0.3506627107087894</t>
         </is>
       </c>
     </row>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>1.3901707743130478</t>
+          <t>1.3962938354731715</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>0.2763556453369372</t>
+          <t>0.27565202861934174</t>
         </is>
       </c>
     </row>
@@ -4912,7 +4912,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>0.3594627758224842</t>
+          <t>0.3584964751461577</t>
         </is>
       </c>
     </row>
@@ -4934,7 +4934,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>0.9644664829408622</t>
+          <t>0.9622408297238838</t>
         </is>
       </c>
     </row>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>1.3257471893775845</t>
+          <t>1.3147456909817492</t>
         </is>
       </c>
     </row>
@@ -4978,7 +4978,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>0.29976631214742</t>
+          <t>0.2984030756340863</t>
         </is>
       </c>
     </row>
@@ -5044,7 +5044,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>1.3368107998542242</t>
+          <t>1.3345206379312444</t>
         </is>
       </c>
     </row>
@@ -5083,12 +5083,12 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>9.422258795321191</t>
+          <t>2.603889535896377</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>68.41057251449232</t>
+          <t>68.384975027314</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>13.528928568701819</t>
+          <t>13.46649034981179</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>16.261087209603293</t>
+          <t>16.272873307687146</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>90.88736004056815</t>
+          <t>90.8598354587483</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>5.494731875911529</t>
+          <t>5.5064559757110665</t>
         </is>
       </c>
     </row>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>0.7167694602299738</t>
+          <t>0.7130846624900848</t>
         </is>
       </c>
     </row>
@@ -5440,7 +5440,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>0.9277362261075695</t>
+          <t>0.9229022955793283</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>2.7168135117211936</t>
+          <t>2.701136743557967</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>56.57631378646745</t>
+          <t>56.53172769036435</t>
         </is>
       </c>
     </row>
@@ -5523,12 +5523,12 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>3.9109581273138696</t>
+          <t>3.559163934909575</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>18.95130385418102</t>
+          <t>18.90467223905086</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>20.36475538403137</t>
+          <t>20.38595159587068</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>0.790303805379419</t>
+          <t>0.7011195136179875</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>2.7341948532785674</t>
+          <t>2.723204167883055</t>
         </is>
       </c>
     </row>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>3.193238201663818</t>
+          <t>3.194061935352062</t>
         </is>
       </c>
     </row>
@@ -5743,12 +5743,12 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>3.3226808377915393</t>
+          <t>2.8780204745867977</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>6.600464299154262</t>
+          <t>6.583058890084688</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>2.5823793475340975</t>
+          <t>2.2413878665082</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>7.563651281401206</t>
+          <t>7.568862629096073</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>56.06335663576398</t>
+          <t>55.93280572880043</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>7.493480722310937</t>
+          <t>7.518236151299324</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>4.665409764655038</t>
+          <t>4.668714147804753</t>
         </is>
       </c>
     </row>
@@ -5985,12 +5985,12 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>7.27455146609668</t>
+          <t>1.9121920057156248</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>13.989112385832605</t>
+          <t>13.943878674262644</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>79.37980440628567</t>
+          <t>79.3991917326151</t>
         </is>
       </c>
     </row>
@@ -6095,12 +6095,12 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>12.351699819684047</t>
+          <t>9.193224297153941</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>9.441713703653079</t>
+          <t>9.436249469861622</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>1.271842190795139</t>
+          <t>1.286914627431307</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>7.867856932263585</t>
+          <t>7.864796419950402</t>
         </is>
       </c>
     </row>
@@ -6183,12 +6183,12 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>2.3000652730717484</t>
+          <t>1.6552346410856202</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>44.08976579666836</t>
+          <t>44.06209112105566</t>
         </is>
       </c>
     </row>
@@ -6342,7 +6342,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>0.45719572198636393</t>
+          <t>0.455606340631742</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>10.072217046945735</t>
+          <t>10.49242316137087</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>5.871808504264908</t>
+          <t>5.7971726291867025</t>
         </is>
       </c>
     </row>
@@ -6584,7 +6584,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>7.295696464584026</t>
+          <t>7.288484078107734</t>
         </is>
       </c>
     </row>
@@ -6623,12 +6623,12 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>13.21967917628702</t>
+          <t>2.683232966951021</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>38.73843436373674</t>
+          <t>38.6925361595361</t>
         </is>
       </c>
     </row>
@@ -6667,12 +6667,12 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>6.785314304133419</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>4.676475017951436</t>
+          <t>4.6909160491912365</t>
         </is>
       </c>
     </row>
@@ -6716,7 +6716,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>7.381496065748709</t>
+          <t>6.300848933217064</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>8.4172333341793</t>
+          <t>8.390385893517223</t>
         </is>
       </c>
     </row>
@@ -6826,7 +6826,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>2.01928877692962</t>
+          <t>2.0130310073965876</t>
         </is>
       </c>
     </row>
@@ -6848,7 +6848,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>1.8232675119921165</t>
+          <t>1.8168332826034466</t>
         </is>
       </c>
     </row>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>1.3258551990165905</t>
+          <t>1.32397634149733</t>
         </is>
       </c>
     </row>
@@ -6914,7 +6914,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>3.027338627344232</t>
+          <t>3.3142357491424725</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>4.187207021857878</t>
+          <t>4.127900841355631</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>14.88979892747012</t>
+          <t>14.90771088371332</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>10.757092689556693</t>
+          <t>10.294606217627724</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>7.730366228530272</t>
+          <t>7.784124963985917</t>
         </is>
       </c>
     </row>
@@ -7222,7 +7222,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>4.27753708689226</t>
+          <t>4.263045639939591</t>
         </is>
       </c>
     </row>
@@ -7244,7 +7244,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>2.292367904836176</t>
+          <t>2.3470633337378586</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>2.9026092706660904</t>
+          <t>2.9033869146013274</t>
         </is>
       </c>
     </row>
@@ -7354,7 +7354,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>2.5778830741057184</t>
+          <t>2.5622470197007785</t>
         </is>
       </c>
     </row>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>2.1583097329992693</t>
+          <t>2.15946438831293</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>3.827810709789974</t>
+          <t>3.8428264745136733</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>63.32151495965024</t>
+          <t>63.15154862340032</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>8.721206634387585</t>
+          <t>8.78377881722487</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Try to use filtered rainbow stats for evaluations
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5.106760855733459</t>
+          <t>1.4433756729740643</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.3034485578175605</t>
+          <t>3.8315856827956516</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2.2898346271860213</t>
+          <t>0.37049174364188264</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.8509043556650404</t>
+          <t>0.38021448115020573</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.9193830948577286</t>
+          <t>0.3147744932624183</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>4.942710365200972</t>
+          <t>0.5272519943537441</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1.710213706139319</t>
+          <t>0.5003903979900011</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>10.80716535705717</t>
+          <t>2.8043741644866276</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.9636098969079292</t>
+          <t>0.34695132402316853</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>6.422778228607779</t>
+          <t>0.7604289623004115</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.2873746001238011</t>
+          <t>0.6009373209614203</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>4.5283260867300825</t>
+          <t>0.5067807888762054</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>5.898390779319075</t>
+          <t>5.833333333333332</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>4.7377401587601735</t>
+          <t>0.8333333333333333</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>6.403559714390065</t>
+          <t>0.40930011810409317</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>3.9993274178410205</t>
+          <t>0.3054626683083246</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>1.075278946048834</t>
+          <t>0.23130088268211232</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>5.079492758476391</t>
+          <t>0.692127162153197</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>1.6357838934475382</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3.3154010358208756</t>
+          <t>0.6331964047096604</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>4.6067889422623995</t>
+          <t>1.096728344127077</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10.254860336918142</t>
+          <t>4.717602726921022</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>7.013988726245884</t>
+          <t>1.2014798145840209</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>3.763595432749121</t>
+          <t>0.8344960168122482</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>5.998875707712465</t>
+          <t>4.166424863988899</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>13.34544908976272</t>
+          <t>7.005465571860014</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2.09547389220487</t>
+          <t>1.5817559830612322</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>5.353240576361516</t>
+          <t>2.1794089044126794</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>3.9151307467612106</t>
+          <t>1.3171015982511909</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>4.745322983057517</t>
+          <t>4.044607433712034</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>10.853545010989887</t>
+          <t>2.1266332316247567</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>4.525259970323061</t>
+          <t>6.921858845594372</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>1.5471527008601313</t>
+          <t>1.3698408639190554</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>3.8568586918725742</t>
+          <t>1.946076891031236</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>20.106848935985056</t>
+          <t>10.427301145948132</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>16.70593453430589</t>
+          <t>15.408265119679609</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4.240025259904726</t>
+          <t>13.993169421959792</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>4.057366480645557</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>5.289165677193682</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>4.317723948459807</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>5.092632848742794</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>6.1045025423440435</t>
+          <t>0.3194783495112404</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>5.27391962299201</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>3.871483908100057</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>5.826855101739504</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>6.434572116543064</t>
+          <t>0.3527209445716921</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>5.090705543188559</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2157,12 +2157,12 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>0.3907698589301063</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>10.65405371412179</t>
+          <t>1.207231315369677</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>4.706748311059482</t>
+          <t>0.4306794675390997</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>3.369981125231632</t>
+          <t>11.000438787530385</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>14.55770449228303</t>
+          <t>4.548537523772909</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>7.591381556604848</t>
+          <t>1.619106178774786</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>3.9938398055501105</t>
+          <t>1.733403185876587</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>1.865205404095235</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>0.4094741841668128</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>2.0967726545419723</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>1.1619195325231022</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>4.271870949755012</t>
+          <t>1.284026265426592</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>2.537679162941929</t>
+          <t>0.23433266072009618</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>4.061664223324982</t>
+          <t>3.41039337680412</t>
         </is>
       </c>
     </row>
@@ -2624,7 +2624,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>1.7263891097903787</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>11.72205959142498</t>
+          <t>6.658766671177399</t>
         </is>
       </c>
     </row>
@@ -2668,7 +2668,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>2.2894298861818627</t>
+          <t>0.2537641061248578</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>4.417216300121261</t>
+          <t>3.209674629674881</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>1.02311457587186</t>
+          <t>0.7908779915306161</t>
         </is>
       </c>
     </row>
@@ -2844,7 +2844,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>1.666179903653175</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>13.46711058678533</t>
+          <t>1.5033780612921988</t>
         </is>
       </c>
     </row>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>1.702620618192863</t>
+          <t>5.615202818334916</t>
         </is>
       </c>
     </row>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>0.6417733367788604</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -3020,7 +3020,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>1.6087972667815311</t>
+          <t>1.25</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>3.8585139043854424</t>
+          <t>0.3771788599082533</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>6.722389146749922</t>
+          <t>0.83642401962363</t>
         </is>
       </c>
     </row>
@@ -3081,12 +3081,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>1.3685276335420795</t>
+          <t>0.34695132402316853</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>3.283388614725382</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>2.1716975202363002</t>
+          <t>0.6009373209614203</t>
         </is>
       </c>
     </row>
@@ -3614,7 +3614,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>1.345896568004517</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>1.5911403726015974</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>3.7869757366020487</t>
+          <t>0.26303249048250205</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>3.1980268189557073</t>
+          <t>1.4433756729740643</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>1.9418391658543042</t>
+          <t>0.24056261216234406</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>2.0295968474360158</t>
+          <t>0.39648497749678946</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>8.771631716820409</t>
+          <t>0.9597738102390321</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>2.4968155834561685</t>
+          <t>0.4678396196778478</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>10.506442875864757</t>
+          <t>9.62612522673948</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>7.917247916334581</t>
+          <t>6.6768458343079296</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>9.30045711428055</t>
+          <t>0.8033668676971861</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>12.045081018239562</t>
+          <t>1.477458277655874</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>4.952928154885152</t>
+          <t>1.5081722901323624</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>4.175098205808009</t>
+          <t>0.6252684993337903</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>0.7853750537906965</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -4494,7 +4494,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>1.8697348939400107</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>1.8510659297872039</t>
+          <t>0.42873867904681484</t>
         </is>
       </c>
     </row>
@@ -4604,7 +4604,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>0.3506627107087894</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>1.3962938354731715</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>0.27565202861934174</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -4912,7 +4912,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>0.3584964751461577</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -4934,7 +4934,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>0.9622408297238838</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>1.3147456909817492</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -4978,7 +4978,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>0.2984030756340863</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5044,7 +5044,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>1.3345206379312444</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5088,7 +5088,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>2.603889535896377</t>
+          <t>0.39918667479354514</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>68.384975027314</t>
+          <t>23.07484559429439</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>13.46649034981179</t>
+          <t>0.5810942076799046</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>16.272873307687146</t>
+          <t>0.917241423058644</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>90.8598354587483</t>
+          <t>73.25793524352409</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>5.5064559757110665</t>
+          <t>5.192621977965413</t>
         </is>
       </c>
     </row>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>0.7130846624900848</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5440,7 +5440,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>0.9229022955793283</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>2.701136743557967</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5501,12 +5501,12 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>56.53172769036435</t>
+          <t>12.47108892582653</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>3.559163934909575</t>
+          <t>2.8846725909179654</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>18.90467223905086</t>
+          <t>1.061820575124136</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>20.38595159587068</t>
+          <t>1.2302546534920695</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>0.7011195136179875</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>2.723204167883055</t>
+          <t>0.4309693399108413</t>
         </is>
       </c>
     </row>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>3.194061935352062</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5748,7 +5748,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>2.8780204745867977</t>
+          <t>0.283509554710371</t>
         </is>
       </c>
     </row>
@@ -5765,12 +5765,12 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>6.583058890084688</t>
+          <t>7.042407236577326</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>2.2413878665082</t>
+          <t>0.438276820359319</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>7.568862629096073</t>
+          <t>21.82212294095504</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>55.93280572880043</t>
+          <t>11.965758906772441</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>7.518236151299324</t>
+          <t>0.37420850780809073</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>4.668714147804753</t>
+          <t>1.6402745764253097</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>1.9121920057156248</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>13.943878674262644</t>
+          <t>19.149144591923193</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>79.3991917326151</t>
+          <t>41.23068539651286</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>9.193224297153941</t>
+          <t>9.569294067353205</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>9.436249469861622</t>
+          <t>2.7328637071264397</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>1.286914627431307</t>
+          <t>4.302266142481382</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>7.864796419950402</t>
+          <t>8.33269484608762</t>
         </is>
       </c>
     </row>
@@ -6188,7 +6188,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>1.6552346410856202</t>
+          <t>0.20786901634898713</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>44.06209112105566</t>
+          <t>6.250569009745783</t>
         </is>
       </c>
     </row>
@@ -6342,7 +6342,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>0.455606340631742</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>10.49242316137087</t>
+          <t>0.8965952414479735</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>5.7971726291867025</t>
+          <t>1.2715819235853518</t>
         </is>
       </c>
     </row>
@@ -6584,7 +6584,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>7.288484078107734</t>
+          <t>1.8436698954755606</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>2.683232966951021</t>
+          <t>0.21366096239331467</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>38.6925361595361</t>
+          <t>4.566547055989128</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>4.6909160491912365</t>
+          <t>0.7713937200103896</t>
         </is>
       </c>
     </row>
@@ -6716,7 +6716,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>6.300848933217064</t>
+          <t>1.5160197967508124</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>8.390385893517223</t>
+          <t>1.4112487804235425</t>
         </is>
       </c>
     </row>
@@ -6826,7 +6826,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>2.0130310073965876</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6848,7 +6848,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>1.8168332826034466</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>1.32397634149733</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6914,7 +6914,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>3.3142357491424725</t>
+          <t>0.3202892787021886</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>4.127900841355631</t>
+          <t>0.28987016646647434</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>14.90771088371332</t>
+          <t>0.6936518776479348</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>10.294606217627724</t>
+          <t>3.7687579112523557</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>7.784124963985917</t>
+          <t>15.673794701454877</t>
         </is>
       </c>
     </row>
@@ -7222,7 +7222,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>4.263045639939591</t>
+          <t>0.23216137540579487</t>
         </is>
       </c>
     </row>
@@ -7244,7 +7244,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>2.3470633337378586</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>2.9033869146013274</t>
+          <t>8.229541321019411</t>
         </is>
       </c>
     </row>
@@ -7354,7 +7354,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>2.5622470197007785</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>2.15946438831293</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>3.8428264745136733</t>
+          <t>11.4095166975838</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>63.15154862340032</t>
+          <t>17.52191206655069</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>8.78377881722487</t>
+          <t>25.09186239626196</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove no eval units from all eval
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.13035243497669</t>
+          <t>0.9622504486493763</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.687166908878922</t>
+          <t>4.342045710791501</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.6763382793410448</t>
+          <t>0.3953354735858779</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.7273981480951476</t>
+          <t>0.37972838858737</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1.1607258857190328</t>
+          <t>0.6338296412257199</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.4497687650439972</t>
+          <t>0.24521502121384797</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.479457202414675</t>
+          <t>0.8118512094156047</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.9195049003918658</t>
+          <t>0.4991767897119047</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.5723323881399061</t>
+          <t>0.5555555555555556</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.9636363836562498</t>
+          <t>0.48046017102042543</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.6998326178037755</t>
+          <t>0.36091376273641906</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1.4464161067266033</t>
+          <t>0.828721712832946</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0.423608940401042</t>
+          <t>0.42213093647310695</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0.9456853491746132</t>
+          <t>0.7311522294180514</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>7.040713360595911</t>
+          <t>4.999084995730655</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2.324169321382072</t>
+          <t>1.3812978562310492</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>1.5630522834301912</t>
+          <t>0.9737779346916476</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>5.812687726030049</t>
+          <t>4.576340802425589</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>3.4671557950874483</t>
+          <t>2.411137889872512</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>4.064491929470826</t>
+          <t>2.4868311017164832</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>7.757458938528724</t>
+          <t>7.520674054328197</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>3.0255043311146177</t>
+          <t>2.2208254241038006</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>15.98991650341617</t>
+          <t>11.922740160760736</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>19.474789851488108</t>
+          <t>16.52125128067391</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>11.10260636679942</t>
+          <t>13.939410246169388</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>0.2467152746633819</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.36616293015606644</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0.2673594280547849</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0.3512138775199222</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.8041805562575471</t>
+          <t>0.3878668903912969</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>0.3745990584132196</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>0.22924405978254223</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>0.4331538676973064</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.8832334829444907</t>
+          <t>0.4299441886243924</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0.3423581159750052</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>2.550682610299318</t>
+          <t>1.413951141061644</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.9784306532026353</t>
+          <t>0.5225681382126862</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>7.8705396123937135</t>
+          <t>10.075412458458345</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>7.67259754386958</t>
+          <t>5.092253580364981</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>0.4363377027486233</t>
+          <t>0.23652425821716255</t>
         </is>
       </c>
     </row>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>0.3621660072766329</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>2.185739268533088</t>
+          <t>1.4377630006974043</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>0.570410048452261</t>
+          <t>0.3067060356747502</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>4.51471423833809</t>
+          <t>3.6970792968836914</t>
         </is>
       </c>
     </row>
@@ -2624,7 +2624,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>0.3753303867223179</t>
+          <t>0.20083125009975278</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>10.082130485281871</t>
+          <t>7.668569463790311</t>
         </is>
       </c>
     </row>
@@ -2668,7 +2668,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>0.5184846252728982</t>
+          <t>0.28485488970007716</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>4.60800512602901</t>
+          <t>3.694187189432139</t>
         </is>
       </c>
     </row>
@@ -2844,7 +2844,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>0.20294887292889363</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>3.2563889897573697</t>
+          <t>1.8082893378883762</t>
         </is>
       </c>
     </row>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>4.057772379809442</t>
+          <t>5.1219867006205755</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>0.8438075495851147</t>
+          <t>0.4566464740200867</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>1.7469445579159992</t>
+          <t>0.9823201801210706</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>0.3862564811011311</t>
+          <t>0.23130088268211232</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>0.39540686349247156</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>0.5808333396296068</t>
+          <t>0.40062488064094687</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>0.6358738213023891</t>
+          <t>0.3238865577238284</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>0.2969663962880267</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>0.7957293638397427</t>
+          <t>0.4891345027892857</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>2.1608886148029627</t>
+          <t>1.1970754661452816</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.7739844184695102</t>
+          <t>0.4613680669038098</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>12.657290892932515</t>
+          <t>10.71777168709035</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>9.04579917265669</t>
+          <t>7.541977052152761</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>1.8889006654743001</t>
+          <t>1.001190568665706</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>1.290880752205205</t>
+          <t>0.9849721851039159</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>2.8105355051028598</t>
+          <t>1.8831840220330058</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>1.2262094060492763</t>
+          <t>0.7093081478178842</t>
         </is>
       </c>
     </row>
@@ -4494,7 +4494,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>0.2082141241812305</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>0.7724559615456688</t>
+          <t>0.4832589025331533</t>
         </is>
       </c>
     </row>
@@ -5088,7 +5088,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>0.8287301751596179</t>
+          <t>0.48694868758564613</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>35.09037587964151</t>
+          <t>25.54986538051179</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>1.472180751253519</t>
+          <t>0.6923774397133089</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>2.1473907166201855</t>
+          <t>1.0636285448632121</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>79.23473227296435</t>
+          <t>73.95126253128637</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>6.645773008929873</t>
+          <t>5.721761286212494</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>0.3332190687035447</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>16.08654859925314</t>
+          <t>13.928229664903663</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>3.9677372466116134</t>
+          <t>3.2801321746669823</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>2.254240374970384</t>
+          <t>1.104858409808856</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>2.896098981414223</t>
+          <t>1.45570369442252</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>0.8750731377407015</t>
+          <t>0.5121226742473157</t>
         </is>
       </c>
     </row>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>0.2803396845646927</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5748,7 +5748,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>0.6304795994556969</t>
+          <t>0.34095116205005327</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>9.126195600115603</t>
+          <t>7.799577162910593</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>0.8943137479411818</t>
+          <t>0.548380312495463</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>17.500045059571995</t>
+          <t>20.951710305018132</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>20.12823422293119</t>
+          <t>13.03909814425472</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.5959099391754378</t>
+          <t>0.2578443263709956</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>2.778459023786683</t>
+          <t>1.9112817559265243</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>0.2427627632524697</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>21.55760770297422</t>
+          <t>20.52247829191431</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>53.7949416742517</t>
+          <t>44.07029818486402</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>11.658684886290935</t>
+          <t>10.021335583598374</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>4.7515106649514545</t>
+          <t>3.116958502658347</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>3.0990526094544055</t>
+          <t>3.970854774127795</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>10.188187338372611</t>
+          <t>8.978613961864628</t>
         </is>
       </c>
     </row>
@@ -6188,7 +6188,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>0.4563781145206107</t>
+          <t>0.258976741950957</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>12.39103246916242</t>
+          <t>7.415552913345212</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>2.0295192869055074</t>
+          <t>1.070626853391384</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>2.4046652098732744</t>
+          <t>1.5076420851176353</t>
         </is>
       </c>
     </row>
@@ -6584,7 +6584,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>3.4067090557193715</t>
+          <t>2.199395756501703</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>0.4769185751491569</t>
+          <t>0.2482044371852905</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>9.652528583273355</t>
+          <t>5.576882766842663</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>1.546580029501185</t>
+          <t>0.9236372922475216</t>
         </is>
       </c>
     </row>
@@ -6716,7 +6716,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>2.9763319915404813</t>
+          <t>1.897403895551504</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>2.5725602644416954</t>
+          <t>1.508961320276801</t>
         </is>
       </c>
     </row>
@@ -6826,7 +6826,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>0.3874158721189018</t>
+          <t>0.20245051461732713</t>
         </is>
       </c>
     </row>
@@ -6848,7 +6848,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>0.3341889439279662</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>0.22783326035598894</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6914,7 +6914,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>0.7343951737968348</t>
+          <t>0.39819888247219903</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.6789455150943496</t>
+          <t>0.34447478728723535</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>1.844658373955503</t>
+          <t>0.8865254422510852</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>6.344429447475912</t>
+          <t>4.3882802625126365</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>15.083271283263501</t>
+          <t>15.929520204745108</t>
         </is>
       </c>
     </row>
@@ -7222,7 +7222,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>0.6225005855869545</t>
+          <t>0.3039933650932868</t>
         </is>
       </c>
     </row>
@@ -7244,7 +7244,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>0.21538254896119302</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>6.376912643056755</t>
+          <t>7.993784059209929</t>
         </is>
       </c>
     </row>
@@ -7354,7 +7354,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>0.37834117088036473</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>0.361530496176804</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>8.959757520829507</t>
+          <t>10.795079637392085</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>29.68969956122453</t>
+          <t>20.79334522714615</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>20.143508262641348</t>
+          <t>23.929752317313536</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Slightly adjustment to MIN_EVALUATION
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.124441370296634</t>
+          <t>1.1632203356842548</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.675788972523023</t>
+          <t>5.74914246859203</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.6732760002958607</t>
+          <t>0.6933100900325817</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.7233373989994243</t>
+          <t>0.7500114526089093</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1.154728682206246</t>
+          <t>1.194063560225489</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.44743860006644415</t>
+          <t>0.4627225502833369</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.471880159463147</t>
+          <t>1.5215687500986799</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.9147042326284731</t>
+          <t>0.9461974690558669</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.5686776564175712</t>
+          <t>0.5927488367852094</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.9578515317006229</t>
+          <t>0.9959055712866902</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.6958475423866107</t>
+          <t>0.7220346966656827</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1.43959343660655</t>
+          <t>1.4842640127144664</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0.42213093647310695</t>
+          <t>0.4385645394024833</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0.940630444623042</t>
+          <t>0.9738067157559511</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>7.02182006166832</t>
+          <t>7.144263707438208</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2.3140090106469433</t>
+          <t>2.3804367128963033</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>1.5569208938202115</t>
+          <t>1.5969258863961242</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>5.802711268250739</t>
+          <t>5.86684962909143</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>3.4571811999921853</t>
+          <t>3.5218995493540364</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>4.047837462048418</t>
+          <t>4.15659423618686</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>7.758455806153715</t>
+          <t>7.750998428569606</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>3.0183454990473297</t>
+          <t>3.0646338968258195</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>15.95408800937209</t>
+          <t>16.18565127955781</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>19.45418431146278</t>
+          <t>19.58546463280412</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>11.126550965973195</t>
+          <t>10.97188176045917</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>0.24477508018104926</t>
+          <t>0.2576126727706408</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.3633958283217983</t>
+          <t>0.3816886267129263</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0.26527351420922346</t>
+          <t>0.2790728234418501</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0.34854829339911103</t>
+          <t>0.3661716361554796</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.799110489599748</t>
+          <t>0.8324955761800378</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>0.3717748876275772</t>
+          <t>0.39044399570676713</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>0.22742825614930617</t>
+          <t>0.23944474634897922</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>0.42993767907758373</t>
+          <t>0.4511911813137516</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.8777383267343062</t>
+          <t>0.9139129435792932</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0.3397529123862247</t>
+          <t>0.3569780444684485</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>2.537855575218365</t>
+          <t>2.6219446000856785</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.9731739727437042</t>
+          <t>1.0076780739436955</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>7.888229341763279</t>
+          <t>7.7741926485242345</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>7.647073347372748</t>
+          <t>7.813128561000995</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>0.43405372873140086</t>
+          <t>0.4490377014074145</t>
         </is>
       </c>
     </row>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>0.36008382201028205</t>
+          <t>0.37376900294907506</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>2.178296851294403</t>
+          <t>2.226730392159442</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>0.5673814186742281</t>
+          <t>0.5872562045786811</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>4.508596219157749</t>
+          <t>4.547746126274898</t>
         </is>
       </c>
     </row>
@@ -2624,7 +2624,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>0.37332065638138</t>
+          <t>0.38651126366711397</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>10.06154948022761</t>
+          <t>10.194302984017652</t>
         </is>
       </c>
     </row>
@@ -2668,7 +2668,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>0.5158354122136073</t>
+          <t>0.5332074076287597</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>4.600867175447419</t>
+          <t>4.646666071876432</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>3.2400595612612646</t>
+          <t>3.347105324426791</t>
         </is>
       </c>
     </row>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>4.066677632166805</t>
+          <t>4.0091754532504025</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>0.839377421658433</t>
+          <t>0.8684430277247774</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>1.7383950362093186</t>
+          <t>1.7944121567399174</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>0.3839877849516608</t>
+          <t>0.398905088747936</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>0.392809093067169</t>
+          <t>0.40992857944695044</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>0.5779873703579028</t>
+          <t>0.5966344830830783</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>0.6321810568427588</t>
+          <t>0.656456667643524</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>0.29517036870115687</t>
+          <t>0.30698657442059646</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>0.7925065494497072</t>
+          <t>0.8135466312285242</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>2.150010254123576</t>
+          <t>2.221325310804554</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.7706236606071899</t>
+          <t>0.7925930191586267</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>12.643859477691539</t>
+          <t>12.729381185862785</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>9.034980223330752</t>
+          <t>9.104039564777292</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>1.8786157630277232</t>
+          <t>1.9461433583296</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>1.2822759515097457</t>
+          <t>1.339011167886784</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>2.8014584479562363</t>
+          <t>2.8604741155293727</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>1.2205362593098732</t>
+          <t>1.2576666381066102</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>0.7694569392266688</t>
+          <t>0.7890205857781263</t>
         </is>
       </c>
     </row>
@@ -5088,7 +5088,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>0.8250187361271202</t>
+          <t>0.8492947561020858</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>34.9997062552446</t>
+          <t>35.58871430050539</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>1.46253048138868</t>
+          <t>1.526137445039931</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>2.1343133526326974</t>
+          <t>2.2203837165334566</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>79.19189246592778</t>
+          <t>79.46819379893032</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>6.639752648318337</t>
+          <t>6.677922298443082</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>0.3310603993055736</t>
+          <t>0.3452820652378276</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>16.0725973125051</t>
+          <t>16.16100728365175</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>3.9627019796096636</t>
+          <t>3.994878973839855</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>2.24029826333001</t>
+          <t>2.332087798595968</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>2.878846825163033</t>
+          <t>2.992345594700509</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>0.8711209574782511</t>
+          <t>0.8969757909078236</t>
         </is>
       </c>
     </row>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>0.27832716171543437</t>
+          <t>0.2916144138971628</t>
         </is>
       </c>
     </row>
@@ -5748,7 +5748,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>0.6271654514443719</t>
+          <t>0.6489096635721943</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>9.11729640413187</t>
+          <t>9.173835535794307</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>0.8906706231432799</t>
+          <t>0.9144572818147054</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>17.531806014972908</t>
+          <t>17.325912253283136</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>20.05520571791057</t>
+          <t>20.53159736229587</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.5915629962219479</t>
+          <t>0.6202779401872459</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>2.7701804175457543</t>
+          <t>2.8239274093078373</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>0.24121088401802407</t>
+          <t>0.25143213720713353</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>21.556637448725862</t>
+          <t>21.560197939339552</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>53.709798710791695</t>
+          <t>54.260745622118804</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>11.647866205765629</t>
+          <t>11.716529834381301</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>4.735192052853999</t>
+          <t>4.8414122341093195</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>3.1061074213233035</t>
+          <t>3.060614417989638</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>10.181046682367175</t>
+          <t>10.225985825863326</t>
         </is>
       </c>
     </row>
@@ -6188,7 +6188,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>0.4541843818255549</t>
+          <t>0.468552665607584</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>12.33706606063009</t>
+          <t>12.6901030696256</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>2.0183783136395994</t>
+          <t>2.091538766545579</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>2.3953757348375295</t>
+          <t>2.4559696598505494</t>
         </is>
       </c>
     </row>
@@ -6584,7 +6584,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>3.3944970322471564</t>
+          <t>3.474046199102666</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>0.47424293009349117</t>
+          <t>0.49182019672414</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>9.607352248140325</t>
+          <t>9.903246178687269</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>1.5398910877009373</t>
+          <t>1.5836139504558506</t>
         </is>
       </c>
     </row>
@@ -6716,7 +6716,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>2.9653052281241186</t>
+          <t>3.0371764186419536</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>2.5609911516632726</t>
+          <t>2.6366712128308056</t>
         </is>
       </c>
     </row>
@@ -6826,7 +6826,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>0.38525691865339035</t>
+          <t>0.3994379847761073</t>
         </is>
       </c>
     </row>
@@ -6848,7 +6848,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>0.332295463461318</t>
+          <t>0.34473680751808716</t>
         </is>
       </c>
     </row>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>0.226508533909614</t>
+          <t>0.23521722733873496</t>
         </is>
       </c>
     </row>
@@ -6914,7 +6914,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>0.7305527592087238</t>
+          <t>0.7557606804612691</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.6749783130345265</t>
+          <t>0.701061217451547</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>1.8329236910574052</t>
+          <t>1.9102232153798058</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>6.325835301318699</t>
+          <t>6.446525834735647</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>15.095872302861409</t>
+          <t>15.012770254768562</t>
         </is>
       </c>
     </row>
@@ -7222,7 +7222,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>0.6186473237698054</t>
+          <t>0.6440101804612461</t>
         </is>
       </c>
     </row>
@@ -7244,7 +7244,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>0.21384670445630807</t>
+          <t>0.22398523729625683</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>6.389848731834391</t>
+          <t>6.306455587443907</t>
         </is>
       </c>
     </row>
@@ -7354,7 +7354,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>0.3760679050285543</t>
+          <t>0.39102199088865663</t>
         </is>
       </c>
     </row>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>0.35943593323950984</t>
+          <t>0.37320453901835404</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>8.976480401511711</t>
+          <t>8.868120651660051</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>29.602822267697942</t>
+          <t>30.16796949021078</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>20.178849467581784</t>
+          <t>19.949606788869488</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add names to summonRatings
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.1632203356842548</t>
+          <t>1.0491344499275668</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.74914246859203</t>
+          <t>4.91911958947221</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.6933100900325817</t>
+          <t>0.7575305364633911</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.7500114526089093</t>
+          <t>0.8947948165783295</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1.194063560225489</t>
+          <t>0.870027040520301</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.4627225502833369</t>
+          <t>0.37778710682941896</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.5215687500986799</t>
+          <t>1.6167196805330453</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.9461974690558669</t>
+          <t>0.7892017907472955</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.5927488367852094</t>
+          <t>0.6366095495548054</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.9959055712866902</t>
+          <t>0.631148730999064</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.7220346966656827</t>
+          <t>0.7358047908330718</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1.4842640127144664</t>
+          <t>1.5114677929462919</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0.4385645394024833</t>
+          <t>0.5676069659720463</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0.9738067157559511</t>
+          <t>1.168370703883813</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>7.144263707438208</t>
+          <t>7.465188252147819</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2.3804367128963033</t>
+          <t>2.2591356001118754</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>1.5969258863961242</t>
+          <t>0.632638458353207</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>5.86684962909143</t>
+          <t>6.55353247046364</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>3.5218995493540364</t>
+          <t>3.5218343341973037</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>0.8780677321674606</t>
+          <t>0.9500928858883221</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>4.15659423618686</t>
+          <t>2.1428130926831703</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>7.750998428569606</t>
+          <t>5.059201245034552</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>3.0646338968258195</t>
+          <t>1.6614286173001709</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>16.18565127955781</t>
+          <t>6.841962765151133</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>19.58546463280412</t>
+          <t>15.448036460632839</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>10.97188176045917</t>
+          <t>8.806524182428788</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>0.2576126727706408</t>
+          <t>0.3634574449933109</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.3816886267129263</t>
+          <t>0.42771252395482945</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0.2790728234418501</t>
+          <t>0.3853812200944283</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0.3661716361554796</t>
+          <t>0.37402054343542773</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.8324955761800378</t>
+          <t>0.3958941324195353</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>0.39044399570676713</t>
+          <t>0.3629511439674982</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>0.23944474634897922</t>
+          <t>0.3339428591063688</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>0.4511911813137516</t>
+          <t>0.4166982272878613</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.9139129435792932</t>
+          <t>0.46005518184814886</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0.3569780444684485</t>
+          <t>0.4809008211261408</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>2.6219446000856785</t>
+          <t>2.71889904145002</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>1.0076780739436955</t>
+          <t>0.6341590446312532</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>7.7741926485242345</t>
+          <t>14.463489109251228</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>7.813128561000995</t>
+          <t>9.759852897489475</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>0.4490377014074145</t>
+          <t>0.35267377229104396</t>
         </is>
       </c>
     </row>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>0.37376900294907506</t>
+          <t>0.48266088198606605</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>2.226730392159442</t>
+          <t>1.542502888154288</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>0.5872562045786811</t>
+          <t>0.48769846641677983</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>4.547746126274898</t>
+          <t>4.72408960238358</t>
         </is>
       </c>
     </row>
@@ -2624,7 +2624,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>0.38651126366711397</t>
+          <t>0.22985714095333412</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>10.194302984017652</t>
+          <t>7.441117382639778</t>
         </is>
       </c>
     </row>
@@ -2668,7 +2668,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>0.5332074076287597</t>
+          <t>0.481007838938688</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>4.646666071876432</t>
+          <t>2.061007663948031</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>3.347105324426791</t>
+          <t>2.469757185115035</t>
         </is>
       </c>
     </row>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>4.0091754532504025</t>
+          <t>5.4384218846036845</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>0.8684430277247774</t>
+          <t>0.869242827296952</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>1.7944121567399174</t>
+          <t>1.4431372370396995</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>0.398905088747936</t>
+          <t>0.23130088268211232</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>0.40992857944695044</t>
+          <t>0.3225412869681684</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>0.5966344830830783</t>
+          <t>0.40062488064094687</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>0.656456667643524</t>
+          <t>0.6028243272819518</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>0.30698657442059646</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>0.8135466312285242</t>
+          <t>0.9357543952797719</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>2.221325310804554</t>
+          <t>1.7093665636572242</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.7925930191586267</t>
+          <t>1.012002258115979</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>12.729381185862785</t>
+          <t>9.793816760980878</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>9.104039564777292</t>
+          <t>7.01286919996388</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>1.9461433583296</t>
+          <t>0.8252515749526593</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>1.339011167886784</t>
+          <t>0.9849721851039159</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>2.8604741155293727</t>
+          <t>2.96746498958057</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>1.2576666381066102</t>
+          <t>1.3446977685042416</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>0.7890205857781263</t>
+          <t>0.46085787254729915</t>
         </is>
       </c>
     </row>
@@ -5088,7 +5088,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>0.8492947561020858</t>
+          <t>0.665999781011232</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>35.58871430050539</t>
+          <t>20.44241548487502</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>1.526137445039931</t>
+          <t>2.109243658126877</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>2.2203837165334566</t>
+          <t>1.4330656750316193</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>79.46819379893032</t>
+          <t>69.96231073210255</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>6.677922298443082</t>
+          <t>3.5340248681753383</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>0.3452820652378276</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>16.16100728365175</t>
+          <t>11.54293567298227</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>3.994878973839855</t>
+          <t>3.4724767753813124</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>2.332087798595968</t>
+          <t>2.697320859173856</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>2.992345594700509</t>
+          <t>2.415249968006912</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>0.8969757909078236</t>
+          <t>0.3771401033088265</t>
         </is>
       </c>
     </row>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>0.2916144138971628</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5748,7 +5748,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>0.6489096635721943</t>
+          <t>0.7734579890462778</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>9.173835535794307</t>
+          <t>2.7166735028756506</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>0.9144572818147054</t>
+          <t>0.5300187499137251</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>17.325912253283136</t>
+          <t>13.686308859965566</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>20.53159736229587</t>
+          <t>24.64782357807381</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.6202779401872459</t>
+          <t>0.39132603841434344</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>2.8239274093078373</t>
+          <t>2.2442907367257177</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>0.25143213720713353</t>
+          <t>0.476297788445569</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>21.560197939339552</t>
+          <t>13.07649002630421</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>54.260745622118804</t>
+          <t>44.30158139339529</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>11.716529834381301</t>
+          <t>11.886226648190423</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>4.8414122341093195</t>
+          <t>3.728548479588924</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>3.060614417989638</t>
+          <t>2.685203859347256</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>10.225985825863326</t>
+          <t>10.01684481187386</t>
         </is>
       </c>
     </row>
@@ -6188,7 +6188,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>0.468552665607584</t>
+          <t>0.5331645916603636</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>12.6901030696256</t>
+          <t>5.608208929578404</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>2.091538766545579</t>
+          <t>1.0177089506770187</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>2.4559696598505494</t>
+          <t>1.5516608567895978</t>
         </is>
       </c>
     </row>
@@ -6584,7 +6584,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>3.474046199102666</t>
+          <t>2.3341311039900625</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>0.49182019672414</t>
+          <t>0.69052309562882</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>9.903246178687269</t>
+          <t>6.863787632059095</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>1.5836139504558506</t>
+          <t>1.7289216269738583</t>
         </is>
       </c>
     </row>
@@ -6716,7 +6716,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>3.0371764186419536</t>
+          <t>1.048317827190461</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>2.6366712128308056</t>
+          <t>2.040220302692428</t>
         </is>
       </c>
     </row>
@@ -6826,7 +6826,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>0.3994379847761073</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6848,7 +6848,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>0.34473680751808716</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>0.23521722733873496</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6914,7 +6914,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>0.7557606804612691</t>
+          <t>0.41485960317701</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.701061217451547</t>
+          <t>0.6932416726053439</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>1.9102232153798058</t>
+          <t>1.518341072413619</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>6.446525834735647</t>
+          <t>4.566698213702369</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>15.012770254768562</t>
+          <t>19.25982428601712</t>
         </is>
       </c>
     </row>
@@ -7222,7 +7222,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>0.6440101804612461</t>
+          <t>0.5265321764685291</t>
         </is>
       </c>
     </row>
@@ -7244,7 +7244,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>0.22398523729625683</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>6.306455587443907</t>
+          <t>11.955185570640921</t>
         </is>
       </c>
     </row>
@@ -7354,7 +7354,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>0.39102199088865663</t>
+          <t>0.504828490388032</t>
         </is>
       </c>
     </row>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>0.37320453901835404</t>
+          <t>0.4806614224131358</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>8.868120651660051</t>
+          <t>8.351002358055275</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>30.16796949021078</t>
+          <t>31.837171582418595</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>19.949606788869488</t>
+          <t>22.322077570922957</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
10th Anni P1 summons :(
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D322"/>
+  <dimension ref="A1:D328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.40613162704345</t>
+          <t>4.909558293807898</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.5436670056775945</t>
+          <t>0.30421525271958005</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.8270988884878415</t>
+          <t>0.6083393539571412</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.7269450475321183</t>
+          <t>0.7226316927759698</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.370724171654574</t>
+          <t>0.2862952103943379</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.2486279405423</t>
+          <t>0.8463023237547902</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.36471136413336946</t>
+          <t>0.2514153694540111</t>
         </is>
       </c>
     </row>
@@ -925,12 +925,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3.8888888888888884</t>
+          <t>0.5555555555555556</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.3327763201137081</t>
+          <t>0.2670832537606312</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.90631498806767</t>
+          <t>0.5996429526135719</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1.100649031113079</t>
+          <t>0.8573017651763901</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0.4617696594750791</t>
+          <t>0.42213093647310695</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>1.2508587266700282</t>
+          <t>0.8459946682788368</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>7.96066281124526</t>
+          <t>4.996927462056149</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2.155766187102445</t>
+          <t>1.6849013215444963</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>0.4645330898451175</t>
+          <t>0.3335935986600007</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>5.854180159455012</t>
+          <t>3.976178950692489</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>4.01743976247084</t>
+          <t>2.3998232891685762</t>
         </is>
       </c>
     </row>
@@ -1563,12 +1563,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>0.8780677321674606</t>
+          <t>0.4390338660837303</t>
         </is>
       </c>
     </row>
@@ -1585,12 +1585,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2.6964049558080228</t>
+          <t>0.3852007079725748</t>
         </is>
       </c>
     </row>
@@ -1607,12 +1607,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>1.658276003929078</t>
+          <t>0.6215699887406969</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>4.942587327773091</t>
+          <t>5.418251122582801</t>
         </is>
       </c>
     </row>
@@ -1783,12 +1783,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>0.9132272426127037</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -1827,12 +1827,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>1.3312293369609804</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>4.230440314261502</t>
+          <t>3.941830703022425</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>17.21345282136048</t>
+          <t>12.017672181475355</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>10.663909096831446</t>
+          <t>11.927919491019885</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>0.23998812715926332</t>
+          <t>0.22461217210683504</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.29741987966991446</t>
+          <t>0.27425920605489384</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0.2566041154177858</t>
+          <t>0.23816916584042036</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0.259446344096453</t>
+          <t>0.24226186630458924</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.45638955007497056</t>
+          <t>0.3767129997820668</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>0.2549190928216798</t>
+          <t>0.24035078045507663</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>0.21577032086213255</t>
+          <t>0.20294898883472937</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>0.2884072666444276</t>
+          <t>0.27038182988241627</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.5496598299815102</t>
+          <t>0.43156184612361487</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0.332046402083238</t>
+          <t>0.3064672286984422</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>1.2982851328546623</t>
+          <t>1.232779322817346</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.6912679759729408</t>
+          <t>0.4568539621534216</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>15.017849352827968</t>
+          <t>14.281713329270183</t>
         </is>
       </c>
     </row>
@@ -2267,12 +2267,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>2.4343429521951885</t>
+          <t>4.896374006544114</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>0.4236876510003378</t>
+          <t>0.38012696977537186</t>
         </is>
       </c>
     </row>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>0.6825468109172736</t>
+          <t>0.5042273088296477</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>1.0254437533567706</t>
+          <t>0.5398060080636155</t>
         </is>
       </c>
     </row>
@@ -2553,12 +2553,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>0.870555228163242</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>9.695916205634743</t>
+          <t>6.41985055534561</t>
         </is>
       </c>
     </row>
@@ -2624,7 +2624,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>0.2768394294536419</t>
+          <t>0.36047955827061506</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>7.758732607651211</t>
+          <t>5.755364480494822</t>
         </is>
       </c>
     </row>
@@ -2668,7 +2668,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>0.2667779427292586</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>1.6248588943473719</t>
+          <t>1.9347794908073617</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>3.4219935496548732</t>
+          <t>2.7438946145284144</t>
         </is>
       </c>
     </row>
@@ -2927,12 +2927,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>5.3957998356830545</t>
+          <t>7.140955264614027</t>
         </is>
       </c>
     </row>
@@ -3015,12 +3015,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>0.8333333333333333</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -3037,12 +3037,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>1.2127189817125412</t>
+          <t>0.21584475250145665</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>1.1315551872180933</t>
+          <t>0.7115566154590928</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>0.23130088268211232</t>
+          <t>0.291149726691148</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>0.32280422906378475</t>
+          <t>0.3376971390819318</t>
         </is>
       </c>
     </row>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -3724,7 +3724,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>0.6510651607238674</t>
+          <t>0.512300253357509</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>1.3916201186999138</t>
+          <t>0.8920192195332045</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>1.9943661624562201</t>
+          <t>1.791646536979793</t>
         </is>
       </c>
     </row>
@@ -3917,12 +3917,12 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>1.1739678468702603</t>
+          <t>0.40093814877214484</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>12.85795458355327</t>
+          <t>9.628473785976409</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>10.304030361375922</t>
+          <t>7.6920653288006005</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>0.5699162990210787</t>
+          <t>0.8385138516424451</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>5.083904525285538</t>
+          <t>3.3049940080926175</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>1.7186979934750368</t>
+          <t>1.1713685698513743</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>0.58633022617866</t>
+          <t>0.4644688308913558</t>
         </is>
       </c>
     </row>
@@ -5088,7 +5088,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>0.4302524507807909</t>
+          <t>0.6705263756255058</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>18.15834492588299</t>
+          <t>15.79036606787081</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>3.127566373476804</t>
+          <t>2.233848332385374</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.7676723632636353</t>
+          <t>0.8837502252446245</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>69.84969407798386</t>
+          <t>55.04180563723715</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>5.77159354746433</t>
+          <t>3.811411963683153</t>
         </is>
       </c>
     </row>
@@ -5440,7 +5440,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>0.33245518100005705</t>
+          <t>0.2993396152929419</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>18.556372537008833</t>
+          <t>6.090076985253597</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>4.296040302150362</t>
+          <t>2.7979367505389647</t>
         </is>
       </c>
     </row>
@@ -5545,12 +5545,12 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>3.858004029611924</t>
+          <t>1.153979412168309</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>1.583984513807338</t>
+          <t>1.6836706162694757</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>0.2390702350859313</t>
+          <t>0.28280701992542917</t>
         </is>
       </c>
     </row>
@@ -5748,7 +5748,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>1.0979661791593482</t>
+          <t>0.7443893846406251</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>4.126676395608076</t>
+          <t>1.571214663013003</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>0.36850001286790146</t>
+          <t>0.23530266027014765</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>13.131693803158354</t>
+          <t>13.83268042679417</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>14.06349245479493</t>
+          <t>13.37722097988723</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.3342790864762784</t>
+          <t>0.4093141102689524</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>3.2061725066568347</t>
+          <t>1.8344245117853675</t>
         </is>
       </c>
     </row>
@@ -5985,12 +5985,12 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>0.618722896431944</t>
+          <t>0.6327543470176672</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>13.531474201782814</t>
+          <t>10.180133334053014</t>
         </is>
       </c>
     </row>
@@ -6029,12 +6029,12 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>34.5296547562633</t>
+          <t>9.190378011760288</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>16.311484323499084</t>
+          <t>12.090701250822901</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>3.332821781149728</t>
+          <t>2.7435315723589198</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>2.333155289310172</t>
+          <t>3.397419860360713</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>8.102984688826972</t>
+          <t>6.446978094924653</t>
         </is>
       </c>
     </row>
@@ -6183,12 +6183,12 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>0.9198895865542349</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>8.013297490104382</t>
+          <t>6.970014314994211</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>0.4040930160476631</t>
+          <t>0.3158849285852084</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>1.6152871351608538</t>
+          <t>0.9392222441507888</t>
         </is>
       </c>
     </row>
@@ -6584,7 +6584,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>2.8423773739271043</t>
+          <t>2.268045023738182</t>
         </is>
       </c>
     </row>
@@ -6623,12 +6623,12 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>1.0703407507219307</t>
+          <t>0.8267037412964751</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>10.31107202962487</t>
+          <t>7.704225494636596</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>3.4370302789930234</t>
+          <t>4.10964196345328</t>
         </is>
       </c>
     </row>
@@ -6716,7 +6716,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>0.4656803996648664</t>
+          <t>0.9757994539451424</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>2.065291470483428</t>
+          <t>1.250085721238284</t>
         </is>
       </c>
     </row>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>0.27020266150139904</t>
+          <t>0.23889539707129392</t>
         </is>
       </c>
     </row>
@@ -6914,7 +6914,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>0.5489650279838301</t>
+          <t>0.5313553089490173</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.7755286469168579</t>
+          <t>0.5456347107398372</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>3.16812301098128</t>
+          <t>3.5318666859946792</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>6.084441286925006</t>
+          <t>4.299645808861484</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>24.6219897178622</t>
+          <t>26.37968401041447</t>
         </is>
       </c>
     </row>
@@ -7222,7 +7222,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>0.8686692488001093</t>
+          <t>0.9116283685127535</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>20.013188769091556</t>
+          <t>24.67180802331191</t>
         </is>
       </c>
     </row>
@@ -7354,7 +7354,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>0.7412269232260577</t>
+          <t>0.5105484507094079</t>
         </is>
       </c>
     </row>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>0.70009538571506</t>
+          <t>0.4865191541420848</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>7.23059446227222</t>
+          <t>5.884308222598272</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>21.754699950106534</t>
+          <t>24.99600852017211</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,139 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>26.736108969275545</t>
+          <t>26.70999351706555</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="1" t="inlineStr">
+        <is>
+          <t>322</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>DF_AGL_Super_Vegito</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>3.1445916824696227</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="1" t="inlineStr">
+        <is>
+          <t>323</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>DF_INT_Buuhan</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="1" t="inlineStr">
+        <is>
+          <t>324</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>BU_STR_Hercule</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>7.28508599540455</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="1" t="inlineStr">
+        <is>
+          <t>325</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>CLR_STR_Evolution_Blue_Vegeta</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>8.738311645233402</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="1" t="inlineStr">
+        <is>
+          <t>326</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>CLR_AGL_SS4_Goku</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>48.84284928427354</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="1" t="inlineStr">
+        <is>
+          <t>327</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>DFLR_TEQ_Super_Vegito</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>5.039928813817795</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
10th Anni Part 2 Summons
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D328"/>
+  <dimension ref="A1:D338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,12 +463,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.054503988707488</t>
+          <t>0.527251994353744</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.530860175034061</t>
+          <t>4.361949032591559</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.33524171825218024</t>
+          <t>0.23574617776442475</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.6421910187283718</t>
+          <t>0.5444660522597279</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.7341485092978091</t>
+          <t>0.640702474809646</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.302280806132716</t>
+          <t>0.25347632076680376</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.8853924709908902</t>
+          <t>0.7574550940708971</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.28620894686401366</t>
+          <t>0.2032737737321053</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.6295595247919629</t>
+          <t>0.5870932792370066</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.9129750512610001</t>
+          <t>0.853498303881991</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0.9185591099221271</t>
+          <t>0.884234533433046</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>5.93048262518319</t>
+          <t>6.36096509062256</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.8748072884322817</t>
+          <t>1.4390696962073428</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>4.567069058296742</t>
+          <t>4.087806639014289</t>
         </is>
       </c>
     </row>
@@ -1541,12 +1541,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2.833348895935714</t>
+          <t>1.2758951062796666</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>0.8563345777772597</t>
+          <t>0.6658023883024011</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>6.5203681092741945</t>
+          <t>4.709333292528688</t>
         </is>
       </c>
     </row>
@@ -1849,12 +1849,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>4.295068795451804</t>
+          <t>3.170928701564671</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>14.318659071896288</t>
+          <t>10.817521314724294</t>
         </is>
       </c>
     </row>
@@ -1915,12 +1915,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>12.200920852053876</t>
+          <t>6.691560799527345</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>0.20236994602990807</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.2482946980630048</t>
+          <t>0.21351661822480747</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0.214986139035276</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0.21950924776208539</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.3748920765173877</t>
+          <t>0.3151653027179109</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>0.25370407699906994</t>
+          <t>0.21760374407851518</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.4299796046327436</t>
+          <t>0.3683803402623974</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0.2825280243742441</t>
+          <t>0.24254382847170267</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>1.3313771002332726</t>
+          <t>1.0185835570913166</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.4519797053827856</t>
+          <t>0.41663353864491204</t>
         </is>
       </c>
     </row>
@@ -2223,12 +2223,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>20.447350071414398</t>
+          <t>5.481245719791488</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>5.918751135571405</t>
+          <t>6.6877308732739715</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>0.42319382932921096</t>
+          <t>0.3521739869560535</t>
         </is>
       </c>
     </row>
@@ -2377,12 +2377,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>0.5195022941207033</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.6439291288542631</t>
+          <t>0.4857808718316848</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>8.349217814182651</t>
+          <t>6.269821995987515</t>
         </is>
       </c>
     </row>
@@ -2624,7 +2624,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>0.3646202810065069</t>
+          <t>0.3155473336779959</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>6.639868695998623</t>
+          <t>5.02504347848755</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>2.235245119783216</t>
+          <t>1.849211317656974</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>3.0690146869626322</t>
+          <t>2.30798425687627</t>
         </is>
       </c>
     </row>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>6.205998012225202</t>
+          <t>6.304683545084495</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>0.2523740888370487</t>
+          <t>0.21445714866870777</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>0.7445128928456889</t>
+          <t>0.3886901286240877</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>0.4602636581799371</t>
+          <t>0.37938916268570144</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>0.33458277763677147</t>
+          <t>0.28201684292622164</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>0.5401356488602246</t>
+          <t>0.4438586829440962</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>0.9890143280291415</t>
+          <t>0.9759374150367902</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>2.4588439255455494</t>
+          <t>2.0371923636241966</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.5082645603725817</t>
+          <t>0.4185592393068056</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>11.00839510514396</t>
+          <t>8.998560924674821</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>8.554253920920349</t>
+          <t>6.800840951423201</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>0.8446599883440677</t>
+          <t>0.7471447865075329</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>3.6005891470680855</t>
+          <t>2.8964425916799597</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>1.2223695908925558</t>
+          <t>1.760487608073925</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>0.5626032332804041</t>
+          <t>0.6048980187830395</t>
         </is>
       </c>
     </row>
@@ -5088,7 +5088,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>0.7216009582392864</t>
+          <t>0.587591927214329</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>17.99015657891317</t>
+          <t>12.22705876560277</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.361921960094894</t>
+          <t>2.205519333945238</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.7051221191560039</t>
+          <t>0.9555647180379135</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>60.0907559934362</t>
+          <t>52.53703389101396</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>5.024068186084601</t>
+          <t>2.6747024223347737</t>
         </is>
       </c>
     </row>
@@ -5440,7 +5440,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>0.3075172232975743</t>
+          <t>0.2649244524493756</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>6.047100676420733</t>
+          <t>6.243052438524984</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>3.487740587444185</t>
+          <t>2.90587840903614</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>1.0883899995358188</t>
+          <t>1.632163020169057</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>1.658274416003498</t>
+          <t>1.342458798290673</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>0.32471897430055635</t>
+          <t>0.28709437588717807</t>
         </is>
       </c>
     </row>
@@ -5743,12 +5743,12 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>0.8140970926724749</t>
+          <t>0.22705927031518014</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>1.8071175059677163</t>
+          <t>1.491381877905745</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>0.26092757733862876</t>
+          <t>0.24371716954058212</t>
         </is>
       </c>
     </row>
@@ -5831,12 +5831,12 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>13.32122932992533</t>
+          <t>5.478692359782769</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>22.826603460413057</t>
+          <t>17.813946906387375</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.3923142367329503</t>
+          <t>0.335556355552918</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>2.248762123240217</t>
+          <t>2.0180768093303287</t>
         </is>
       </c>
     </row>
@@ -5985,12 +5985,12 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>0.656699365342837</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6007,12 +6007,12 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>12.13576047658956</t>
+          <t>5.2077314916527015</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>8.577602169705301</t>
+          <t>9.53223544517617</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>6.022366633752269</t>
+          <t>4.696001942963229</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>3.07017787788702</t>
+          <t>2.234226659006703</t>
         </is>
       </c>
     </row>
@@ -6139,12 +6139,12 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>3.0414459213636906</t>
+          <t>2.503292608221715</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>7.814819103039379</t>
+          <t>6.0508738972152685</t>
         </is>
       </c>
     </row>
@@ -6188,7 +6188,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>0.21163104681600053</t>
+          <t>0.20962493103719204</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>8.030965911603506</t>
+          <t>6.414917950036044</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>0.3153946600914156</t>
+          <t>0.2515007720514022</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>1.0714192394976862</t>
+          <t>0.8474154512779297</t>
         </is>
       </c>
     </row>
@@ -6579,12 +6579,12 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>2.547906389679379</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>0.8995106518280123</t>
+          <t>1.00317494048871</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>8.362484699022628</t>
+          <t>6.755142769102023</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>3.339120000809444</t>
+          <t>2.6032275927244135</t>
         </is>
       </c>
     </row>
@@ -6716,7 +6716,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>1.0932430020604087</t>
+          <t>0.8467153665882885</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.386222123489415</t>
+          <t>1.5827626370724364</t>
         </is>
       </c>
     </row>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>0.25139255137154803</t>
+          <t>0.2006487348882513</t>
         </is>
       </c>
     </row>
@@ -6914,7 +6914,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>0.6409017719029362</t>
+          <t>0.4970895183802982</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.5581704967474692</t>
+          <t>0.5859291292878581</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>3.816346946994098</t>
+          <t>3.00259134006887</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>4.805979061197458</t>
+          <t>3.708361847259125</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>31.501364947143163</t>
+          <t>26.09117957317322</t>
         </is>
       </c>
     </row>
@@ -7222,7 +7222,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>0.9357899564347253</t>
+          <t>0.7894701166027333</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>20.236362440796597</t>
+          <t>28.441856260873077</t>
         </is>
       </c>
     </row>
@@ -7354,7 +7354,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>0.5665462687332092</t>
+          <t>0.742554864501276</t>
         </is>
       </c>
     </row>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>0.5185693194572787</t>
+          <t>0.5013459053481271</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>6.5065755781949095</t>
+          <t>5.754743187802573</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>18.4069255820103</t>
+          <t>19.82671989211166</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>28.572182760867378</t>
+          <t>25.76613502069712</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>3.734173322371305</t>
+          <t>3.191122613070496</t>
         </is>
       </c>
     </row>
@@ -7569,12 +7569,12 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>8.4156126858001</t>
+          <t>6.72272974787775</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>9.696056013261876</t>
+          <t>6.678260223991702</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>51.39986624238975</t>
+          <t>43.48545620117249</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,227 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>5.265189493447437</t>
+          <t>6.1745635938019205</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="1" t="inlineStr">
+        <is>
+          <t>328</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>DF_INT_Super_Janemba</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="1" t="inlineStr">
+        <is>
+          <t>329</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>DF_STR_Super_Gogeta</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="1" t="inlineStr">
+        <is>
+          <t>330</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>DFLR_AGL_Full_Power_Frieza</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="1" t="inlineStr">
+        <is>
+          <t>331</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>DFLR_INT_Super_Saiyan_Goku</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>7.804904195241505</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="1" t="inlineStr">
+        <is>
+          <t>332</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>DF_TEQ_Perfect_Cell</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>4.803419409659969</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="1" t="inlineStr">
+        <is>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>LR_INT_SS2_Gohan</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>5.4848703177516995</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="1" t="inlineStr">
+        <is>
+          <t>334</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>BU_AGL_Beerus</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>4.122127814960759</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="1" t="inlineStr">
+        <is>
+          <t>335</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>CLR_INT_Goku_Frieza</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>34.30228673596306</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="1" t="inlineStr">
+        <is>
+          <t>336</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>CLR_PHY_SS2_Gohan</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>6.013127318312613</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="1" t="inlineStr">
+        <is>
+          <t>337</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>DFLR_AGL_Super_Gogeta</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>96.0249786545603</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
10th anniversay part 3 stone and rainbow tickets
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D338"/>
+  <dimension ref="A1:D341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.361949032591559</t>
+          <t>5.147151951407842</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.23574617776442475</t>
+          <t>0.2514861654743399</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.5444660522597279</t>
+          <t>0.6185115447768779</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.640702474809646</t>
+          <t>0.3852007079725748</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.7574550940708971</t>
+          <t>0.8305678974962332</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.2032737737321053</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -925,12 +925,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.6088181617418025</t>
+          <t>0.30440908087090124</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.5870932792370066</t>
+          <t>0.6249144108027461</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.853498303881991</t>
+          <t>0.780015877729443</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0.884234533433046</t>
+          <t>0.854527206960871</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>6.36096509062256</t>
+          <t>4.3755703331991995</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.4390696962073428</t>
+          <t>1.31768415351112</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>4.087806639014289</t>
+          <t>3.4003029950827397</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>1.2758951062796666</t>
+          <t>1.7739422867197543</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>0.6658023883024011</t>
+          <t>0.37633598531839096</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>4.709333292528688</t>
+          <t>1.4560343301113907</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>3.170928701564671</t>
+          <t>1.8382241710713654</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>10.817521314724294</t>
+          <t>5.958233802081503</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>6.691560799527345</t>
+          <t>5.1601351607319685</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.21351661822480747</t>
+          <t>0.3089593851688409</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.24384577650036013</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.3151653027179109</t>
+          <t>0.40517236063483547</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.261267344493279</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>0.21760374407851518</t>
+          <t>0.28120418872615055</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.3683803402623974</t>
+          <t>0.46370370555211504</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0.24254382847170267</t>
+          <t>0.3564428860868816</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>1.0185835570913166</t>
+          <t>0.6553688053305415</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.41663353864491204</t>
+          <t>0.4837682722766091</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>5.481245719791488</t>
+          <t>7.369267468604704</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>6.6877308732739715</t>
+          <t>8.958224320187643</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>0.3521739869560535</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.4857808718316848</t>
+          <t>0.491439493571427</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>6.269821995987515</t>
+          <t>3.516138009917059</t>
         </is>
       </c>
     </row>
@@ -2624,7 +2624,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>0.3155473336779959</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>5.02504347848755</t>
+          <t>5.751336936139</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>1.849211317656974</t>
+          <t>0.8460619514923551</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>2.30798425687627</t>
+          <t>1.3127006439134168</t>
         </is>
       </c>
     </row>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>6.304683545084495</t>
+          <t>5.299292343968347</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>0.21445714866870777</t>
+          <t>0.3001388460521803</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>0.3886901286240877</t>
+          <t>0.5017533944495435</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>0.37938916268570144</t>
+          <t>0.25347632076680376</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>0.28201684292622164</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>0.4438586829440962</t>
+          <t>0.345543576982281</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>0.9759374150367902</t>
+          <t>0.8809925543567287</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>2.0371923636241966</t>
+          <t>1.1370510020497602</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.4185592393068056</t>
+          <t>0.36928158244274556</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>8.998560924674821</t>
+          <t>7.664627398907729</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>6.800840951423201</t>
+          <t>4.453073512039786</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>0.7471447865075329</t>
+          <t>0.3563959877323074</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>2.8964425916799597</t>
+          <t>1.9500517555017227</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>1.760487608073925</t>
+          <t>1.3166382408761903</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>0.6048980187830395</t>
+          <t>0.36121892262945554</t>
         </is>
       </c>
     </row>
@@ -5088,7 +5088,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>0.587591927214329</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>12.22705876560277</t>
+          <t>11.50271850717192</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.205519333945238</t>
+          <t>2.372677889027049</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.9555647180379135</t>
+          <t>0.4640873660557289</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>52.53703389101396</t>
+          <t>56.87342871578694</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>2.6747024223347737</t>
+          <t>3.392658374337549</t>
         </is>
       </c>
     </row>
@@ -5440,7 +5440,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>0.2649244524493756</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>6.243052438524984</t>
+          <t>9.131986764198928</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>2.90587840903614</t>
+          <t>3.935911033002274</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>1.632163020169057</t>
+          <t>1.0903414444951376</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>1.342458798290673</t>
+          <t>0.8988016519360076</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>0.28709437588717807</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5748,7 +5748,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>0.22705927031518014</t>
+          <t>0.21003086090337852</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>1.491381877905745</t>
+          <t>6.366836286823892</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>0.24371716954058212</t>
+          <t>0.23512769880574474</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>5.478692359782769</t>
+          <t>7.886748860894485</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>17.813946906387375</t>
+          <t>8.009437520771026</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.335556355552918</t>
+          <t>0.6397888351014138</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>2.0180768093303287</t>
+          <t>1.550610968743939</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>5.2077314916527015</t>
+          <t>3.094788066995569</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>9.53223544517617</t>
+          <t>13.26245623401097</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>4.696001942963229</t>
+          <t>5.147495365459464</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>2.234226659006703</t>
+          <t>0.6360664067784588</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>2.503292608221715</t>
+          <t>2.8979755096283464</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>6.0508738972152685</t>
+          <t>6.154296379344521</t>
         </is>
       </c>
     </row>
@@ -6188,7 +6188,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>0.20962493103719204</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>6.414917950036044</t>
+          <t>1.9861074812826018</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>0.2515007720514022</t>
+          <t>0.3433187417469352</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>0.8474154512779297</t>
+          <t>0.9538117935943325</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>1.00317494048871</t>
+          <t>0.8730243497598953</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>6.755142769102023</t>
+          <t>6.295817148787153</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>2.6032275927244135</t>
+          <t>0.7594599559910206</t>
         </is>
       </c>
     </row>
@@ -6716,7 +6716,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>0.8467153665882885</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.5827626370724364</t>
+          <t>1.3586051278019424</t>
         </is>
       </c>
     </row>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>0.2006487348882513</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6914,7 +6914,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>0.4970895183802982</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.5859291292878581</t>
+          <t>0.6499645485430372</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>3.00259134006887</t>
+          <t>0.7869266552145665</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>3.708361847259125</t>
+          <t>2.6110252083728884</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>26.09117957317322</t>
+          <t>8.85072764255467</t>
         </is>
       </c>
     </row>
@@ -7222,7 +7222,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>0.7894701166027333</t>
+          <t>0.3458311366242411</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>28.441856260873077</t>
+          <t>34.32310560524295</t>
         </is>
       </c>
     </row>
@@ -7354,7 +7354,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>0.742554864501276</t>
+          <t>0.4625256143195366</t>
         </is>
       </c>
     </row>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>0.5013459053481271</t>
+          <t>0.5163334304244711</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>5.754743187802573</t>
+          <t>8.74088292277886</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>19.82671989211166</t>
+          <t>14.07665325481563</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>25.76613502069712</t>
+          <t>19.174355031292478</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>3.191122613070496</t>
+          <t>5.347467576922535</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>6.72272974787775</t>
+          <t>7.68575862084333</t>
         </is>
       </c>
     </row>
@@ -7591,12 +7591,12 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>6.678260223991702</t>
+          <t>17.55069144050915</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>43.48545620117249</t>
+          <t>47.81727955742368</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>6.1745635938019205</t>
+          <t>13.843388130662065</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>7.804904195241505</t>
+          <t>7.485716831580664</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>4.803419409659969</t>
+          <t>13.138712910077244</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>5.4848703177516995</t>
+          <t>8.00962100680775</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>4.122127814960759</t>
+          <t>5.628099406303551</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>34.30228673596306</t>
+          <t>34.7634032788478</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>6.013127318312613</t>
+          <t>7.685074535361351</t>
         </is>
       </c>
     </row>
@@ -7855,12 +7855,78 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>96.0249786545603</t>
+          <t>4.053138781884925</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="1" t="inlineStr">
+        <is>
+          <t>338</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>F2P_PHY_Trunks_Goten</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="1" t="inlineStr">
+        <is>
+          <t>339</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>F2PLR_AGL_Demon_King_Piccolo</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="1" t="inlineStr">
+        <is>
+          <t>340</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>LR_STR_Kaioken_Goku</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>3.9793022549399226</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add STR Cell Banner
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D346"/>
+  <dimension ref="A1:D353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.5778010619588624</t>
+          <t>0.6331964047096604</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.148350354764268</t>
+          <t>5.1097911767253485</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.21106546823655348</t>
+          <t>0.23130088268211232</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.30440908087090124</t>
+          <t>0.3335935986600007</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.9132272426127037</t>
+          <t>1.0007807959800024</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.45023294336197556</t>
+          <t>0.43320612230368494</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2.886751345948129</t>
+          <t>3.163511966122465</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.42213093647310695</t>
+          <t>0.46260176536422465</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.40062488064094687</t>
+          <t>0.4390338660837303</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2.4037492838456807</t>
+          <t>2.634203196502382</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2.2452510468485443</t>
+          <t>2.4605093069841395</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.2777777777777778</t>
+          <t>0.30440908087090124</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.756471486759053</t>
+          <t>0.7320087445396901</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2.5965708291023617</t>
+          <t>2.5748454376806587</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2.886751345948129</t>
+          <t>3.163511966122465</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.3335935986600007</t>
+          <t>0.3655761147090257</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.6671871973200014</t>
+          <t>0.7311522294180514</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.3207501495497921</t>
+          <t>0.3515013295691628</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.6476002595255947</t>
+          <t>0.6279245769581694</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.8472367604537439</t>
+          <t>0.8188014344283372</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0.5069526415336075</t>
+          <t>0.5555555555555556</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.4811252243246881</t>
+          <t>0.527251994353744</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0.8785048196846343</t>
+          <t>0.9622504486493763</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>0.8333333333333333</t>
+          <t>0.9132272426127037</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3.5020743146828295</t>
+          <t>3.45959617828694</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.4481632545294802</t>
+          <t>1.4160270041296572</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>0.40062488064094687</t>
+          <t>0.4390338660837303</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>1.5208579246008234</t>
+          <t>1.6666666666666665</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>0.8333333333333333</t>
+          <t>3.763376538332825</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>3.290185032381231</t>
+          <t>3.605623925768521</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>3.0571957995350694</t>
+          <t>3.0117094647045413</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>5.608748328973255</t>
+          <t>6.146474125172224</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>1.2663928094193209</t>
+          <t>1.387805296092674</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>0.8333333333333333</t>
+          <t>4.995514570902137</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>3.290185032381231</t>
+          <t>3.605623925768521</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.5594279192143468</t>
+          <t>0.5517554967238465</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>0.527251994353744</t>
+          <t>0.5778010619588624</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>0.46260176536422465</t>
+          <t>0.5069526415336075</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>0.26361372900287794</t>
+          <t>0.25538197943196894</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>1.4357798047714738</t>
+          <t>1.3924896197617855</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>1.2161002018432159</t>
+          <t>1.1860652118028128</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>3.0901408927102922</t>
+          <t>2.997376534362459</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4.741383723023766</t>
+          <t>4.752921356981709</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.3306436611283617</t>
+          <t>0.31890474157610726</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0.2610572506404627</t>
+          <t>0.2514525966694305</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.2908312992409778</t>
+          <t>0.2819949401837128</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>0.27829116285590055</t>
+          <t>0.268076833119676</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>0.2971784419796575</t>
+          <t>0.28628884687773315</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.29206138974924295</t>
+          <t>0.2835964317900078</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0.3729676997640233</t>
+          <t>0.35994189560178724</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>0.42501697999329396</t>
+          <t>0.41151924765781644</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.48342007519484126</t>
+          <t>0.4671399140430351</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>8.94473387189344</t>
+          <t>8.972337885708328</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>5.746678807640219</t>
+          <t>5.657342790315582</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>1.2962962962962958</t>
+          <t>1.4205757107308723</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>1.387805296092674</t>
+          <t>1.5208579246008234</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.3587297537959491</t>
+          <t>0.34826447889590206</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>1.103324400362609</t>
+          <t>1.0651329781457262</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>5.10434937495214</t>
+          <t>5.025816885146192</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>0.5149921126125698</t>
+          <t>0.505472241279256</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>0.6331964047096604</t>
+          <t>0.693902648046337</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>1.230534146315152</t>
+          <t>1.190715762305378</t>
         </is>
       </c>
     </row>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>3.743898240591197</t>
+          <t>3.763485849263174</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>1.4433756729740645</t>
+          <t>1.5817559830612324</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>0.273126333350474</t>
+          <t>0.2639679692713095</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>0.3957702516231805</t>
+          <t>0.3839434633864113</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>0.2777777777777778</t>
+          <t>0.30440908087090124</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>0.4811252243246881</t>
+          <t>0.527251994353744</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>1.317101598251191</t>
+          <t>1.4433756729740645</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>1.1556021239177248</t>
+          <t>1.2663928094193209</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>0.8721788409453686</t>
+          <t>0.8511366464695271</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>0.7128192420100414</t>
+          <t>0.6900714965953486</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.32354049091618986</t>
+          <t>0.31371671969226345</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>6.823573839528946</t>
+          <t>6.740318442152397</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>3.271486721758933</t>
+          <t>3.1922104565367464</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>0.34244193077931295</t>
+          <t>0.3303574641958599</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>1.1828894969117507</t>
+          <t>1.2962962962962958</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>0.842819541173392</t>
+          <t>0.8229642314553349</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>1.4852255091698625</t>
+          <t>1.4565396715513828</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>0.30832865869755466</t>
+          <t>0.30620160017605613</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>8.734982021158638</t>
+          <t>8.57062206126565</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.50396934157678</t>
+          <t>2.41012547033572</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.37729316215769426</t>
+          <t>0.3651033410292895</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>10.002290985425383</t>
+          <t>10.017300796207039</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>1.5981894637358895</t>
+          <t>1.5476209612012324</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>12.079221465633246</t>
+          <t>12.107348771453786</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>2.180421494649069</t>
+          <t>2.13326486134147</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>1.0496328812652562</t>
+          <t>1.0256680540909953</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>0.9849721851039159</t>
+          <t>1.0794041191831907</t>
         </is>
       </c>
     </row>
@@ -5743,7 +5743,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -5770,7 +5770,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>2.7585753808601363</t>
+          <t>2.6815339594133625</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>0.20333168742934404</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>8.931643074437595</t>
+          <t>8.95894895693003</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>4.658203191359647</t>
+          <t>4.564176907467944</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.6982086851636129</t>
+          <t>0.6712914952897368</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>0.4756128886333354</t>
+          <t>0.4596174046687628</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>7.755281366001679</t>
+          <t>7.70981098670779</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>10.479058710929323</t>
+          <t>10.368483019247691</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>2.773782377370461</t>
+          <t>2.7274117143083902</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.3844972138262874</t>
+          <t>0.3730357624404607</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>6.057199802326575</t>
+          <t>6.100933938412704</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>5.115815482106296</t>
+          <t>5.021011510341831</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>3.5577018954856525</t>
+          <t>3.457388044172497</t>
         </is>
       </c>
     </row>
@@ -6403,12 +6403,12 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>0.33528272828819466</t>
+          <t>0.24139226948829218</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>0.8576182274988603</t>
+          <t>0.8316178029087808</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>0.932363220173678</t>
+          <t>0.9066866778031439</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>2.645881877065856</t>
+          <t>2.563191353737057</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>0.48988068475454455</t>
+          <t>0.4723600248920257</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.2058009496953161</t>
+          <t>1.1802073634222567</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.7245083337127021</t>
+          <t>0.7057767394895853</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>0.3675723993896604</t>
+          <t>0.3538007180231855</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>1.4653682710362572</t>
+          <t>1.420274550089951</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>5.297166377248052</t>
+          <t>5.206855091072776</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>15.99757819784864</t>
+          <t>16.00937791198877</t>
         </is>
       </c>
     </row>
@@ -7349,12 +7349,12 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>0.6149994264397224</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -7415,12 +7415,12 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>0.5481018068821593</t>
+          <t>0.6434067289567031</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>6.172338856837851</t>
+          <t>6.087189867972359</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>9.495536926182734</t>
+          <t>9.287431137906683</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>18.491211434882004</t>
+          <t>18.323099028269553</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>3.3546679722384667</t>
+          <t>3.3073746963071144</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>7.656131784053651</t>
+          <t>7.643918580158791</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>7.202091358693308</t>
+          <t>7.02218280725348</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>17.025676863311</t>
+          <t>16.970831032029174</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>8.656687595712967</t>
+          <t>8.533964789315064</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>4.375848467056815</t>
+          <t>4.339862976320477</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>7.860432173319486</t>
+          <t>7.892596162422837</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>6.219300086838104</t>
+          <t>6.15083844164785</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>2.1979854125729386</t>
+          <t>2.150690785447379</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>28.31897990225758</t>
+          <t>27.74655359406637</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>10.31028174623647</t>
+          <t>10.411118020271978</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>5.641720633859251</t>
+          <t>5.619778795139041</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>2.436854571670405</t>
+          <t>2.378676272218593</t>
         </is>
       </c>
     </row>
@@ -7970,7 +7970,7 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>4.252801047097823</t>
+          <t>4.1664278715909235</t>
         </is>
       </c>
     </row>
@@ -7992,7 +7992,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>1.787654880691924</t>
+          <t>1.774113964407824</t>
         </is>
       </c>
     </row>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>1.5036398406563283</t>
+          <t>1.459513189176923</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,161 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>17.22485524094945</t>
+          <t>16.78897592422427</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="1" t="inlineStr">
+        <is>
+          <t>346</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>F2P_STR_Goku_Black</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>0.975139350229086</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="1" t="inlineStr">
+        <is>
+          <t>347</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>F2P_TEQ_Gotenks</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="1" t="inlineStr">
+        <is>
+          <t>348</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>F2P_PHY_Jackie_Chun</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="1" t="inlineStr">
+        <is>
+          <t>349</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>F2PLR_AGL_SS_Bardock</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="1" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>BU_PHY_Android_18</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>5.010623465139139</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="1" t="inlineStr">
+        <is>
+          <t>351</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>DF_STR_Cell_Perfect_Form</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>15.71384425906206</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="1" t="inlineStr">
+        <is>
+          <t>352</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>F2P_PHY_Para_Para_Bros</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>0.2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kale & Caulidla banner
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D361"/>
+  <dimension ref="A1:D367"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.6331964047096604</t>
+          <t>0.693902648046337</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.064508719172281</t>
+          <t>5.115465800333862</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.23130088268211232</t>
+          <t>0.25347632076680376</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.3335935986600007</t>
+          <t>0.3655761147090257</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.0007807959800024</t>
+          <t>1.096728344127077</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.38346037001470584</t>
+          <t>0.3644350876632149</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3.163511966122465</t>
+          <t>3.466806371753173</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.46260176536422465</t>
+          <t>0.5069526415336075</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.4390338660837303</t>
+          <t>0.4811252243246881</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2.634203196502382</t>
+          <t>2.886751345948129</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2.4605093069841395</t>
+          <t>2.6964049558080228</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.30440908087090124</t>
+          <t>0.3335935986600007</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.6786465660021828</t>
+          <t>0.7311522294180514</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>4.175550618586431</t>
+          <t>4.171696068981469</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3.163511966122465</t>
+          <t>3.466806371753173</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.3655761147090257</t>
+          <t>0.40062488064094687</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.7311522294180514</t>
+          <t>0.8012497612818937</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.3515013295691628</t>
+          <t>0.3852007079725748</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.58217942169996</t>
+          <t>0.5676110228331634</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.7505795728184741</t>
+          <t>0.7287760928014371</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0.5555555555555556</t>
+          <t>0.6088181617418025</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.527251994353744</t>
+          <t>0.5778010619588624</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0.9622504486493763</t>
+          <t>1.054503988707488</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>0.9132272426127037</t>
+          <t>1.0007807959800024</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3.2400493314217</t>
+          <t>3.22750693039068</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.3334682859748073</t>
+          <t>1.3180596521288082</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>0.4390338660837303</t>
+          <t>0.4811252243246881</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>1.6666666666666665</t>
+          <t>1.8264544852254074</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>5.496473049264533</t>
+          <t>5.548913642584572</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>6.179575255637341</t>
+          <t>6.150416627073601</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2.9518955804034412</t>
+          <t>2.9191135239553514</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>6.146474125172224</t>
+          <t>6.735753140545633</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>1.387805296092674</t>
+          <t>1.5208579246008234</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>4.911890486509735</t>
+          <t>4.920070614381428</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2.4627890622114257</t>
+          <t>2.458228100066297</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.5229736565604937</t>
+          <t>0.5160810086423834</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>0.5778010619588624</t>
+          <t>0.6331964047096604</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>0.5069526415336075</t>
+          <t>0.5555555555555556</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>0.2255309713110849</t>
+          <t>0.21580506869300287</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>1.227696399101349</t>
+          <t>1.1869929854821306</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>1.13075885376783</t>
+          <t>1.071913391759753</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2.7452662063221283</t>
+          <t>2.598464431638534</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4.870147912049184</t>
+          <t>4.883013866098651</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.2662230503627709</t>
+          <t>0.2500384830923253</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0.20821378390405748</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.24565671356849042</t>
+          <t>0.23344357618825323</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>0.23848970482277812</t>
+          <t>0.22286061669014093</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.24871050969145506</t>
+          <t>0.23787876058242025</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0.2999107552556894</t>
+          <t>0.28122979011747223</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>0.35101343464386525</t>
+          <t>0.3312832763265048</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.43021078393206597</t>
+          <t>0.4017834461802574</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>9.26037733728218</t>
+          <t>9.245473650344351</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>5.6031036623021375</t>
+          <t>5.585466047493879</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>1.4205757107308723</t>
+          <t>1.5567701270800032</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>1.5208579246008234</t>
+          <t>1.6666666666666665</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.3171940153404691</t>
+          <t>0.3050232705384787</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>0.9218338537781517</t>
+          <t>0.86762962456038</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>5.07409369519522</t>
+          <t>5.088915463590048</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>0.3771135361347633</t>
+          <t>0.36506578452846195</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>0.693902648046337</t>
+          <t>0.7604289623004117</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>1.097181060957338</t>
+          <t>1.065784963443189</t>
         </is>
       </c>
     </row>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>3.852799370971762</t>
+          <t>3.9012871849860336</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>1.5817559830612324</t>
+          <t>4.9939565582866425</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>0.23533333467836112</t>
+          <t>0.228848101167564</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>0.34258376490753334</t>
+          <t>0.3288134345106524</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>0.30440908087090124</t>
+          <t>0.3335935986600007</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>0.527251994353744</t>
+          <t>0.5778010619588624</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>1.4433756729740645</t>
+          <t>1.5817559830612324</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>1.2663928094193209</t>
+          <t>1.387805296092674</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.20817079441390107</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>0.8410929678079326</t>
+          <t>0.8333185018118512</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>0.6291336671747167</t>
+          <t>0.5958844958632094</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.29474172675266885</t>
+          <t>0.28849617282870454</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>6.619820832658048</t>
+          <t>6.692553758589616</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>3.156732334402836</t>
+          <t>2.9879488637227976</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>0.3207501495497921</t>
+          <t>0.3515013295691628</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>1.2962962962962958</t>
+          <t>1.4205757107308723</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>0.7105174489561629</t>
+          <t>0.6932148991050822</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>1.4324931367873273</t>
+          <t>1.4173205489033176</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>0.2793025161978706</t>
+          <t>0.27927148942983493</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>7.747501325241572</t>
+          <t>7.664778834820622</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.172624219253894</t>
+          <t>2.092121280692673</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.29470283086379645</t>
+          <t>0.27615509956497203</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>10.52585599392259</t>
+          <t>10.597562101023712</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>1.4750199503836559</t>
+          <t>1.4436080553523452</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>12.357524727778177</t>
+          <t>12.441379099340011</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>2.1338643957085117</t>
+          <t>1.6533872191049066</t>
         </is>
       </c>
     </row>
@@ -5545,12 +5545,12 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>1.1743280809287082</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>1.0794041191831907</t>
+          <t>1.1828894969117507</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>2.572506361528603</t>
+          <t>2.5011246979168136</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>9.066639437090629</t>
+          <t>9.114602076706532</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>4.253797215511758</t>
+          <t>4.118051958521447</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.581017346078505</t>
+          <t>0.5465512964263467</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>0.4055706726573892</t>
+          <t>0.38862347481697446</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>7.895415655537128</t>
+          <t>8.024274299627852</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>9.913556435035101</t>
+          <t>9.555081452450288</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>2.6310049511576747</t>
+          <t>2.603659037714796</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.3128879659773654</t>
+          <t>0.29349821001811494</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>6.416561547585242</t>
+          <t>6.487232644811542</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>4.863064306950799</t>
+          <t>4.794027336717848</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>3.03758520938641</t>
+          <t>2.990138839457762</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>0.21114072383807292</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>0.7954363457314444</t>
+          <t>0.7762872908308381</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>0.8742987529259798</t>
+          <t>0.859992256244849</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>2.30933010816998</t>
+          <t>2.226246633585183</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>0.4248964432514785</t>
+          <t>0.405996393274927</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.1404700885132921</t>
+          <t>1.113418444305252</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.6585845799537391</t>
+          <t>0.6414080804377651</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>0.2974224555313996</t>
+          <t>0.279513903433363</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>1.322145495916371</t>
+          <t>1.285877399057601</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>5.151761005092862</t>
+          <t>5.083878818314353</t>
         </is>
       </c>
     </row>
@@ -7217,7 +7217,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>16.487115065099374</t>
+          <t>16.555149670977443</t>
         </is>
       </c>
     </row>
@@ -7349,7 +7349,7 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
@@ -7420,7 +7420,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>0.61083375986978</t>
+          <t>0.5958575939888231</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>5.993267240635909</t>
+          <t>5.97248086428023</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>8.389755290932648</t>
+          <t>8.165600830294125</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>18.205272537419077</t>
+          <t>17.890370273739034</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>3.18284939039927</t>
+          <t>3.1659159699899044</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>7.555257772604542</t>
+          <t>7.63690450149447</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>6.599747298265699</t>
+          <t>6.485873160704825</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>17.5239524848022</t>
+          <t>17.4664364025448</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>8.691928538094189</t>
+          <t>8.6915975498883</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>4.25492248957655</t>
+          <t>4.254000640897765</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>7.931347340045062</t>
+          <t>7.953193048143646</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>6.140641633849044</t>
+          <t>6.132201281672706</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>2.1204673744426703</t>
+          <t>2.111952932385</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>26.244864296927734</t>
+          <t>26.1447906964883</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>10.751275187247678</t>
+          <t>10.885042886306657</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>5.869289490370619</t>
+          <t>5.763346581903036</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>2.2905187797382625</t>
+          <t>2.141364605665139</t>
         </is>
       </c>
     </row>
@@ -7970,7 +7970,7 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>4.141091986662926</t>
+          <t>4.132850063831648</t>
         </is>
       </c>
     </row>
@@ -7992,7 +7992,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>1.493159816496397</t>
+          <t>1.474224318428229</t>
         </is>
       </c>
     </row>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>1.231863674654132</t>
+          <t>1.183091590976732</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>15.89588174507386</t>
+          <t>15.847789955456882</t>
         </is>
       </c>
     </row>
@@ -8058,7 +8058,7 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>0.9056354272361974</t>
+          <t>0.8895336582668022</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>4.591148582901005</t>
+          <t>4.425785480915729</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>14.7570831304079</t>
+          <t>14.61765407928939</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>34.38736678404419</t>
+          <t>33.65071579353501</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>2.296781222681973</t>
+          <t>2.192864030300972</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>30.01588952780522</t>
+          <t>58.209040570612274</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>21.74120759306507</t>
+          <t>14.84559696142368</t>
         </is>
       </c>
     </row>
@@ -8367,6 +8367,138 @@
       <c r="D361" t="inlineStr">
         <is>
           <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="1" t="inlineStr">
+        <is>
+          <t>361</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>F2P_STR_Tien</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="1" t="inlineStr">
+        <is>
+          <t>362</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>F2PLR_STR_Mercenary_Tao</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="1" t="inlineStr">
+        <is>
+          <t>363</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>F2P_INT_SS_Future_Gohan</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>0.7307605124613712</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="1" t="inlineStr">
+        <is>
+          <t>364</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>F2P_PHY_Boujack</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="1" t="inlineStr">
+        <is>
+          <t>365</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>F2P_TEQ_Mecha_Frieza</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="1" t="inlineStr">
+        <is>
+          <t>366</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>CLR_PHY_SS2_Caulifla_Kale</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>14.38824648440677</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Get TEQ Kefla with coins
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.115465800333862</t>
+          <t>5.0606226089739685</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.3644350876632149</t>
+          <t>0.3605759356505258</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>4.171696068981469</t>
+          <t>4.214855077218388</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3.466806371753173</t>
+          <t>17.434919509342816</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.5676110228331634</t>
+          <t>0.5586793142970299</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.7287760928014371</t>
+          <t>0.7026007960080971</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3.22750693039068</t>
+          <t>3.138430595540349</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.3180596521288082</t>
+          <t>1.2851814653880562</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>5.548913642584572</t>
+          <t>5.541474699070654</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>6.150416627073601</t>
+          <t>6.103638792654679</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2.9191135239553514</t>
+          <t>2.9472898109265095</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>4.920070614381428</t>
+          <t>4.9369323810577885</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2.458228100066297</t>
+          <t>2.4677187350622063</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.5160810086423834</t>
+          <t>0.5169362667957346</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>0.21580506869300287</t>
+          <t>0.21422835064360005</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>1.1869929854821306</t>
+          <t>1.1686013209994512</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>1.071913391759753</t>
+          <t>1.0883584965951858</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2.598464431638534</t>
+          <t>2.5930364463617592</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4.883013866098651</t>
+          <t>4.820539392994206</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.2500384830923253</t>
+          <t>0.2420191886925882</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.23344357618825323</t>
+          <t>0.22702047174595535</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>0.22286061669014093</t>
+          <t>0.21573068858525893</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.23787876058242025</t>
+          <t>0.2316059319042534</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0.28122979011747223</t>
+          <t>0.2723113366998503</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>0.3312832763265048</t>
+          <t>0.32591454937541564</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.4017834461802574</t>
+          <t>0.39270969918746557</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>9.245473650344351</t>
+          <t>9.207796159736823</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>5.585466047493879</t>
+          <t>5.584871561711122</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.3050232705384787</t>
+          <t>0.3009890695541519</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>0.86762962456038</t>
+          <t>0.854586274491064</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>5.088915463590048</t>
+          <t>5.094882517071628</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>0.36506578452846195</t>
+          <t>0.36019455449775806</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>1.065784963443189</t>
+          <t>1.047395615938452</t>
         </is>
       </c>
     </row>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>3.9012871849860336</t>
+          <t>3.9275577291176473</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>4.9939565582866425</t>
+          <t>4.730535933042728</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>0.228848101167564</t>
+          <t>0.21800084596242178</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>0.3288134345106524</t>
+          <t>0.3243780436059737</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>0.8333185018118512</t>
+          <t>0.8343720142143859</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>0.5958844958632094</t>
+          <t>0.591536981134159</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.28849617282870454</t>
+          <t>0.2831822851814172</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>6.692553758589616</t>
+          <t>6.633340146564193</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>2.9879488637227976</t>
+          <t>3.1022939179357127</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>0.6932148991050822</t>
+          <t>0.6905285669533175</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>1.4173205489033176</t>
+          <t>1.412354483737026</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>0.27927148942983493</t>
+          <t>0.27155013538773876</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>7.664778834820622</t>
+          <t>7.47200190820389</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.092121280692673</t>
+          <t>2.03208685318577</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.27615509956497203</t>
+          <t>0.2672357703032776</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>10.597562101023712</t>
+          <t>10.691573249031272</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>1.4436080553523452</t>
+          <t>1.4259084461702682</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>12.441379099340011</t>
+          <t>12.554225955914553</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>1.6533872191049066</t>
+          <t>1.441494679199058</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>2.5011246979168136</t>
+          <t>2.5066184048677584</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>9.114602076706532</t>
+          <t>9.130636980433081</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>4.118051958521447</t>
+          <t>4.1644128202390736</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.5465512964263467</t>
+          <t>0.5369916917262897</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>0.38862347481697446</t>
+          <t>0.37922549699852054</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>8.024274299627852</t>
+          <t>8.117796775285477</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>9.555081452450288</t>
+          <t>9.66278568226636</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>2.603659037714796</t>
+          <t>2.5716749318750405</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.29349821001811494</t>
+          <t>0.28669020813860774</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>6.487232644811542</t>
+          <t>6.587737591989622</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>4.794027336717848</t>
+          <t>4.768077413527978</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>2.990138839457762</t>
+          <t>2.874788903235739</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>0.7762872908308381</t>
+          <t>0.7664270726599696</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>0.859992256244849</t>
+          <t>0.8483739046786671</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>2.226246633585183</t>
+          <t>2.186584409775653</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>0.405996393274927</t>
+          <t>0.40243981924232247</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.113418444305252</t>
+          <t>1.1097785581861839</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.6414080804377651</t>
+          <t>0.6316229742739923</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>0.279513903433363</t>
+          <t>0.2693003429645484</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>1.285877399057601</t>
+          <t>1.2743295490951623</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>5.083878818314353</t>
+          <t>5.131792625819012</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>16.555149670977443</t>
+          <t>16.731723171522226</t>
         </is>
       </c>
     </row>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>0.5958575939888231</t>
+          <t>0.5871768134646951</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>5.97248086428023</t>
+          <t>6.033096173558272</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>8.165600830294125</t>
+          <t>10.74745035096173</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>17.890370273739034</t>
+          <t>18.07950799062408</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>3.1659159699899044</t>
+          <t>3.1769025451359765</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>7.63690450149447</t>
+          <t>7.535455346059519</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>6.485873160704825</t>
+          <t>6.486811250030035</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>17.4664364025448</t>
+          <t>17.554906892789354</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>8.6915975498883</t>
+          <t>8.440022438170189</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>4.254000640897765</t>
+          <t>4.219217474818955</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>7.953193048143646</t>
+          <t>7.992153454460699</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>6.132201281672706</t>
+          <t>6.173337844305144</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>2.111952932385</t>
+          <t>2.0971303315508205</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>26.1447906964883</t>
+          <t>26.15909904575567</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>10.885042886306657</t>
+          <t>10.874479692685306</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>5.763346581903036</t>
+          <t>5.756985094558729</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>2.141364605665139</t>
+          <t>2.140581016548841</t>
         </is>
       </c>
     </row>
@@ -7970,7 +7970,7 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>4.132850063831648</t>
+          <t>4.128768666934561</t>
         </is>
       </c>
     </row>
@@ -7992,7 +7992,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>1.474224318428229</t>
+          <t>1.436276267097917</t>
         </is>
       </c>
     </row>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>1.183091590976732</t>
+          <t>1.576132202644427</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>15.847789955456882</t>
+          <t>15.39300492857368</t>
         </is>
       </c>
     </row>
@@ -8058,7 +8058,7 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>0.8895336582668022</t>
+          <t>0.8742389788016768</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>4.425785480915729</t>
+          <t>4.345897870004435</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>14.61765407928939</t>
+          <t>14.58097448912503</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>33.65071579353501</t>
+          <t>33.61435211534555</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>2.192864030300972</t>
+          <t>2.168424155594008</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>58.209040570612274</t>
+          <t>29.934171664873688</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>14.84559696142368</t>
+          <t>14.827726678464032</t>
         </is>
       </c>
     </row>
@@ -8432,7 +8432,7 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>0.7307605124613712</t>
+          <t>0.7175744651657553</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>14.38824648440677</t>
+          <t>14.93954707339017</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add SS Hybrids Banner
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D399"/>
+  <dimension ref="A1:D402"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.546845902540257</t>
+          <t>2.5423472441845085</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.2588653777429838</t>
+          <t>0.2537330197797297</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2.9862594049407427</t>
+          <t>2.9786295898545183</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>8.308804637701614</t>
+          <t>8.307002102083835</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.4654135533305186</t>
+          <t>0.4597916277454612</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>6.003590661594146</t>
+          <t>5.964484368252976</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>1.478148728952813</t>
+          <t>1.458810846796931</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2.264840790504686</t>
+          <t>2.2472305848654606</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2.5478177315596975</t>
+          <t>2.5249238187100285</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>1.3923731997791222</t>
+          <t>1.376246612022955</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>4.932943286197067</t>
+          <t>4.941569962096486</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>1.4169950864858396</t>
+          <t>1.4215931523876952</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.23281197966985215</t>
+          <t>0.2293038700092393</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.4950331893910344</t>
+          <t>0.48842210471839387</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0.48467436452650414</t>
+          <t>0.4786110919558322</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>1.3439536121701492</t>
+          <t>1.3275419748146309</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2.9803105756864485</t>
+          <t>2.9894579943947406</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.28625534843017225</t>
+          <t>0.28342307577955034</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>11.784592536281089</t>
+          <t>14.466145721137472</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>0.3297833657201261</t>
+          <t>0.32484364583247194</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>2.4456546229092186</t>
+          <t>2.4438979782549204</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>6.188709463676639</t>
+          <t>6.199022669461144</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>0.6647553793143953</t>
+          <t>0.6546067263196684</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2.440606153706441</t>
+          <t>2.4459582569965557</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>0.4491628271557584</t>
+          <t>0.44585753255766136</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>0.4050393342411643</t>
+          <t>0.40068813951261917</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>3.613411748176585</t>
+          <t>3.5810037544732944</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1.4765081141771979</t>
+          <t>1.454102357231383</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>0.33942192742246596</t>
+          <t>0.3324387964582936</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>0.8046561920692666</t>
+          <t>0.8037663959530414</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>4.039827056178428</t>
+          <t>3.968518719073099</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>1.597638347812634</t>
+          <t>1.5729734233028143</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.28665595954342815</t>
+          <t>0.27959456380059444</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>6.817638272490747</t>
+          <t>6.81870195483544</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>0.5940103351592135</t>
+          <t>0.5859899987283762</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>8.285284785195639</t>
+          <t>8.27068244492525</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>0.6341445595301786</t>
+          <t>0.6306519175828466</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>0.9517050863207015</t>
+          <t>0.9449736446753657</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>5.3337248217636315</t>
+          <t>5.31638141654323</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>1.59480578918068</t>
+          <t>1.5734505310840703</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.5398140382314854</t>
+          <t>0.5294732219187072</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>4.06923314770224</t>
+          <t>4.03934572483622</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>0.9847755906468894</t>
+          <t>0.9787443039282102</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>6.28488825394116</t>
+          <t>6.305994778777377</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>2.083004621525836</t>
+          <t>2.0654678908282085</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>1.857818089476861</t>
+          <t>1.806829189192417</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>0.5052934577228037</t>
+          <t>0.5037224639153011</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>1.462814797386696</t>
+          <t>1.439666919836852</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>0.2925824961827059</t>
+          <t>0.28810023416094294</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>0.6328735047635601</t>
+          <t>0.6307581628250734</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.41676147703491884</t>
+          <t>0.413629643672456</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.7648462638916091</t>
+          <t>0.7524901419650931</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>2.36457639762133</t>
+          <t>2.3562039644997546</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>10.56740292883843</t>
+          <t>10.524947631076781</t>
         </is>
       </c>
     </row>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>0.38351575111747804</t>
+          <t>0.3811282828223051</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>6.117741992946267</t>
+          <t>6.016242255845177</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>8.142281648117939</t>
+          <t>8.153223652727862</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>1.1450588513577102</t>
+          <t>1.1315135390944393</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>0.8962595390896286</t>
+          <t>0.8947843322238213</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>6.741508363509366</t>
+          <t>6.655852884244747</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>4.778112816396849</t>
+          <t>4.781925135785599</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>18.887682052326937</t>
+          <t>19.04115432715492</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>2.3294738536454225</t>
+          <t>2.2990971738345594</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>4.005713582004205</t>
+          <t>4.007106022010905</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>2.430362055506487</t>
+          <t>2.4193412474157387</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>0.9366142201667724</t>
+          <t>0.9336821727242645</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>9.09115693780451</t>
+          <t>9.03709721645108</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>8.071904645476444</t>
+          <t>8.0756816463714</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>15.946266134074492</t>
+          <t>16.108860748737534</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>1.0751273823141068</t>
+          <t>1.0620302517635718</t>
         </is>
       </c>
     </row>
@@ -7970,7 +7970,7 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>1.6739863036779845</t>
+          <t>1.6637896954003697</t>
         </is>
       </c>
     </row>
@@ -7992,7 +7992,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>0.8229527270557838</t>
+          <t>0.7811033707882434</t>
         </is>
       </c>
     </row>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>1.252812793078675</t>
+          <t>1.230190623815638</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>7.09454301175179</t>
+          <t>6.90439753795507</t>
         </is>
       </c>
     </row>
@@ -8058,7 +8058,7 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>0.4830925667688474</t>
+          <t>0.47576286487873287</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>2.988518576306209</t>
+          <t>2.961594927856082</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>11.95043090013553</t>
+          <t>11.71837018502669</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>7.090023123555609</t>
+          <t>7.098772293993131</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>0.34605168926271235</t>
+          <t>0.34331057692049916</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>15.70734236768849</t>
+          <t>15.601749746604101</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>21.512721412830313</t>
+          <t>21.51667605263761</t>
         </is>
       </c>
     </row>
@@ -8432,7 +8432,7 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>0.38381047959694276</t>
+          <t>0.37846318245606253</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>7.179627053302537</t>
+          <t>7.018083374564155</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>5.178777172345293</t>
+          <t>5.145199124576654</t>
         </is>
       </c>
     </row>
@@ -8542,7 +8542,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>2.4808849629717455</t>
+          <t>2.40316073298291</t>
         </is>
       </c>
     </row>
@@ -8564,7 +8564,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>0.39291885081587247</t>
+          <t>0.3901457939798222</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>9.277219835839432</t>
+          <t>9.325363148634594</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>4.14786397946601</t>
+          <t>4.2073889346430775</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>19.981634797408624</t>
+          <t>20.053616169909837</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>2.138999738986051</t>
+          <t>2.0983958668304</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>1.898105599083687</t>
+          <t>1.864025388811892</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>7.462950344189366</t>
+          <t>7.55903136263683</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>14.370342769685038</t>
+          <t>14.555259600530817</t>
         </is>
       </c>
     </row>
@@ -9004,7 +9004,7 @@
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>10.63781488603764</t>
+          <t>10.627535427330633</t>
         </is>
       </c>
     </row>
@@ -9026,7 +9026,7 @@
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>5.338802555470234</t>
+          <t>5.843791610761826</t>
         </is>
       </c>
     </row>
@@ -9202,7 +9202,73 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>4.2515176807740405</t>
+          <t>4.224576651953931</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="1" t="inlineStr">
+        <is>
+          <t>399</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>LR_AGL_Goten_Trunks</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>3.0011734427997685</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="1" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>BU_PHY_Spopovich</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>4.156832533038856</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="1" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>DFLR_INT_SS_Hybrid_Saiyans</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>20.75501999881234</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Peppy gals banner
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D402"/>
+  <dimension ref="A1:D406"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3.48246046439664</t>
+          <t>5.282736753751919</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.29072719555264886</t>
+          <t>0.34194032529579477</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2.777608430529609</t>
+          <t>1.3957761535334205</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>5.2227419997476865</t>
+          <t>3.3957020268833427</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.6312979498820557</t>
+          <t>1.0017769507309495</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.645795358326648</t>
+          <t>0.9362958087496331</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>7.763004541435874</t>
+          <t>9.59202158492104</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2.0939429055966414</t>
+          <t>3.32493803795305</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.099868628429304</t>
+          <t>1.7687560051701905</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2.2426208044831717</t>
+          <t>4.466519100842142</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2.981925294227106</t>
+          <t>2.6773874148906254</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>1.9621288864307296</t>
+          <t>3.1624190508324688</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>5.492747431509739</t>
+          <t>5.868424583953217</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>1.7318463691820205</t>
+          <t>3.7504825531854022</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.32637327205290084</t>
+          <t>0.46451627549856916</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.5395259997512826</t>
+          <t>0.7592499250367513</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0.7369231149686373</t>
+          <t>0.946088671129556</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>1.124981979661848</t>
+          <t>0.8625384322917742</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>3.680840605206811</t>
+          <t>4.199332225960198</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.20043998780570407</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.21457686017515018</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.36889625614058663</t>
+          <t>0.5198607599174442</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>14.47246386863075</t>
+          <t>15.348074482573859</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.2712823900841203</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>0.262167245931918</t>
+          <t>0.33404131537763715</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>3.8608803775576312</t>
+          <t>6.766094198051</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>11.134155822987397</t>
+          <t>6.389936314705482</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>0.647234071340347</t>
+          <t>0.5581402372037465</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2.249509319218861</t>
+          <t>2.675401935845493</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>0.6414554362048445</t>
+          <t>1.0895964369618933</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>0.4185448676455623</t>
+          <t>0.4970080068402776</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.2998232716632314</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>4.093054720513955</t>
+          <t>3.2176131470277802</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1.6735101429058146</t>
+          <t>1.76574913184073</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>1.132817357322823</t>
+          <t>2.9582045738074974</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>4.161420892430288</t>
+          <t>1.7060218686421196</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>1.978898820160567</t>
+          <t>2.772220624436631</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.28425204718132857</t>
+          <t>0.28330812609209527</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>8.073683686732942</t>
+          <t>8.669002442563468</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>0.46676865661484923</t>
+          <t>0.20218994232205978</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>8.322754867653977</t>
+          <t>4.86282441831478</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>0.6120519750620169</t>
+          <t>0.8838316548877033</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>0.3155411814182408</t>
+          <t>0.3534338449783347</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.2034245369404104</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>6.018845623838409</t>
+          <t>6.18468062397524</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>1.2432209669809762</t>
+          <t>0.9596095183439681</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.6071908320060513</t>
+          <t>0.6563787013949942</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>2.319112934694532</t>
+          <t>2.187625560665712</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>0.9275193920595436</t>
+          <t>1.3922068132457064</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.22305589356894623</t>
+          <t>0.2639587031861148</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>6.371959940062437</t>
+          <t>3.361405360631453</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>2.3642863209111913</t>
+          <t>2.2136517224987466</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>1.510468606069046</t>
+          <t>1.226665800098623</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>0.20808883700317996</t>
+          <t>0.32504035486776417</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>0.6962160497562877</t>
+          <t>1.1379317258154815</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>0.29141350043176906</t>
+          <t>0.395402824041325</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>0.883732153265012</t>
+          <t>1.4273908521004597</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.5537865096919188</t>
+          <t>0.822512712300191</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.6721804845540089</t>
+          <t>0.7248405348808276</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>3.596951136956635</t>
+          <t>4.482558101987888</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>14.255886289880529</t>
+          <t>10.86453988969351</t>
         </is>
       </c>
     </row>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>0.5224199666609142</t>
+          <t>0.8441196383192744</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>7.609514215614433</t>
+          <t>11.4449459997094</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>13.30413216054449</t>
+          <t>16.451702580836397</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>1.7903713932015148</t>
+          <t>1.6208579324815475</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>0.4832189716328888</t>
+          <t>0.97092847186215</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>4.590120157124332</t>
+          <t>4.6492212105199355</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>10.908455922020487</t>
+          <t>16.025033483659612</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>22.212320140429142</t>
+          <t>25.448783108483976</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>2.5240660060558726</t>
+          <t>0.8595366922594957</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>5.063390153417177</t>
+          <t>8.718396649424813</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>1.7033977517623797</t>
+          <t>1.580418634492396</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>0.9114042342443991</t>
+          <t>0.5982453702859143</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>11.293394715717342</t>
+          <t>10.67921167824929</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>10.15842409492516</t>
+          <t>5.360265517269859</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>16.31342674193428</t>
+          <t>12.219500802183788</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>0.8303572231547852</t>
+          <t>0.6676008246311237</t>
         </is>
       </c>
     </row>
@@ -7970,7 +7970,7 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>2.0221134570728565</t>
+          <t>0.8694888362212813</t>
         </is>
       </c>
     </row>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>1.377529820833623</t>
+          <t>1.709594639875005</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>9.522640221983327</t>
+          <t>4.854788224958444</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>3.8364202975021517</t>
+          <t>5.528210907507161</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>10.81804246168071</t>
+          <t>4.18465979669984</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>6.109990325453619</t>
+          <t>7.0690678242618015</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>0.4582275693470161</t>
+          <t>0.745004612950737</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>21.33616779915481</t>
+          <t>32.65837719540821</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>22.188499540275</t>
+          <t>16.075077254245407</t>
         </is>
       </c>
     </row>
@@ -8432,7 +8432,7 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>0.29599848012167845</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>3.833079353927842</t>
+          <t>2.039508598870059</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>6.898552816594917</t>
+          <t>10.48584381666107</t>
         </is>
       </c>
     </row>
@@ -8542,7 +8542,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>2.0879462778347</t>
+          <t>1.08021037643291</t>
         </is>
       </c>
     </row>
@@ -8564,7 +8564,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>0.5460287236306728</t>
+          <t>0.7921166996164796</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>9.066735833421184</t>
+          <t>18.119761760754578</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>3.9209666108186525</t>
+          <t>4.020239920875511</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>17.04863914110097</t>
+          <t>21.926318567548872</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>0.7964166277818737</t>
+          <t>0.435726503648778</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.9541252141454664</t>
+          <t>0.6925411725268137</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>19.388582490522936</t>
+          <t>24.313454766835214</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>13.17575773818186</t>
+          <t>18.92665986559888</t>
         </is>
       </c>
     </row>
@@ -9004,7 +9004,7 @@
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>4.17779600978341</t>
+          <t>3.494033280594053</t>
         </is>
       </c>
     </row>
@@ -9026,7 +9026,7 @@
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>2.439282775881299</t>
+          <t>2.253449345365709</t>
         </is>
       </c>
     </row>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>3.9852282294345946</t>
+          <t>6.486076867523357</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>3.0799272588067272</t>
+          <t>4.032445649726195</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>2.490341460900245</t>
+          <t>5.260504774975272</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,95 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>12.601451192866804</t>
+          <t>7.947093099750347</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="1" t="inlineStr">
+        <is>
+          <t>402</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>LR_TEQ_SS2_Gohan</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>10.34840713840645</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="1" t="inlineStr">
+        <is>
+          <t>403</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>BU_PHY_Fasha</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>0.506034915012714</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="1" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>BU_TEQ_Ranfan</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>7.352576230049309</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="1" t="inlineStr">
+        <is>
+          <t>405</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>BU_AGL_Videl</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>0.2344412889806784</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Golden Frieza + Gogeta banner
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D406"/>
+  <dimension ref="A1:D410"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.282736753751919</t>
+          <t>5.5765947400608695</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.34194032529579477</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -859,12 +859,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.3957761535334205</t>
+          <t>1.8772250623065965</t>
         </is>
       </c>
     </row>
@@ -881,12 +881,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3.3957020268833427</t>
+          <t>2.935527304789746</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>1.0017769507309495</t>
+          <t>0.9613101445951078</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.9362958087496331</t>
+          <t>0.9334035840696839</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>9.59202158492104</t>
+          <t>9.737460381687818</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3.32493803795305</t>
+          <t>3.431487285259418</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.7687560051701905</t>
+          <t>1.7005163678368014</t>
         </is>
       </c>
     </row>
@@ -1299,12 +1299,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>4.466519100842142</t>
+          <t>7.08033599872199</t>
         </is>
       </c>
     </row>
@@ -1343,12 +1343,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2.6773874148906254</t>
+          <t>5.706903094102774</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>3.1624190508324688</t>
+          <t>3.0698051650371205</t>
         </is>
       </c>
     </row>
@@ -1431,12 +1431,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2.0015615919600047</t>
+          <t>1.0007807959800024</t>
         </is>
       </c>
     </row>
@@ -1453,12 +1453,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>5.868424583953217</t>
+          <t>4.322806229155444</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>3.7504825531854022</t>
+          <t>3.744994527801852</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.46451627549856916</t>
+          <t>0.4801573928843139</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.7592499250367513</t>
+          <t>0.6692012815490624</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0.946088671129556</t>
+          <t>0.8384523921250074</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>0.8625384322917742</t>
+          <t>0.741743302139011</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4.199332225960198</t>
+          <t>4.156716498455985</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.20043998780570407</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.21457686017515018</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.5198607599174442</t>
+          <t>0.4879302695476937</t>
         </is>
       </c>
     </row>
@@ -2289,12 +2289,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>2.0488247083907414</t>
+          <t>0.2926892440558202</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>15.348074482573859</t>
+          <t>15.242485906199043</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.2712823900841203</t>
+          <t>0.2501100096054711</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>0.33404131537763715</t>
+          <t>0.28577441249509206</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>6.766094198051</t>
+          <t>6.8149424301242405</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>6.389936314705482</t>
+          <t>6.059208390147677</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>0.5581402372037465</t>
+          <t>0.5218570506356909</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2.675401935845493</t>
+          <t>2.6225059888481</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>1.0895964369618933</t>
+          <t>1.0677555159141265</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>0.4970080068402776</t>
+          <t>0.4448658739075828</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.2998232716632314</t>
+          <t>0.2857363370383226</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>3.2176131470277802</t>
+          <t>3.693183496693578</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1.76574913184073</t>
+          <t>1.4756445545241519</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>2.9582045738074974</t>
+          <t>2.8531178502610373</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.772220624436631</t>
+          <t>2.62401011437987</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.28330812609209527</t>
+          <t>0.34415340671088296</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>8.669002442563468</t>
+          <t>8.865838249503085</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>0.20218994232205978</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5479,7 +5479,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>4.86282441831478</t>
+          <t>4.909628482225408</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>0.8838316548877033</t>
+          <t>0.834171547994984</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>0.3534338449783347</t>
+          <t>0.3110748566586753</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>0.2034245369404104</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>6.18468062397524</t>
+          <t>6.0184232833940285</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>0.9596095183439681</t>
+          <t>0.8602300325271708</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.6563787013949942</t>
+          <t>0.562906210686051</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>2.187625560665712</t>
+          <t>2.00443399432778</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>1.3922068132457064</t>
+          <t>1.4070159756038316</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.2639587031861148</t>
+          <t>0.23219650970634914</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>3.361405360631453</t>
+          <t>2.522930536738791</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>2.2136517224987466</t>
+          <t>2.0023138458201424</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>1.226665800098623</t>
+          <t>1.24886068478635</t>
         </is>
       </c>
     </row>
@@ -6337,7 +6337,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>0.32504035486776417</t>
+          <t>0.30295113794431644</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>1.1379317258154815</t>
+          <t>1.1107571221170414</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>0.395402824041325</t>
+          <t>0.35129445866580783</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.4273908521004597</t>
+          <t>1.3853250507347394</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.822512712300191</t>
+          <t>0.7832316252016271</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.7248405348808276</t>
+          <t>0.6422528335456902</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>4.482558101987888</t>
+          <t>4.24432357983011</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>10.86453988969351</t>
+          <t>7.08861363835094</t>
         </is>
       </c>
     </row>
@@ -7349,7 +7349,7 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
@@ -7415,12 +7415,12 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>0.8441196383192744</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>11.4449459997094</t>
+          <t>10.7159057886858</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>16.451702580836397</t>
+          <t>15.91944376464247</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>1.6208579324815475</t>
+          <t>1.538852025272349</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>0.97092847186215</t>
+          <t>0.9389433553841791</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>4.6492212105199355</t>
+          <t>4.220549282187873</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>16.025033483659612</t>
+          <t>15.370732310938193</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>25.448783108483976</t>
+          <t>23.678060791202675</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>0.8595366922594957</t>
+          <t>0.7686958492712899</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>8.718396649424813</t>
+          <t>8.544825659211343</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>1.580418634492396</t>
+          <t>1.4628788924077516</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>0.5982453702859143</t>
+          <t>0.5595192050364757</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>10.67921167824929</t>
+          <t>10.421879519734519</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>5.360265517269859</t>
+          <t>5.003038927106211</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>12.219500802183788</t>
+          <t>12.778256731219168</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>0.6676008246311237</t>
+          <t>0.42209629539635307</t>
         </is>
       </c>
     </row>
@@ -7965,12 +7965,12 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>0.8694888362212813</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>1.709594639875005</t>
+          <t>1.581935923466624</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>4.854788224958444</t>
+          <t>4.062037900663307</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>5.528210907507161</t>
+          <t>5.264671236996373</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>4.18465979669984</t>
+          <t>3.66952045814922</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>7.0690678242618015</t>
+          <t>6.855101362585138</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>0.745004612950737</t>
+          <t>0.6982870053242229</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>32.65837719540821</t>
+          <t>32.09475278245678</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>16.075077254245407</t>
+          <t>15.731566972377017</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>2.039508598870059</t>
+          <t>1.718795935775477</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>10.48584381666107</t>
+          <t>10.09148923022982</t>
         </is>
       </c>
     </row>
@@ -8542,7 +8542,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>1.08021037643291</t>
+          <t>0.9808314820514329</t>
         </is>
       </c>
     </row>
@@ -8564,7 +8564,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>0.7921166996164796</t>
+          <t>0.7881486774032597</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>18.119761760754578</t>
+          <t>18.45993500263849</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>4.020239920875511</t>
+          <t>4.041913886373479</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>21.926318567548872</t>
+          <t>22.03509123806623</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>0.435726503648778</t>
+          <t>0.3824598690291807</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.6925411725268137</t>
+          <t>0.6850444273091363</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>24.313454766835214</t>
+          <t>15.068844984985633</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>18.92665986559888</t>
+          <t>21.60748490916555</t>
         </is>
       </c>
     </row>
@@ -9004,7 +9004,7 @@
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>3.494033280594053</t>
+          <t>3.1963398122945823</t>
         </is>
       </c>
     </row>
@@ -9026,7 +9026,7 @@
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>2.253449345365709</t>
+          <t>1.983371886327645</t>
         </is>
       </c>
     </row>
@@ -9197,12 +9197,12 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>6.486076867523357</t>
+          <t>12.039994594163934</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>4.032445649726195</t>
+          <t>3.871552565866407</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>5.260504774975272</t>
+          <t>4.831803262484551</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>7.947093099750347</t>
+          <t>8.759410385974064</t>
         </is>
       </c>
     </row>
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>10.34840713840645</t>
+          <t>10.019416871574691</t>
         </is>
       </c>
     </row>
@@ -9312,7 +9312,7 @@
       </c>
       <c r="D404" t="inlineStr">
         <is>
-          <t>0.506034915012714</t>
+          <t>0.47612245203453174</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>7.352576230049309</t>
+          <t>7.07519335922703</t>
         </is>
       </c>
     </row>
@@ -9356,7 +9356,95 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>0.2344412889806784</t>
+          <t>0.2057991983109635</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="1" t="inlineStr">
+        <is>
+          <t>406</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>F2P_INT_Annin</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>0.282869268194648</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="1" t="inlineStr">
+        <is>
+          <t>407</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>F2P_TEQ_Yamcha</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>1.283809063882794</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="1" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>BU_INT_DBS_Broly_Vegeta</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>4.488085382596886</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="1" t="inlineStr">
+        <is>
+          <t>409</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>DFLR_TEQ_Golden_Frieza_Gogeta</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>81.53173589251217</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Baby possessed banner
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D415"/>
+  <dimension ref="A1:D422"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.0007807959800024</t>
+          <t>1.096728344127077</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.21353445652834</t>
+          <t>6.17064039995385</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.3655761147090257</t>
+          <t>0.40062488064094687</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.5817559830612324</t>
+          <t>1.7334031858765866</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.693902648046337</t>
+          <t>0.7604289623004117</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>4.1634158882780214</t>
+          <t>4.56257377380247</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>3.8888888888888884</t>
+          <t>4.261727132192617</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.4811252243246881</t>
+          <t>0.527251994353744</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.054503988707488</t>
+          <t>1.1556021239177248</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2.18573815540885</t>
+          <t>2.132332714079098</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3.005018817437332</t>
+          <t>3.006294108422466</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.5778010619588624</t>
+          <t>0.6331964047096604</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1.1556021239177248</t>
+          <t>1.2663928094193209</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.5555555555555556</t>
+          <t>0.6088181617418025</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>1.1159278109994588</t>
+          <t>1.0948837394798392</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1.111517217183212</t>
+          <t>1.0789216344495691</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0.8780677321674606</t>
+          <t>0.9622504486493763</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.8333333333333333</t>
+          <t>0.9132272426127037</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>9.255307538292833</t>
+          <t>9.259738246443591</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1.4433756729740645</t>
+          <t>1.5817559830612324</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3.5162202478290094</t>
+          <t>3.489123402690609</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2.014707830179246</t>
+          <t>1.9745004314946584</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>0.693902648046337</t>
+          <t>0.7604289623004117</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2.634203196502382</t>
+          <t>2.886751345948129</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>9.967050664739151</t>
+          <t>9.89718133764697</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>4.637572008407244</t>
+          <t>4.585770641651896</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>4.160636534983439</t>
+          <t>4.132293659608109</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>9.714637072648715</t>
+          <t>10.646005472205763</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>1.096728344127077</t>
+          <t>1.2018746419228403</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>4.405215830526797</t>
+          <t>4.430922600600683</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>3.763405394391926</t>
+          <t>3.783912191635829</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.5367061069308079</t>
+          <t>0.5319156235246268</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>0.9132272426127037</t>
+          <t>1.0007807959800024</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>0.8012497612818937</t>
+          <t>0.8780677321674606</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.4215553039590265</t>
+          <t>0.41030672372375926</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0.5168733096205269</t>
+          <t>0.5054736405823124</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>0.6958271901668671</t>
+          <t>0.6764830964548461</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4.013990899748329</t>
+          <t>4.0467685003687635</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.20865807245338586</t>
+          <t>0.2014546494593155</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>0.46260176536422465</t>
+          <t>0.5069526415336075</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.5407120336902049</t>
+          <t>0.5255418642203459</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>0.613152354337152</t>
+          <t>0.5950932509468597</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>10.747994170698766</t>
+          <t>10.63026198285205</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.4412375800401994</t>
+          <t>0.4323179227907339</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>1.381860478054982</t>
+          <t>1.378492060559438</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>0.40062488064094687</t>
+          <t>0.4390338660837303</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>4.371194915947911</t>
+          <t>4.301952432699249</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>0.4768774548890691</t>
+          <t>0.46326203304283187</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2.9947725651819326</t>
+          <t>2.989785064970411</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>0.4811252243246881</t>
+          <t>0.527251994353744</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>0.8333333333333333</t>
+          <t>0.9132272426127037</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>2.281286886901235</t>
+          <t>2.5</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>2.0015615919600047</t>
+          <t>2.193456688254154</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>0.3002342387940007</t>
+          <t>0.32901850323812315</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>1.2478740394688481</t>
+          <t>1.2345321521337513</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>0.49092916560376826</t>
+          <t>0.47494312394737837</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.2658717065201124</t>
+          <t>0.26153275525536834</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>4.079235829594733</t>
+          <t>4.030723781999785</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1.5906296616918432</t>
+          <t>1.5601793954488485</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>0.25347632076680376</t>
+          <t>0.2777777777777778</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>0.2926892440558202</t>
+          <t>0.3207501495497921</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>3.6011786324443262</t>
+          <t>3.550737820630887</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>1.8695827763244182</t>
+          <t>2.0488247083907414</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.9324574053907666</t>
+          <t>2.8652834809278054</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.33488687004424117</t>
+          <t>0.3223964661073091</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>8.316463106814872</t>
+          <t>8.360292805198405</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>4.751680488706221</t>
+          <t>4.771595009013673</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>0.48715964368596737</t>
+          <t>0.4811427965485804</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>1.7060218686421196</t>
+          <t>1.8695827763244182</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>0.22023035346294684</t>
+          <t>0.21590070946234743</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>0.22191129916567778</t>
+          <t>0.21745812676523862</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>6.460311342788778</t>
+          <t>6.485396625226969</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>0.4212636106504534</t>
+          <t>0.4082625583720914</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.6039751004045997</t>
+          <t>0.582346657670827</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>1.7922808576794402</t>
+          <t>1.7640036506954608</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>1.4910329241596818</t>
+          <t>1.4666307304222534</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.2509893023651805</t>
+          <t>0.24198503875064667</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>1.3827064937538631</t>
+          <t>1.3745854618158242</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>0.7783394077164241</t>
+          <t>0.7664361569018014</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>1.2962962962962958</t>
+          <t>1.4205757107308723</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>0.3345684662529665</t>
+          <t>0.3286866496822063</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>1.2904211984427105</t>
+          <t>1.2700094760444456</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>1.2962962962962958</t>
+          <t>1.4205757107308723</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>0.3705392345669769</t>
+          <t>0.36027726841643887</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.6139209621150596</t>
+          <t>1.5824682688713019</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.9005159794251275</t>
+          <t>0.8798538265376852</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>0.3548668490735252</t>
+          <t>0.3888888888888888</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.7214662104211261</t>
+          <t>0.7022302340283141</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>2.3277051204733166</t>
+          <t>2.2921093678505216</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>10.81329370105327</t>
+          <t>10.616084387353489</t>
         </is>
       </c>
     </row>
@@ -7415,12 +7415,12 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>2.561771334276101</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>12.2130839035753</t>
+          <t>11.98113475792205</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>14.29162910832062</t>
+          <t>14.340948531889481</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>1.3521437835857069</t>
+          <t>1.3185060307494203</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>2.161512428531349</t>
+          <t>2.15802277079038</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>4.395180127112706</t>
+          <t>4.270794451847028</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>10.926735300954723</t>
+          <t>10.774251512055516</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>25.182766834426747</t>
+          <t>25.285504359967018</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>0.6745393618155344</t>
+          <t>0.6556180847597329</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>8.259249178478116</t>
+          <t>8.205650959807679</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>1.5369079326588428</t>
+          <t>1.5097101955851007</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>0.6110269437736138</t>
+          <t>0.5987826599260506</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>9.594584836912581</t>
+          <t>9.50783801762075</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>3.8803613665671013</t>
+          <t>3.8384069229976703</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>12.404010531937281</t>
+          <t>12.448011017558246</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>0.7342964365712291</t>
+          <t>0.7151034695332946</t>
         </is>
       </c>
     </row>
@@ -7992,7 +7992,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>0.820169768994713</t>
+          <t>0.8988016519360076</t>
         </is>
       </c>
     </row>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>1.735637715581498</t>
+          <t>1.681728273355257</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>2.315762874486631</t>
+          <t>2.243849723402082</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>5.983023824356252</t>
+          <t>5.82749457037785</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>8.062692035920684</t>
+          <t>7.976505514861958</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>7.090835565045619</t>
+          <t>7.029202863861812</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>0.7912246326354264</t>
+          <t>0.7777568958173363</t>
         </is>
       </c>
     </row>
@@ -8300,7 +8300,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>0.2245251046848544</t>
+          <t>0.2460509306984139</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>6.995685992853964</t>
+          <t>6.984255205371589</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>5.810215094152646</t>
+          <t>5.8327914475395275</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>1.7494873969017288</t>
+          <t>1.690217647020984</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>11.623926422905</t>
+          <t>11.36233160792764</t>
         </is>
       </c>
     </row>
@@ -8542,7 +8542,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>0.8414593637060035</t>
+          <t>0.8063261449256588</t>
         </is>
       </c>
     </row>
@@ -8564,7 +8564,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>0.8602292929663286</t>
+          <t>0.8576502721450814</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>24.92463167609415</t>
+          <t>25.005771438812396</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>4.291056895144351</t>
+          <t>4.326296969298355</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>25.299591510402337</t>
+          <t>25.4264427408276</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>0.4152800283457145</t>
+          <t>0.3987445773894692</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.6713274165488817</t>
+          <t>0.6404029936869543</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>20.791890990972675</t>
+          <t>21.1797546035298</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>26.33166088950626</t>
+          <t>26.706200212615283</t>
         </is>
       </c>
     </row>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>7.7554938253441295</t>
+          <t>7.828960360176979</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>4.148852134742479</t>
+          <t>3.843822811259166</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>4.936283603090603</t>
+          <t>4.868145581021032</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>7.867125623185571</t>
+          <t>7.987238380834199</t>
         </is>
       </c>
     </row>
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>6.691015115636041</t>
+          <t>6.602182049150279</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>8.145422570718578</t>
+          <t>7.961424481551759</t>
         </is>
       </c>
     </row>
@@ -9356,7 +9356,7 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>0.3019267910113714</t>
+          <t>0.2904264719644244</t>
         </is>
       </c>
     </row>
@@ -9378,7 +9378,7 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>0.3198226407736543</t>
+          <t>0.3158565079186206</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>1.0638075427232003</t>
+          <t>1.046158862809984</t>
         </is>
       </c>
     </row>
@@ -9422,7 +9422,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>1.6225423833181454</t>
+          <t>1.5918408795364727</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9444,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>1.8036800977147605</t>
+          <t>1.840485682696226</t>
         </is>
       </c>
     </row>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>8.494865498649897</t>
+          <t>8.328513194839285</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>5.749759781410594</t>
+          <t>5.681356922945177</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,161 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>14.539704395397266</t>
+          <t>14.670245650932145</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="1" t="inlineStr">
+        <is>
+          <t>415</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>LR_TEQ_Super_17</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="1" t="inlineStr">
+        <is>
+          <t>416</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>LR_INT_Baby_Possessed_Bros</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>15.74188923701543</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="1" t="inlineStr">
+        <is>
+          <t>417</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>LR_AGL_Majin_Vegeta</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>5.271436657421702</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="1" t="inlineStr">
+        <is>
+          <t>418</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>F2P_TEQ_Baby_Possessed_Gohan</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="1" t="inlineStr">
+        <is>
+          <t>419</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>F2P_PHY_Baby_Possessed_Goten</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="1" t="inlineStr">
+        <is>
+          <t>420</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>F2P_INT_Baby_Possessed_Trunks</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="1" t="inlineStr">
+        <is>
+          <t>421</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>F2PLR_STR_Chi_Chi</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>4.145062396081411</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Daima SS4 Goku Summons
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D422"/>
+  <dimension ref="A1:D425"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.17064039995385</t>
+          <t>6.27511326988952</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2.132332714079098</t>
+          <t>1.9775662158415226</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3.006294108422466</t>
+          <t>2.9291078153044845</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>1.0948837394798392</t>
+          <t>1.0631421963683494</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1.0789216344495691</t>
+          <t>1.0391906782086666</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>9.259738246443591</t>
+          <t>9.367110747355085</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3.489123402690609</t>
+          <t>3.118269073713419</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.9745004314946584</t>
+          <t>1.9280085059469263</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>9.89718133764697</t>
+          <t>9.739934870120434</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>4.585770641651896</t>
+          <t>5.12042165125668</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>4.132293659608109</t>
+          <t>4.029721844962268</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>4.430922600600683</t>
+          <t>4.384776355234135</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>3.783912191635829</t>
+          <t>3.771262573599267</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.5319156235246268</t>
+          <t>0.5126194832447912</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.41030672372375926</t>
+          <t>0.38444710171983026</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0.5054736405823124</t>
+          <t>0.4661077054450167</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>0.6764830964548461</t>
+          <t>0.6258342572683173</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4.0467685003687635</t>
+          <t>4.071056143039584</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.2014546494593155</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.5255418642203459</t>
+          <t>0.5058589227515468</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>0.5950932509468597</t>
+          <t>0.5739851645477984</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>10.63026198285205</t>
+          <t>10.836362920824051</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.4323179227907339</t>
+          <t>0.41293330944061346</t>
         </is>
       </c>
     </row>
@@ -2641,12 +2641,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>1.378492060559438</t>
+          <t>1.7477988090448449</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>4.301952432699249</t>
+          <t>4.026590867444948</t>
         </is>
       </c>
     </row>
@@ -2861,12 +2861,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>0.46326203304283187</t>
+          <t>0.7304715850215887</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2.989785064970411</t>
+          <t>2.912231472641559</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>1.2345321521337513</t>
+          <t>1.2001245749042393</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>0.47494312394737837</t>
+          <t>0.44745841415399623</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.26153275525536834</t>
+          <t>0.2529492017133732</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>4.030723781999785</t>
+          <t>4.150183438740635</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1.5601793954488485</t>
+          <t>1.4332918358276419</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>3.550737820630887</t>
+          <t>3.1987681367485115</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.8652834809278054</t>
+          <t>2.8000360912370645</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.3223964661073091</t>
+          <t>0.3140861821689471</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>8.360292805198405</t>
+          <t>8.226268541067924</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>4.771595009013673</t>
+          <t>4.781093223871898</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>0.4811427965485804</t>
+          <t>0.4551974566870456</t>
         </is>
       </c>
     </row>
@@ -5567,12 +5567,12 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>1.8695827763244182</t>
+          <t>0.33123402300463406</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>0.21590070946234743</t>
+          <t>0.20923415617259672</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>0.21745812676523862</t>
+          <t>0.21018891583520166</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>6.485396625226969</t>
+          <t>6.350582581730627</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>0.4082625583720914</t>
+          <t>0.5154584915772658</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.582346657670827</t>
+          <t>0.5484644119165465</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>1.7640036506954608</t>
+          <t>1.6536208167695108</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>1.4666307304222534</t>
+          <t>1.4254510322626892</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.24198503875064667</t>
+          <t>0.22732189077929288</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>1.3745854618158242</t>
+          <t>1.3276929279594</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>0.7664361569018014</t>
+          <t>0.7252416682528198</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>0.3286866496822063</t>
+          <t>0.3162506836926721</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>1.2700094760444456</t>
+          <t>1.238654079042825</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>0.36027726841643887</t>
+          <t>0.33965428223127153</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.5824682688713019</t>
+          <t>1.5376245511429605</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.8798538265376852</t>
+          <t>0.8559533914509156</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.7022302340283141</t>
+          <t>0.6554622015032378</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>2.2921093678505216</t>
+          <t>2.1620571313495622</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>10.616084387353489</t>
+          <t>8.936896996470168</t>
         </is>
       </c>
     </row>
@@ -7415,12 +7415,12 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>2.561771334276101</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>11.98113475792205</t>
+          <t>12.2731404735573</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>14.340948531889481</t>
+          <t>14.16647486551598</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>1.3185060307494203</t>
+          <t>1.2662528978097105</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>2.15802277079038</t>
+          <t>2.1804462100961306</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>4.270794451847028</t>
+          <t>3.9828812622342875</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>10.774251512055516</t>
+          <t>10.306194242436971</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>25.285504359967018</t>
+          <t>24.89234306215721</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>0.6556180847597329</t>
+          <t>0.6004010642790676</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>8.205650959807679</t>
+          <t>7.9646503273075435</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>1.5097101955851007</t>
+          <t>1.441518175360958</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>0.5987826599260506</t>
+          <t>0.5767897513596196</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>9.50783801762075</t>
+          <t>9.07315417296447</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>3.8384069229976703</t>
+          <t>3.5623352227785308</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>12.448011017558246</t>
+          <t>14.380604299557127</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>0.7151034695332946</t>
+          <t>0.6571466008688598</t>
         </is>
       </c>
     </row>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>1.681728273355257</t>
+          <t>1.6451082526088767</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>2.243849723402082</t>
+          <t>2.041324484845279</t>
         </is>
       </c>
     </row>
@@ -8053,7 +8053,7 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>5.82749457037785</t>
+          <t>5.684194068920413</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>7.976505514861958</t>
+          <t>7.569283033526993</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>7.029202863861812</t>
+          <t>6.822573015050082</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>0.7777568958173363</t>
+          <t>0.7305164572872074</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>6.984255205371589</t>
+          <t>6.862899769139162</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>5.8327914475395275</t>
+          <t>7.168612628501322</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>1.690217647020984</t>
+          <t>1.590053725975505</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>11.36233160792764</t>
+          <t>11.06869849646139</t>
         </is>
       </c>
     </row>
@@ -8542,7 +8542,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>0.8063261449256588</t>
+          <t>0.7513653130876512</t>
         </is>
       </c>
     </row>
@@ -8564,7 +8564,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>0.8576502721450814</t>
+          <t>0.8504978112354858</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>25.005771438812396</t>
+          <t>24.92469089920612</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>4.326296969298355</t>
+          <t>4.245436584318327</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>25.4264427408276</t>
+          <t>25.236748624394572</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>0.3987445773894692</t>
+          <t>0.4512937372715812</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.6404029936869543</t>
+          <t>0.6046391306235978</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>21.1797546035298</t>
+          <t>22.27125982122574</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>26.706200212615283</t>
+          <t>27.863574874677976</t>
         </is>
       </c>
     </row>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>7.828960360176979</t>
+          <t>7.959432688033303</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>3.843822811259166</t>
+          <t>3.727517948719715</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>4.868145581021032</t>
+          <t>4.728704723316338</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>7.987238380834199</t>
+          <t>8.43611539362142</t>
         </is>
       </c>
     </row>
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>6.602182049150279</t>
+          <t>6.287953283753065</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>7.961424481551759</t>
+          <t>7.768236635894428</t>
         </is>
       </c>
     </row>
@@ -9356,7 +9356,7 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>0.2904264719644244</t>
+          <t>0.2823424725783134</t>
         </is>
       </c>
     </row>
@@ -9378,7 +9378,7 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>0.3158565079186206</t>
+          <t>0.3051944582833101</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>1.046158862809984</t>
+          <t>1.0176340658313023</t>
         </is>
       </c>
     </row>
@@ -9422,7 +9422,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>1.5918408795364727</t>
+          <t>1.566174330445139</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9444,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>1.840485682696226</t>
+          <t>1.913538606647677</t>
         </is>
       </c>
     </row>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>8.328513194839285</t>
+          <t>7.644481925630623</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>5.681356922945177</t>
+          <t>5.362598274447428</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>14.670245650932145</t>
+          <t>15.183360848716191</t>
         </is>
       </c>
     </row>
@@ -9598,7 +9598,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>15.74188923701543</t>
+          <t>14.75301672365481</t>
         </is>
       </c>
     </row>
@@ -9620,7 +9620,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>5.271436657421702</t>
+          <t>3.1896805178116003</t>
         </is>
       </c>
     </row>
@@ -9703,12 +9703,78 @@
       </c>
       <c r="C422" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>2.9330946722245756</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="1" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>F2P_INT_Goten_Icarus</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="1" t="inlineStr">
+        <is>
+          <t>423</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>BU_PHY_Piccolo_Mini_Daima</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="D422" t="inlineStr">
-        <is>
-          <t>4.145062396081411</t>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>16.3014367892922</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="1" t="inlineStr">
+        <is>
+          <t>424</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>DF_TEQ_SS4_Goku_Mini_Daima</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>41.21476162219281</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add new files and add EZA kid GOhan
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D425"/>
+  <dimension ref="A1:D435"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.772653450953843</t>
+          <t>5.3302449585271106</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.7837348063994507</t>
+          <t>1.8716516898579418</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3.0627766375594376</t>
+          <t>2.988461169604335</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>1.007905355670706</t>
+          <t>0.9779957746022129</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.9747320640873163</t>
+          <t>0.966757479760932</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>8.638772553617304</t>
+          <t>8.82335779223691</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2.8291901680256277</t>
+          <t>2.921240013122681</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.7822516487872342</t>
+          <t>1.7456626393609234</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>8.853708615629175</t>
+          <t>8.418693051961043</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>4.568340378025192</t>
+          <t>3.7462772055644056</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>3.66170446988481</t>
+          <t>3.523889439951571</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>3.4087850124921846</t>
+          <t>3.3480049564679177</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>3.655779170196786</t>
+          <t>3.638861298261271</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.48777814930307173</t>
+          <t>0.46273009131762066</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.3536825707350435</t>
+          <t>0.363490768887438</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0.42717818399114904</t>
+          <t>0.44489584422710493</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>0.5859687330333005</t>
+          <t>0.6240653225312063</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4.040981211321274</t>
+          <t>4.022041760704674</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.48087268502932534</t>
+          <t>0.48370844305605076</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>0.517396733080124</t>
+          <t>0.5265327059118905</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>9.417149272733333</t>
+          <t>8.588331087506374</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.37190877813854123</t>
+          <t>0.36783502024326986</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>1.6234043452534763</t>
+          <t>1.5884921678842403</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>3.714055442736943</t>
+          <t>4.041964438109833</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>0.6959012995268222</t>
+          <t>0.7034810570908788</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2.677854684038477</t>
+          <t>2.6653088060257364</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>1.0933952486154601</t>
+          <t>1.054758677734096</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>0.41223775944802243</t>
+          <t>0.4290554761277068</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.24504096184973623</t>
+          <t>0.23827672924428797</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>4.121913566550518</t>
+          <t>3.7761384138113963</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1.323676406469625</t>
+          <t>1.4037904400957673</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>2.918293377223036</t>
+          <t>2.841465124208519</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.694666211509644</t>
+          <t>2.662938515690052</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.31829137467799723</t>
+          <t>0.33280984877236147</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>8.251794612237752</t>
+          <t>8.791051787531103</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>4.776605968205189</t>
+          <t>4.791347023086814</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>0.5437142724895979</t>
+          <t>0.5937585943715828</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>0.3704095446429516</t>
+          <t>0.3618523107151006</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>0.39182248118976415</t>
+          <t>0.41709374984005365</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>7.856423708697868</t>
+          <t>7.782723063789639</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>0.4685161566304945</t>
+          <t>0.4897134025512835</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.5608748328973255</t>
+          <t>0.5934880455548311</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>1.45613271601888</t>
+          <t>1.4675948539878014</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>1.4134023542043161</t>
+          <t>1.3818808234142483</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.2311224775182495</t>
+          <t>0.24164579226036106</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>1.2117415238196594</t>
+          <t>1.2002704453719701</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>0.6430419795045932</t>
+          <t>0.6439814395125705</t>
         </is>
       </c>
     </row>
@@ -6562,7 +6562,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>0.28377593555755454</t>
+          <t>0.27799070939236153</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>1.1402084208316436</t>
+          <t>1.1049826750880305</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>0.3281680200725084</t>
+          <t>0.34079958863888565</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.4048111483111472</t>
+          <t>1.3703319427938025</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.801298939065135</t>
+          <t>0.7869903961291587</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.6242965143826038</t>
+          <t>0.6562869859910475</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>1.9552431966840782</t>
+          <t>1.9914500892440472</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>8.0014389100003</t>
+          <t>7.979434800884368</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>11.36958738516831</t>
+          <t>11.19807058757315</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>13.34337490374677</t>
+          <t>13.235116755239538</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>1.1443963566430033</t>
+          <t>1.1423898193526818</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>1.9824754295638412</t>
+          <t>1.7953392698949315</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>3.9980065067431987</t>
+          <t>4.143016538857054</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>14.854705361116052</t>
+          <t>14.668292421120741</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>23.07395442650456</t>
+          <t>22.68671004531214</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>0.5459410097836628</t>
+          <t>0.5735483520183936</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>8.285152246732524</t>
+          <t>8.095432763905492</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>1.2861075168061495</t>
+          <t>1.294664927650323</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>0.52083427618496</t>
+          <t>0.5178197257544985</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>8.17580806742445</t>
+          <t>8.122770295046559</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>3.14089938425729</t>
+          <t>3.2580509388212597</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>14.779825771857723</t>
+          <t>14.775874804079699</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>0.5917289032239177</t>
+          <t>0.6285084486914435</t>
         </is>
       </c>
     </row>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>1.605708702168416</t>
+          <t>1.604484373017472</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>1.957235466379031</t>
+          <t>2.045661651845483</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>5.372546259500848</t>
+          <t>5.325068310202655</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>7.991090651171374</t>
+          <t>8.03303867198928</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>6.19234553986929</t>
+          <t>6.081200605544581</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>0.6755735835461798</t>
+          <t>0.681161715866025</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>6.318642185467169</t>
+          <t>6.191761106523138</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>7.057300892678327</t>
+          <t>7.029515512598131</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>1.519440388172085</t>
+          <t>1.599121552356608</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>10.40698309128574</t>
+          <t>10.22871955390339</t>
         </is>
       </c>
     </row>
@@ -8542,7 +8542,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>0.8566717554477196</t>
+          <t>0.9010992061283113</t>
         </is>
       </c>
     </row>
@@ -8564,7 +8564,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>0.7240926851766005</t>
+          <t>0.6764880247155247</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>24.109238146174437</t>
+          <t>23.60662468660984</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>5.099143537949175</t>
+          <t>5.8120361814273025</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>23.93888980398149</t>
+          <t>23.63124815763126</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>0.4558815311233534</t>
+          <t>0.4912887413647867</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.6034057443428419</t>
+          <t>0.6498075504218223</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>23.81318283384283</t>
+          <t>24.215831656547643</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>19.372284472055185</t>
+          <t>19.074868282446147</t>
         </is>
       </c>
     </row>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>4.464132610567243</t>
+          <t>4.429105789174327</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>3.3248194179309976</t>
+          <t>3.2590289598352866</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>4.452504690242627</t>
+          <t>4.408654540297153</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>9.607077684827601</t>
+          <t>9.708572722376786</t>
         </is>
       </c>
     </row>
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>5.499889809735308</t>
+          <t>5.506012575412364</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>7.529886212638512</t>
+          <t>7.388008753175241</t>
         </is>
       </c>
     </row>
@@ -9356,7 +9356,7 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>0.2886333862688523</t>
+          <t>0.3032129132480611</t>
         </is>
       </c>
     </row>
@@ -9378,7 +9378,7 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>0.27546898431367695</t>
+          <t>0.2718923215556574</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>0.9368678150352134</t>
+          <t>0.9153770251443437</t>
         </is>
       </c>
     </row>
@@ -9422,7 +9422,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>1.4416676392882435</t>
+          <t>1.363708964660395</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9444,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>2.288682555972997</t>
+          <t>2.418662622625007</t>
         </is>
       </c>
     </row>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>6.851043928973827</t>
+          <t>3.241464102498444</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>4.7650945147594985</t>
+          <t>4.838278114921345</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>16.047734681074303</t>
+          <t>15.881461867616842</t>
         </is>
       </c>
     </row>
@@ -9598,7 +9598,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>14.27699286422908</t>
+          <t>13.83246215592572</t>
         </is>
       </c>
     </row>
@@ -9620,7 +9620,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>2.802925606900415</t>
+          <t>2.8939299915603938</t>
         </is>
       </c>
     </row>
@@ -9708,7 +9708,7 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>2.6598050607150716</t>
+          <t>2.6328069882171206</t>
         </is>
       </c>
     </row>
@@ -9752,7 +9752,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>9.237631522771624</t>
+          <t>9.5625412698179</t>
         </is>
       </c>
     </row>
@@ -9774,7 +9774,227 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>40.26560463158606</t>
+          <t>40.05506045624512</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="1" t="inlineStr">
+        <is>
+          <t>425</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>F2P_PHY_Goku_Mini_Daima</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="1" t="inlineStr">
+        <is>
+          <t>426</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>F2P_INT_Vegeta_Mini_Daima</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="1" t="inlineStr">
+        <is>
+          <t>427</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>F2P_INT_Masked_Majin_Panzy</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="1" t="inlineStr">
+        <is>
+          <t>428</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>F2P_STR_Glorio</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="1" t="inlineStr">
+        <is>
+          <t>429</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>F2P_AGL_Manga_Goku</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="1" t="inlineStr">
+        <is>
+          <t>430</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>BU_PHY_Manga_Piccolo_Jr</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>0.3706989318842199</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="1" t="inlineStr">
+        <is>
+          <t>431</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>BU_STR_Manga_Vegeta</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="1" t="inlineStr">
+        <is>
+          <t>432</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>BU_TEQ_Manga_SS2_Gohan</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="1" t="inlineStr">
+        <is>
+          <t>433</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>BU_INT_Manga_Final_Form_Frieza</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>9.800042947424899</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="1" t="inlineStr">
+        <is>
+          <t>434</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>BU_AGL_Manga_Majin_Buu</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>0.5469621491631673</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Future gohan and trunks summons
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D439"/>
+  <dimension ref="A1:D444"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.2018746419228403</t>
+          <t>1.317101598251191</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.523288333772758</t>
+          <t>5.3356026821642</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.4390338660837303</t>
+          <t>0.4811252243246881</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.8995892141289816</t>
+          <t>2.0817079441390107</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5.479363455676221</t>
+          <t>5.304360145149349</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.8333333333333333</t>
+          <t>0.9132272426127037</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>7.003479206809121</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.6671871973200014</t>
+          <t>0.7311522294180514</t>
         </is>
       </c>
     </row>
@@ -815,12 +815,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.5778010619588624</t>
+          <t>0.6331964047096604</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.2663928094193209</t>
+          <t>1.387805296092674</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.9258912922177345</t>
+          <t>2.0614008583474157</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3.010313651506483</t>
+          <t>3.0110305976653775</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.693902648046337</t>
+          <t>0.7604289623004117</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1.387805296092674</t>
+          <t>1.5208579246008234</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.6671871973200014</t>
+          <t>0.7311522294180514</t>
         </is>
       </c>
     </row>
@@ -1013,12 +1013,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.9824684008871645</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.9214530598969362</t>
+          <t>0.8450024856517123</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>1.054503988707488</t>
+          <t>1.1556021239177248</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1.0007807959800024</t>
+          <t>1.096728344127077</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>9.218918178385737</t>
+          <t>8.942596546362797</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1.7334031858765866</t>
+          <t>1.8995892141289816</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2.709875908260541</t>
+          <t>3.007499584967011</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.6865977128541596</t>
+          <t>1.7114921266887766</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>0.8333333333333333</t>
+          <t>0.9132272426127037</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3.163511966122465</t>
+          <t>3.466806371753173</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>8.609942464440504</t>
+          <t>8.9155291752097</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>4.336282145857739</t>
+          <t>4.12777232536542</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>3.662627630180392</t>
+          <t>3.8357403093908182</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>11.666666666666664</t>
+          <t>12.78518139657785</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>1.317101598251191</t>
+          <t>1.4433756729740645</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>3.411804537888935</t>
+          <t>3.424147050400991</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>3.4659407282183747</t>
+          <t>3.6946828206479427</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.4761737182275684</t>
+          <t>0.5006930329182429</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>1.096728344127077</t>
+          <t>1.2018746419228403</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>0.9622504486493763</t>
+          <t>1.054503988707488</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.36035869412944965</t>
+          <t>0.3849622862097024</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0.45272777820095955</t>
+          <t>0.49150924832226206</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>0.5987832462807359</t>
+          <t>0.5937131654982567</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4.098113213848009</t>
+          <t>4.076831689929811</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>0.5555555555555556</t>
+          <t>0.6088181617418025</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.47589515502741003</t>
+          <t>0.4424976149686115</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>0.5087299629616816</t>
+          <t>0.46580238372174054</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>9.848557978410613</t>
+          <t>10.448845961093513</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.3641569043710687</t>
+          <t>0.3791652655047262</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>1.6362454267791797</t>
+          <t>1.62165231800223</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>0.4811252243246881</t>
+          <t>0.527251994353744</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>4.06046117494016</t>
+          <t>3.9860527656758884</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>0.6851523718378347</t>
+          <t>0.6481382416961651</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2.6464433715798674</t>
+          <t>2.553290373012608</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>0.5778010619588624</t>
+          <t>0.6331964047096604</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.20015615919600044</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>1.0007807959800024</t>
+          <t>1.096728344127077</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>5.34028350213552</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.20015615919600044</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>2.4037492838456807</t>
+          <t>2.634203196502382</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>0.36056239257685213</t>
+          <t>0.39513047947535734</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>1.0791265903033187</t>
+          <t>1.1243977796511169</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>0.4117294676241007</t>
+          <t>0.42213093647310695</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.23695509413413163</t>
+          <t>0.211943592995258</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>4.039743696149515</t>
+          <t>4.205517610242191</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1.3440137683271849</t>
+          <t>1.3624777515889923</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>0.30440908087090124</t>
+          <t>0.3335935986600007</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>0.3515013295691628</t>
+          <t>0.3852007079725748</t>
         </is>
       </c>
     </row>
@@ -4225,12 +4225,12 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>2.9108251089681088</t>
+          <t>0.23038838191942443</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -5039,7 +5039,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>2.2452510468485443</t>
+          <t>2.4605093069841395</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.590992051904661</t>
+          <t>2.340568978789372</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.3222946097810382</t>
+          <t>0.3027204468658454</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>8.576326001958186</t>
+          <t>8.097804619778884</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>4.788065201422363</t>
+          <t>4.778962590194347</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>0.9426594219932736</t>
+          <t>0.9430367217537945</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>0.36704675268573084</t>
+          <t>0.3515532794364562</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>0.40391097293258715</t>
+          <t>0.3976885464316451</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>7.85279126766011</t>
+          <t>7.888311819253616</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>0.49514762414423424</t>
+          <t>0.5216245466963807</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.5692715661697995</t>
+          <t>0.6146474125172223</t>
         </is>
       </c>
     </row>
@@ -5985,7 +5985,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>1.3879037978991942</t>
+          <t>1.3070872094491708</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.2156833150580725</t>
+          <t>0.2393860984181974</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>1.2256514922872725</t>
+          <t>1.2674210334402858</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>0.6352964405145025</t>
+          <t>0.6237902801063031</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>1.5567701270800032</t>
+          <t>1.7060218686421196</t>
         </is>
       </c>
     </row>
@@ -6557,12 +6557,12 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>0.2736880162267933</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>1.1042857942048965</t>
+          <t>0.9719876118407306</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>1.5567701270800032</t>
+          <t>1.7060218686421196</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>0.32025530081852915</t>
+          <t>0.3175781670853322</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.3933206341184812</t>
+          <t>1.3301463156134377</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.7841400819509121</t>
+          <t>0.7101995758141642</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>0.4261727132192617</t>
+          <t>0.4670310381240009</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.6418569812192334</t>
+          <t>0.6726909916852046</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>2.0422543505755577</t>
+          <t>2.120341998787347</t>
         </is>
       </c>
     </row>
@@ -7327,12 +7327,12 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>8.0224118494898</t>
+          <t>3.49506728095119</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>11.34403800003847</t>
+          <t>12.10544263382634</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>13.449005677085118</t>
+          <t>13.392618567395907</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>1.1722075447971407</t>
+          <t>1.181340997077648</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>1.9660401961237302</t>
+          <t>1.8264830277306405</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>4.1989529339203955</t>
+          <t>4.380954941789566</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>15.147145174266118</t>
+          <t>15.560033032678668</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>18.238798909221934</t>
+          <t>17.112806790797826</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>0.5510811987690402</t>
+          <t>0.5584407400568359</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>8.443458316211435</t>
+          <t>8.487883939733631</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>1.3084202772581712</t>
+          <t>1.299920072485215</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>0.5185319361248473</t>
+          <t>0.47575193596633625</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>8.551492210543751</t>
+          <t>9.79599499979006</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>3.335868997074721</t>
+          <t>3.743277284041671</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>14.452600846982811</t>
+          <t>13.010184714080815</t>
         </is>
       </c>
     </row>
@@ -7921,12 +7921,12 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>0.6174361888125667</t>
+          <t>0.38232928277723294</t>
         </is>
       </c>
     </row>
@@ -7992,7 +7992,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>0.9849721851039159</t>
+          <t>1.0794041191831907</t>
         </is>
       </c>
     </row>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>1.547284509851166</t>
+          <t>1.419048271191924</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>1.987871073392471</t>
+          <t>1.811694854213578</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>5.258860626964181</t>
+          <t>4.775106335458797</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>8.34615587164634</t>
+          <t>8.865383059568588</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>6.17088462727957</t>
+          <t>5.975815029786009</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>0.6654589518102249</t>
+          <t>0.6457988925761109</t>
         </is>
       </c>
     </row>
@@ -8295,12 +8295,12 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>0.2696404955808023</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>6.212365530829459</t>
+          <t>6.044128155272347</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>6.995378400445495</t>
+          <t>6.880308614840196</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>1.5523381573656263</t>
+          <t>1.7119453622031051</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>10.23717998179486</t>
+          <t>9.578617212179257</t>
         </is>
       </c>
     </row>
@@ -8542,7 +8542,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>0.8376360491382426</t>
+          <t>0.8988016519360076</t>
         </is>
       </c>
     </row>
@@ -8559,12 +8559,12 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>0.6987170999662544</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>24.355592288015373</t>
+          <t>24.110857674304754</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>5.147669406380416</t>
+          <t>4.079749757848603</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>24.018374781214924</t>
+          <t>24.100011026104642</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>0.466519533371276</t>
+          <t>0.4400447667842795</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.6081647681510437</t>
+          <t>0.5804071135913977</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>23.991212109437654</t>
+          <t>23.185118943086415</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>19.599279027517582</t>
+          <t>19.627079769963572</t>
         </is>
       </c>
     </row>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>4.517156022490273</t>
+          <t>4.484091720346303</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>3.2409593161472916</t>
+          <t>2.9714841940716585</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>4.627931237461654</t>
+          <t>4.367396108608081</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>9.695315544343899</t>
+          <t>9.873494095339751</t>
         </is>
       </c>
     </row>
@@ -9285,12 +9285,12 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>5.606575876277777</t>
+          <t>18.040935766396775</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>7.358697439463536</t>
+          <t>6.723176398497506</t>
         </is>
       </c>
     </row>
@@ -9351,12 +9351,12 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>0.29156509740737</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -9378,7 +9378,7 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>0.27844746628481937</t>
+          <t>0.2571247849858876</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>0.9095157719129833</t>
+          <t>0.813649453073825</t>
         </is>
       </c>
     </row>
@@ -9422,7 +9422,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>1.2170618712539518</t>
+          <t>1.225277182896666</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9444,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>2.350244450209942</t>
+          <t>1.9473046993213075</t>
         </is>
       </c>
     </row>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>1.46614185261953</t>
+          <t>1.5612493531952343</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>4.911571966378705</t>
+          <t>4.822275186490415</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>16.024396971129036</t>
+          <t>16.662385617303222</t>
         </is>
       </c>
     </row>
@@ -9598,7 +9598,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>13.32950753964379</t>
+          <t>11.80147383263223</t>
         </is>
       </c>
     </row>
@@ -9620,7 +9620,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>3.549734516910506</t>
+          <t>3.047191784869996</t>
         </is>
       </c>
     </row>
@@ -9708,7 +9708,7 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>2.6116598894512055</t>
+          <t>2.3733963100492086</t>
         </is>
       </c>
     </row>
@@ -9752,7 +9752,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>9.53698829486335</t>
+          <t>8.949001609974639</t>
         </is>
       </c>
     </row>
@@ -9774,7 +9774,7 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>39.84234619366222</t>
+          <t>42.32532922302563</t>
         </is>
       </c>
     </row>
@@ -9906,7 +9906,7 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>5.942937676661159</t>
+          <t>5.821591205089637</t>
         </is>
       </c>
     </row>
@@ -10016,7 +10016,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>51.7759985842511</t>
+          <t>53.44259384479737</t>
         </is>
       </c>
     </row>
@@ -10038,7 +10038,7 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>9.58991512834453</t>
+          <t>8.828850635620103</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10060,7 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>4.447409622692827</t>
+          <t>4.330420177683115</t>
         </is>
       </c>
     </row>
@@ -10083,6 +10083,116 @@
       <c r="D439" t="inlineStr">
         <is>
           <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="1" t="inlineStr">
+        <is>
+          <t>439</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>BU_INT_Androids_19_20</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="1" t="inlineStr">
+        <is>
+          <t>440</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>F2PLR_INT_Jackie_Chun</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="1" t="inlineStr">
+        <is>
+          <t>441</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>F2P_AGL_Piccolo_Jr</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="1" t="inlineStr">
+        <is>
+          <t>442</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>F2P_INT_Broly_Movie_Trunks</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="1" t="inlineStr">
+        <is>
+          <t>443</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>CLR_INT_Future_Gohan_Trunks</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>73.73078048738537</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Allow duplicate units in summons
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -9703,12 +9703,12 @@
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>2.3733963100492086</t>
+          <t>2.0622497345449142</t>
         </is>
       </c>
     </row>
@@ -10187,12 +10187,12 @@
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>73.73078048738537</t>
+          <t>12.274177075228536</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add New Years DF banners
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D444"/>
+  <dimension ref="A1:D446"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.3356026821642</t>
+          <t>5.473527238176587</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5.304360145149349</t>
+          <t>5.311176355840945</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.003479206809121</t>
+          <t>7.032646613750743</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2.0614008583474157</t>
+          <t>2.087082630694401</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3.0110305976653775</t>
+          <t>3.0415943197784054</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.8450024856517123</t>
+          <t>0.8530575830163791</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>8.942596546362797</t>
+          <t>8.956762835340434</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3.007499584967011</t>
+          <t>3.0422606126902796</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.7114921266887766</t>
+          <t>1.7443489708451876</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>8.9155291752097</t>
+          <t>9.06144234592061</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>4.12777232536542</t>
+          <t>4.189073453698123</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>3.8357403093908182</t>
+          <t>3.8917769124068085</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>3.424147050400991</t>
+          <t>3.4604491633286854</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>3.6946828206479427</t>
+          <t>3.724468526240514</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.5006930329182429</t>
+          <t>0.5104281988623417</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.3849622862097024</t>
+          <t>0.3833544606377244</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0.49150924832226206</t>
+          <t>0.49607543548344774</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>0.5937131654982567</t>
+          <t>0.5861946171635851</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4.076831689929811</t>
+          <t>4.078050690962144</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.4424976149686115</t>
+          <t>0.4454203730470037</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>0.46580238372174054</t>
+          <t>0.46056419557589506</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>10.448845961093513</t>
+          <t>10.413187508401085</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.3791652655047262</t>
+          <t>0.3767870572140275</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>1.62165231800223</t>
+          <t>1.6513593344579185</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>3.9860527656758884</t>
+          <t>3.908229522396541</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>0.6481382416961651</t>
+          <t>0.6478199788220182</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2.553290373012608</t>
+          <t>2.5636632279152543</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>5.34028350213552</t>
+          <t>5.28162386448918</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>1.1243977796511169</t>
+          <t>1.15461079740155</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.211943592995258</t>
+          <t>0.21448482880690187</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>4.205517610242191</t>
+          <t>4.30795682527773</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1.3624777515889923</t>
+          <t>1.3714319377921886</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>0.23038838191942443</t>
+          <t>0.23952110209630156</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.340568978789372</t>
+          <t>2.331493683434772</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.3027204468658454</t>
+          <t>0.29456833803954846</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>8.097804619778884</t>
+          <t>8.089232335807395</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>4.778962590194347</t>
+          <t>4.800384942173963</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>0.9430367217537945</t>
+          <t>0.9653491985850933</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>0.3515532794364562</t>
+          <t>0.3580230813671861</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>0.3976885464316451</t>
+          <t>0.3937003352742413</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>7.888311819253616</t>
+          <t>7.963978923592869</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>0.5216245466963807</t>
+          <t>0.5208131435291063</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>1.3070872094491708</t>
+          <t>1.305775226414863</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.2393860984181974</t>
+          <t>0.23549548605391102</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>1.2674210334402858</t>
+          <t>1.2968915620745998</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>0.6237902801063031</t>
+          <t>0.6270249185431762</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>0.9719876118407306</t>
+          <t>0.9925536855941326</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>0.3175781670853322</t>
+          <t>0.3156888911192743</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.3301463156134377</t>
+          <t>1.3659495558535735</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.7101995758141642</t>
+          <t>0.7215407882170508</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.6726909916852046</t>
+          <t>0.6684758328592033</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>2.120341998787347</t>
+          <t>2.1572813929433767</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>3.49506728095119</t>
+          <t>3.4814173360304217</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>12.10544263382634</t>
+          <t>12.24562135267711</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>13.392618567395907</t>
+          <t>13.52084994911661</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>1.181340997077648</t>
+          <t>1.1880486870304994</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>1.8264830277306405</t>
+          <t>1.882346471153289</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>4.380954941789566</t>
+          <t>4.324850921284426</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>15.560033032678668</t>
+          <t>15.68958604840993</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>17.112806790797826</t>
+          <t>17.034011467767876</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>0.5584407400568359</t>
+          <t>0.5439810315410089</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>8.487883939733631</t>
+          <t>8.59614795884794</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>1.299920072485215</t>
+          <t>1.311074177584412</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>0.47575193596633625</t>
+          <t>0.478283456122802</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>9.79599499979006</t>
+          <t>9.767025316096381</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>3.743277284041671</t>
+          <t>3.766062789163609</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>13.010184714080815</t>
+          <t>12.934049450237964</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>0.38232928277723294</t>
+          <t>0.3799492113684699</t>
         </is>
       </c>
     </row>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>1.419048271191924</t>
+          <t>1.405824632859204</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>1.811694854213578</t>
+          <t>1.754852303743439</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>4.775106335458797</t>
+          <t>4.81358763685753</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>8.865383059568588</t>
+          <t>8.941239690880497</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>5.975815029786009</t>
+          <t>6.075661839997571</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>0.6457988925761109</t>
+          <t>0.656467090097737</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>6.044128155272347</t>
+          <t>6.085452753076737</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>6.880308614840196</t>
+          <t>6.892706607441241</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>1.7119453622031051</t>
+          <t>1.67065464681619</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>9.578617212179257</t>
+          <t>9.741343292399367</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>24.110857674304754</t>
+          <t>24.319539596638123</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>4.079749757848603</t>
+          <t>3.9476075517086</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>24.100011026104642</t>
+          <t>24.276310633049626</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>0.4400447667842795</t>
+          <t>0.4310318365230144</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.5804071135913977</t>
+          <t>0.5665195366826327</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>23.185118943086415</t>
+          <t>23.209672099141386</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>19.627079769963572</t>
+          <t>19.84737726151606</t>
         </is>
       </c>
     </row>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>4.484091720346303</t>
+          <t>4.511781868845617</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>2.9714841940716585</t>
+          <t>2.968655107646743</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>4.367396108608081</t>
+          <t>4.356037629224545</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>9.873494095339751</t>
+          <t>9.825407378797223</t>
         </is>
       </c>
     </row>
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>18.040935766396775</t>
+          <t>18.193361460961412</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>6.723176398497506</t>
+          <t>6.819465210957303</t>
         </is>
       </c>
     </row>
@@ -9378,7 +9378,7 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>0.2571247849858876</t>
+          <t>0.26373985646880166</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>0.813649453073825</t>
+          <t>0.8180132662705097</t>
         </is>
       </c>
     </row>
@@ -9422,7 +9422,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>1.225277182896666</t>
+          <t>1.2444619179508116</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9444,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>1.9473046993213075</t>
+          <t>1.867271135784392</t>
         </is>
       </c>
     </row>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>1.5612493531952343</t>
+          <t>1.486829100138507</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>4.822275186490415</t>
+          <t>4.767637255992635</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>16.662385617303222</t>
+          <t>16.640067379190903</t>
         </is>
       </c>
     </row>
@@ -9598,7 +9598,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>11.80147383263223</t>
+          <t>11.90402632409664</t>
         </is>
       </c>
     </row>
@@ -9620,7 +9620,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>3.047191784869996</t>
+          <t>3.0396535217963745</t>
         </is>
       </c>
     </row>
@@ -9708,7 +9708,7 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>2.0622497345449142</t>
+          <t>2.06612061886257</t>
         </is>
       </c>
     </row>
@@ -9752,7 +9752,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>8.949001609974639</t>
+          <t>9.071240738747928</t>
         </is>
       </c>
     </row>
@@ -9774,7 +9774,7 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>42.32532922302563</t>
+          <t>42.47829928372439</t>
         </is>
       </c>
     </row>
@@ -9906,7 +9906,7 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>5.821591205089637</t>
+          <t>5.884959778445882</t>
         </is>
       </c>
     </row>
@@ -10016,7 +10016,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>53.44259384479737</t>
+          <t>53.344064852407186</t>
         </is>
       </c>
     </row>
@@ -10038,7 +10038,7 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>8.828850635620103</t>
+          <t>8.911361246342734</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10060,7 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>4.330420177683115</t>
+          <t>4.205017278063393</t>
         </is>
       </c>
     </row>
@@ -10192,7 +10192,51 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>12.274177075228536</t>
+          <t>12.093196356694977</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="1" t="inlineStr">
+        <is>
+          <t>444</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>DF_AGL_Gohan_Gamma1</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>22.860714566219535</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="1" t="inlineStr">
+        <is>
+          <t>445</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>DF_STR_Gamma2_Piccolo</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>56.99345644491073</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
New strongest T1 normal
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.473527238176587</t>
+          <t>5.453394090827377</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5.311176355840945</t>
+          <t>5.318982377315061</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.032646613750743</t>
+          <t>7.029438614704981</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2.087082630694401</t>
+          <t>2.0807333197320954</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3.0415943197784054</t>
+          <t>3.0612976586625877</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.8530575830163791</t>
+          <t>0.8463578949005178</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>8.956762835340434</t>
+          <t>8.94698391864735</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3.0422606126902796</t>
+          <t>3.030113826664308</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.7443489708451876</t>
+          <t>1.735837561684525</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>9.06144234592061</t>
+          <t>9.046263133321363</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>4.189073453698123</t>
+          <t>4.178396238344562</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>3.8917769124068085</t>
+          <t>3.88108025278483</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>3.4604491633286854</t>
+          <t>3.4652890805666283</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>3.724468526240514</t>
+          <t>3.7308582438491755</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.5104281988623417</t>
+          <t>0.5103634713730715</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.3833544606377244</t>
+          <t>0.38063382407725116</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0.49607543548344774</t>
+          <t>0.4936236538224028</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>0.5861946171635851</t>
+          <t>0.5814183692497968</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4.078050690962144</t>
+          <t>4.085028972119552</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.4454203730470037</t>
+          <t>0.44164971827090643</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>0.46056419557589506</t>
+          <t>0.45640413667261825</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>10.413187508401085</t>
+          <t>10.3983829227471</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.3767870572140275</t>
+          <t>0.37491668414130935</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>1.6513593344579185</t>
+          <t>1.6500176255460026</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>3.908229522396541</t>
+          <t>3.9004030905676204</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>0.6478199788220182</t>
+          <t>0.6419437281905944</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2.5636632279152543</t>
+          <t>2.5642281433111394</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>5.28162386448918</t>
+          <t>5.298618523148503</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>1.15461079740155</t>
+          <t>1.149208373712592</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.21448482880690187</t>
+          <t>0.2136892464376645</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>4.30795682527773</t>
+          <t>4.310880170091618</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1.3714319377921886</t>
+          <t>1.3620270930951186</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>0.23952110209630156</t>
+          <t>0.23921146204813834</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.331493683434772</t>
+          <t>2.310133773741166</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.29456833803954846</t>
+          <t>0.29156294680380196</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>8.089232335807395</t>
+          <t>8.101320149956578</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>4.800384942173963</t>
+          <t>4.808516354504086</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>0.9653491985850933</t>
+          <t>0.9627819262235657</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>0.3580230813671861</t>
+          <t>0.3558709057598657</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>0.3937003352742413</t>
+          <t>0.3908524273065783</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>7.963978923592869</t>
+          <t>7.962322994345996</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>0.5208131435291063</t>
+          <t>0.5184847789432183</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>1.305775226414863</t>
+          <t>1.3007987869626005</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.23549548605391102</t>
+          <t>0.2338491239936035</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>1.2968915620745998</t>
+          <t>1.2972043291166497</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>0.6270249185431762</t>
+          <t>0.6264919060123111</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>0.9925536855941326</t>
+          <t>0.9873795661098814</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>0.3156888911192743</t>
+          <t>0.31380707387427614</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.3659495558535735</t>
+          <t>1.3576799764822087</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.7215407882170508</t>
+          <t>0.7173412092553848</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.6684758328592033</t>
+          <t>0.6640907742226697</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>2.1572813929433767</t>
+          <t>2.1500357203843716</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>3.4814173360304217</t>
+          <t>3.4783529995709017</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>12.24562135267711</t>
+          <t>12.16961936230205</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>13.52084994911661</t>
+          <t>13.520098180079962</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>1.1880486870304994</t>
+          <t>1.1820141861226168</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>1.882346471153289</t>
+          <t>1.8742076093470799</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>4.324850921284426</t>
+          <t>4.306124630571519</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>15.68958604840993</t>
+          <t>15.658963692857037</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>17.034011467767876</t>
+          <t>17.049038678326077</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>0.5439810315410089</t>
+          <t>0.5420689551026929</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>8.59614795884794</t>
+          <t>8.596845584259283</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>1.311074177584412</t>
+          <t>1.309358719309192</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>0.478283456122802</t>
+          <t>0.47701033525097714</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>9.767025316096381</t>
+          <t>9.759871667775469</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>3.766062789163609</t>
+          <t>3.760577356024509</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>12.934049450237964</t>
+          <t>12.960453610750648</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>0.3799492113684699</t>
+          <t>0.3801953292987706</t>
         </is>
       </c>
     </row>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>1.405824632859204</t>
+          <t>1.393376980581201</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>1.754852303743439</t>
+          <t>1.742494812473059</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>4.81358763685753</t>
+          <t>4.77418418862251</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>8.941239690880497</t>
+          <t>8.915881756740017</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>6.075661839997571</t>
+          <t>6.059952223929109</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>0.656467090097737</t>
+          <t>0.651647042397018</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>6.085452753076737</t>
+          <t>6.080642171092613</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>6.892706607441241</t>
+          <t>6.902439585690935</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>1.67065464681619</t>
+          <t>1.6590991920503388</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>9.741343292399367</t>
+          <t>9.671261344259289</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>24.319539596638123</t>
+          <t>24.327393246852907</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>3.9476075517086</t>
+          <t>3.952830043398592</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>24.276310633049626</t>
+          <t>24.277243729223045</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>0.4310318365230144</t>
+          <t>0.4274150019989122</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.5665195366826327</t>
+          <t>0.56191528045561</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>23.209672099141386</t>
+          <t>23.258797230360706</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>19.84737726151606</t>
+          <t>19.899349921466225</t>
         </is>
       </c>
     </row>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>4.511781868845617</t>
+          <t>4.523863216752017</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>2.968655107646743</t>
+          <t>2.9621379054226447</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>4.356037629224545</t>
+          <t>4.321543701119355</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>9.825407378797223</t>
+          <t>9.857995687799075</t>
         </is>
       </c>
     </row>
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>18.193361460961412</t>
+          <t>18.1968201873957</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>6.819465210957303</t>
+          <t>6.764200935204028</t>
         </is>
       </c>
     </row>
@@ -9378,7 +9378,7 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>0.26373985646880166</t>
+          <t>0.26299220571393633</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>0.8180132662705097</t>
+          <t>0.8118247267504173</t>
         </is>
       </c>
     </row>
@@ -9422,7 +9422,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>1.2444619179508116</t>
+          <t>1.2373919772146786</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9444,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>1.867271135784392</t>
+          <t>1.8654147709301157</t>
         </is>
       </c>
     </row>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>1.486829100138507</t>
+          <t>1.483906731830788</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>4.767637255992635</t>
+          <t>4.761434365738809</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>16.640067379190903</t>
+          <t>16.68009896389494</t>
         </is>
       </c>
     </row>
@@ -9598,7 +9598,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>11.90402632409664</t>
+          <t>11.83719385850374</t>
         </is>
       </c>
     </row>
@@ -9620,7 +9620,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>3.0396535217963745</t>
+          <t>3.0342734689520476</t>
         </is>
       </c>
     </row>
@@ -9708,7 +9708,7 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>2.06612061886257</t>
+          <t>2.0534531828093083</t>
         </is>
       </c>
     </row>
@@ -9752,7 +9752,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>9.071240738747928</t>
+          <t>9.006452135502904</t>
         </is>
       </c>
     </row>
@@ -9774,7 +9774,7 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>42.47829928372439</t>
+          <t>42.36683811290101</t>
         </is>
       </c>
     </row>
@@ -9906,7 +9906,7 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>5.884959778445882</t>
+          <t>5.86588721427542</t>
         </is>
       </c>
     </row>
@@ -10016,7 +10016,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>53.344064852407186</t>
+          <t>53.33705166599155</t>
         </is>
       </c>
     </row>
@@ -10038,7 +10038,7 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>8.911361246342734</t>
+          <t>8.84752426805085</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10060,7 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>4.205017278063393</t>
+          <t>4.17752174675393</t>
         </is>
       </c>
     </row>
@@ -10192,7 +10192,7 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>12.093196356694977</t>
+          <t>12.138252969697177</t>
         </is>
       </c>
     </row>
@@ -10214,7 +10214,7 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>22.860714566219535</t>
+          <t>26.34999468340454</t>
         </is>
       </c>
     </row>
@@ -10236,7 +10236,7 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>56.99345644491073</t>
+          <t>54.35374626416631</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Initial NY Step Up Summons
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.317101598251191</t>
+          <t>1.4433756729740645</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.452020690416141</t>
+          <t>5.446866721690121</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.4811252243246881</t>
+          <t>0.527251994353744</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.0817079441390107</t>
+          <t>2.281286886901235</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5.326720459076871</t>
+          <t>5.332097027102871</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.9132272426127037</t>
+          <t>1.0007807959800024</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.052916280637967</t>
+          <t>7.051898903836293</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.7311522294180514</t>
+          <t>0.8012497612818937</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.6331964047096604</t>
+          <t>0.693902648046337</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.387805296092674</t>
+          <t>1.5208579246008234</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2.0759981060507284</t>
+          <t>2.0718352515060245</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2.808578338120519</t>
+          <t>2.809215116141685</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.7604289623004117</t>
+          <t>0.8333333333333333</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1.5208579246008234</t>
+          <t>1.6666666666666665</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.7311522294180514</t>
+          <t>0.8012497612818937</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.20817079441390107</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.8191991853626801</t>
+          <t>0.8180743625423681</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>1.1556021239177248</t>
+          <t>1.2663928094193209</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1.096728344127077</t>
+          <t>1.2018746419228403</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>8.990485240478371</t>
+          <t>8.985804148902648</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1.8995892141289816</t>
+          <t>2.0817079441390107</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3.04127654196299</t>
+          <t>3.03626892832906</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.7312741762225419</t>
+          <t>1.7293408366724834</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>0.9132272426127037</t>
+          <t>1.0007807959800024</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3.466806371753173</t>
+          <t>3.7991784282579633</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>8.943609982912891</t>
+          <t>8.768621780443937</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>4.137912225029143</t>
+          <t>3.310400285770183</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2.880783432445579</t>
+          <t>2.880545772603739</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>1.8264544852254074</t>
+          <t>2.0015615919600047</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>1.4433756729740645</t>
+          <t>1.5817559830612324</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>3.8294751001729423</t>
+          <t>3.830863797744318</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>3.7487671295843286</t>
+          <t>3.7498961957776515</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.5138406426044821</t>
+          <t>0.5139797199344653</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>1.2018746419228403</t>
+          <t>1.317101598251191</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>1.054503988707488</t>
+          <t>1.1556021239177248</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.37140075916084125</t>
+          <t>0.37096525868971547</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0.48959180667444224</t>
+          <t>0.4882465942292753</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>0.5578871854062714</t>
+          <t>0.6088181617418025</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4.119013276103878</t>
+          <t>4.118352964106435</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>0.6088181617418025</t>
+          <t>0.6671871973200014</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.44391590871184033</t>
+          <t>0.44335969943172343</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>0.4491359459719823</t>
+          <t>0.46260176536422465</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>10.369644483685523</t>
+          <t>10.509934344174505</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.37724338182611766</t>
+          <t>0.3765304336631434</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>1.6509838831038195</t>
+          <t>1.650218176924529</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>0.527251994353744</t>
+          <t>0.5778010619588624</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>3.8554829221582763</t>
+          <t>3.856647940548316</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>0.6329956130398727</t>
+          <t>0.631706049168806</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2.2647690801097093</t>
+          <t>2.259186032007402</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>0.6331964047096604</t>
+          <t>0.693902648046337</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>0.20015615919600044</t>
+          <t>0.2193456688254154</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>5.3386578187937515</t>
+          <t>5.148347433084852</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>0.20015615919600044</t>
+          <t>0.2193456688254154</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>2.634203196502382</t>
+          <t>2.886751345948129</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>0.39513047947535734</t>
+          <t>0.4330127018922193</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>1.1554172248004306</t>
+          <t>1.1559227860599854</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>0.42213093647310695</t>
+          <t>0.46260176536422465</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.21492692082068474</t>
+          <t>0.21513703899881698</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>4.269174507216054</t>
+          <t>4.259698170583151</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1.3675507562895077</t>
+          <t>1.3647263780398027</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>0.3335935986600007</t>
+          <t>0.3655761147090257</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>0.3852007079725748</t>
+          <t>0.42213093647310695</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>2.4605093069841395</t>
+          <t>2.6964049558080228</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.317204226887918</t>
+          <t>2.313308321412077</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.2839832809570614</t>
+          <t>0.28310183911630005</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>7.9925273369091485</t>
+          <t>8.002457065080847</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>4.8168275509302205</t>
+          <t>4.8175572966244005</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>0.9636748695697119</t>
+          <t>0.9611046100307579</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>0.2497585725119027</t>
+          <t>0.2490520615975722</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>0.38180463155216554</t>
+          <t>0.3806831702684232</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>7.9800683375087464</t>
+          <t>7.981209298903792</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>0.49839213005165117</t>
+          <t>0.4963572871668003</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.6146474125172223</t>
+          <t>0.6735753140545633</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>1.2854174618281284</t>
+          <t>1.2849114320382269</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.23563881752036017</t>
+          <t>0.2349305705115658</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>1.2990816490292483</t>
+          <t>1.3619762130453177</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>0.6213615858602939</t>
+          <t>0.6197677057911424</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>1.7060218686421196</t>
+          <t>1.8695827763244182</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>0.9892331138182566</t>
+          <t>0.984833862538129</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>1.7060218686421196</t>
+          <t>1.8695827763244182</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>0.3052613537589305</t>
+          <t>0.3045632433364596</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.3667572121072744</t>
+          <t>1.3666317145421953</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.7214449370633838</t>
+          <t>0.720745232851042</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>0.4670310381240009</t>
+          <t>0.5118065605926359</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.6538519593360621</t>
+          <t>0.6525816312670444</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>2.122826044759762</t>
+          <t>2.1183715454235985</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>3.742875349153959</t>
+          <t>3.74473467990715</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>12.05746286454855</t>
+          <t>12.01911015300918</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>13.48315319410888</t>
+          <t>13.308072646608942</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>1.195540592798038</t>
+          <t>1.1929800999889126</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>1.8826397006382705</t>
+          <t>2.051279870460281</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>4.3734272341919755</t>
+          <t>4.651804564448513</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>15.544580234683963</t>
+          <t>15.550853907731181</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>16.389265285688722</t>
+          <t>16.29762714015458</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>0.5346092678885458</t>
+          <t>0.5330923575517352</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>8.626920940512512</t>
+          <t>8.627216580860116</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>1.3026796353861332</t>
+          <t>1.3038991096993942</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>0.44147511906840364</t>
+          <t>0.4408527883538307</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>9.74172767774016</t>
+          <t>9.714159542573672</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>3.7540403980981374</t>
+          <t>3.752108407402641</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>12.936624081606283</t>
+          <t>12.252499562136078</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>0.5054697175592268</t>
+          <t>0.5059487770577432</t>
         </is>
       </c>
     </row>
@@ -7992,7 +7992,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>1.0794041191831907</t>
+          <t>1.1828894969117507</t>
         </is>
       </c>
     </row>
@@ -8009,12 +8009,12 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>1.369638004195441</t>
+          <t>0.7289102397586371</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>1.585283610714609</t>
+          <t>1.575498359004792</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>4.801493820686367</t>
+          <t>4.793199068655599</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>9.027321910134269</t>
+          <t>9.867226220061273</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>6.0671552293841815</t>
+          <t>6.068125689815709</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>0.6528851599960981</t>
+          <t>0.6521389098927619</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>6.095827752127289</t>
+          <t>6.042917200522417</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>3.582889878581966</t>
+          <t>3.586589242959704</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>1.6137744083182093</t>
+          <t>1.6077302192863927</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>9.716260480771847</t>
+          <t>9.691145194310385</t>
         </is>
       </c>
     </row>
@@ -8542,7 +8542,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>0.8988016519360076</t>
+          <t>0.9849721851039159</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>25.08121142525726</t>
+          <t>25.084831262463233</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>4.010788743184904</t>
+          <t>4.026668275862249</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>24.301234532769122</t>
+          <t>24.495906904416053</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>0.4184997398923854</t>
+          <t>0.4174128171977745</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.5565693523909259</t>
+          <t>0.5546895028478129</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>23.406245884558274</t>
+          <t>23.429479624870048</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>20.52627149702751</t>
+          <t>20.545307950496678</t>
         </is>
       </c>
     </row>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>4.9810511823537444</t>
+          <t>4.983729041356958</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>2.972936961846161</t>
+          <t>2.972206036429585</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>4.328324504115557</t>
+          <t>4.659622994626416</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>9.84209418498402</t>
+          <t>9.880765989594991</t>
         </is>
       </c>
     </row>
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>18.5944354649698</t>
+          <t>18.883098593207084</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>6.734817668622205</t>
+          <t>6.722392870402423</t>
         </is>
       </c>
     </row>
@@ -9378,7 +9378,7 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>0.3115155171050356</t>
+          <t>0.31108788299078277</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>0.8059390289958621</t>
+          <t>0.805639540960069</t>
         </is>
       </c>
     </row>
@@ -9422,7 +9422,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>1.166685763070424</t>
+          <t>1.1659713670672245</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9444,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>1.9070177994300364</t>
+          <t>1.9101275168396512</t>
         </is>
       </c>
     </row>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>1.423473491453324</t>
+          <t>1.419653387583357</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>4.749428504757009</t>
+          <t>4.878601078277417</t>
         </is>
       </c>
     </row>
@@ -9532,7 +9532,7 @@
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.2048824708390741</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>16.66921054744725</t>
+          <t>16.6231734873967</t>
         </is>
       </c>
     </row>
@@ -9598,7 +9598,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>11.85587025614679</t>
+          <t>11.80971984092477</t>
         </is>
       </c>
     </row>
@@ -9620,7 +9620,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>3.0334392024673207</t>
+          <t>3.0321887737120963</t>
         </is>
       </c>
     </row>
@@ -9708,7 +9708,7 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>2.0554179783299285</t>
+          <t>2.049672109878583</t>
         </is>
       </c>
     </row>
@@ -9752,7 +9752,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>8.96143774226424</t>
+          <t>8.942113887518767</t>
         </is>
       </c>
     </row>
@@ -9774,7 +9774,7 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>41.88776481433148</t>
+          <t>41.84119810179821</t>
         </is>
       </c>
     </row>
@@ -9906,7 +9906,7 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>5.904788228531778</t>
+          <t>5.871852641650472</t>
         </is>
       </c>
     </row>
@@ -10016,7 +10016,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>53.402869196798484</t>
+          <t>53.34397450054901</t>
         </is>
       </c>
     </row>
@@ -10038,7 +10038,7 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>8.783388583721248</t>
+          <t>8.76928237792506</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10060,7 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>4.189692754102724</t>
+          <t>4.18572177163142</t>
         </is>
       </c>
     </row>
@@ -10192,7 +10192,7 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>12.299272853250827</t>
+          <t>12.311600908961992</t>
         </is>
       </c>
     </row>
@@ -10214,7 +10214,7 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>25.99379473761343</t>
+          <t>27.13016174565653</t>
         </is>
       </c>
     </row>
@@ -10236,7 +10236,7 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>20.594093582907888</t>
+          <t>20.762999072156987</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NY Step Up Summons
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -969,7 +969,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2949,12 +2949,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2.259186032007402</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -4071,12 +4071,12 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>0.42213093647310695</t>
+          <t>0.21106546823655348</t>
         </is>
       </c>
     </row>
@@ -5501,12 +5501,12 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>4.8175572966244005</t>
+          <t>1.1874814616453477</t>
         </is>
       </c>
     </row>
@@ -7921,12 +7921,12 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>0.5059487770577432</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -8009,12 +8009,12 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>0.7289102397586371</t>
+          <t>0.9416231862323259</t>
         </is>
       </c>
     </row>
@@ -8251,12 +8251,12 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>6.068125689815709</t>
+          <t>3.1522512988899436</t>
         </is>
       </c>
     </row>
@@ -8295,7 +8295,7 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
@@ -8515,12 +8515,12 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>9.691145194310385</t>
+          <t>1.6892085406500001</t>
         </is>
       </c>
     </row>
@@ -8713,12 +8713,12 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>0.4174128171977745</t>
+          <t>0.5438322006452276</t>
         </is>
       </c>
     </row>
@@ -8911,12 +8911,12 @@
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.5546895028478129</t>
+          <t>0.5367532386900891</t>
         </is>
       </c>
     </row>
@@ -9417,12 +9417,12 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>1.1659713670672245</t>
+          <t>0.30006228566031456</t>
         </is>
       </c>
     </row>
@@ -9461,12 +9461,12 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>1.419653387583357</t>
+          <t>14.371367003566315</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 4000 day goku
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.74685470409246</t>
+          <t>6.4790755214902305</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3.746578547599808</t>
+          <t>3.813580451424619</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>6.120148846985221</t>
+          <t>5.456755624262623</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.41074376066408486</t>
+          <t>0.4102190563199619</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2.553480929692398</t>
+          <t>2.557670500177439</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1.1110756792947454</t>
+          <t>1.0798292817046762</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10.108348892956286</t>
+          <t>10.108706100044593</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3.8541878979342012</t>
+          <t>3.750323177956508</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2.2096780150824857</t>
+          <t>2.2238982493074166</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>5.431745932917669</t>
+          <t>5.2447800001205565</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2.026099695881819</t>
+          <t>1.6977672773917412</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>3.349128453304129</t>
+          <t>3.4227682337343914</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>6.348507134005853</t>
+          <t>6.482759661679495</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2.9162784120789644</t>
+          <t>2.4728219323486633</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.6667798042514477</t>
+          <t>0.6619270865372724</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.4028193093385412</t>
+          <t>0.37258589816035104</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>3.225815248434344</t>
+          <t>3.280171489876416</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.5786317057707349</t>
+          <t>0.5623455637768636</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>7.1933328174649604</t>
+          <t>5.7046244024045105</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.2970058480274846</t>
+          <t>0.2894178264171252</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>1.1973513475731963</t>
+          <t>1.220846629472831</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>2.804028436292348</t>
+          <t>3.551027695237188</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>0.6367182846963463</t>
+          <t>0.5944750627799527</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>5.459221258121378</t>
+          <t>4.842718355256733</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>4.466649905148204</t>
+          <t>4.0435210118891565</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>1.4088567747256378</t>
+          <t>1.4449747191285005</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.2813551694668952</t>
+          <t>0.28118495131116816</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>4.69375449813549</t>
+          <t>4.259738186849946</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1.809890457298733</t>
+          <t>1.8818836664031684</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>3.0010582092343037</t>
+          <t>2.901938401316272</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.2972965438375014</t>
+          <t>0.24503021055142843</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>6.2897554553522355</t>
+          <t>6.155336049534539</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>1.0223196211463517</t>
+          <t>0.997018553795499</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>0.7018384147353943</t>
+          <t>0.7206219889295419</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>0.27045164480064976</t>
+          <t>0.2753884053453408</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>0.23574334753072737</t>
+          <t>0.23199220010740565</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>0.22970090624105716</t>
+          <t>0.22615506563553261</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>6.756842357783903</t>
+          <t>6.462186613469434</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>0.3324890266789211</t>
+          <t>0.24284723055388024</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.6921524022464949</t>
+          <t>0.6735753140545633</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>1.2109312163304347</t>
+          <t>1.2106412462811948</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.34293080932847814</t>
+          <t>0.29422892207391355</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>2.2184723264434996</t>
+          <t>2.2497376803534013</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>0.7354743273175259</t>
+          <t>0.7192226731128111</t>
         </is>
       </c>
     </row>
@@ -6188,7 +6188,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>0.20290934983311892</t>
+          <t>0.20754694607635926</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>1.2453394347904005</t>
+          <t>1.2573217496236744</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.837763295943546</t>
+          <t>1.8479885251600223</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.9688459459376468</t>
+          <t>0.9408345137278369</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.5596947667989487</t>
+          <t>0.5250005451171186</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>1.5538092162323895</t>
+          <t>1.4464646057940163</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>4.3632683667832985</t>
+          <t>4.20035212607937</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>14.01262865751433</t>
+          <t>14.01754246192197</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>5.9815085610747225</t>
+          <t>12.895472437196371</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>1.1598293820202226</t>
+          <t>1.064588336577166</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>1.5920871685328812</t>
+          <t>1.5336616199241995</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>2.576640664652369</t>
+          <t>2.2715488169532305</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>10.508137732413362</t>
+          <t>10.035939744695568</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>16.091141756419752</t>
+          <t>16.758281116424584</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>8.826534419787093</t>
+          <t>8.986341862668242</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>1.0343845114571855</t>
+          <t>0.994412450068532</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>0.3587605762889705</t>
+          <t>0.3469167367146362</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>8.739590386784489</t>
+          <t>9.643955514779929</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>3.7160877426553203</t>
+          <t>3.362997077623609</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>14.614591485145155</t>
+          <t>14.582728804395188</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>1.1828894969117507</t>
+          <t>1.401824548813484</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>6.445610109414459</t>
+          <t>6.25920474034274</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>6.678296985518274</t>
+          <t>6.289775808437862</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>3.7741970078434126</t>
+          <t>3.8400293569609474</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>0.7786154385185391</t>
+          <t>0.793687030569119</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>6.72589050621906</t>
+          <t>6.821139151785316</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>2.1323395769423996</t>
+          <t>2.1068092211882714</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>1.185780290229832</t>
+          <t>1.34737696790514</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>2.1589600062696697</t>
+          <t>2.212976469472812</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>20.010579395819263</t>
+          <t>20.27706392141487</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>4.446863243902712</t>
+          <t>4.683648777727598</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>28.469050367387727</t>
+          <t>28.321746267924595</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>0.528792891653538</t>
+          <t>0.501019275880096</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.6834689290293248</t>
+          <t>0.6812457883642304</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>30.558463401570002</t>
+          <t>20.13402112061111</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>33.63128744615188</t>
+          <t>34.25855571805802</t>
         </is>
       </c>
     </row>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>14.568363014889982</t>
+          <t>14.674789824131759</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>3.4555583650286485</t>
+          <t>3.7416816683034355</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>3.557362172687966</t>
+          <t>3.3572840362722665</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>9.675418843914372</t>
+          <t>9.752880416331166</t>
         </is>
       </c>
     </row>
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>6.4065613125892265</t>
+          <t>6.053670203804272</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>8.588059674733625</t>
+          <t>8.4700440164383</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>0.8579949182404283</t>
+          <t>0.9272317458652477</t>
         </is>
       </c>
     </row>
@@ -9422,7 +9422,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>0.2721259051571723</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9444,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>1.608812127344294</t>
+          <t>1.738086484182361</t>
         </is>
       </c>
     </row>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>12.545906718640465</t>
+          <t>14.193744439351889</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>2.64716789114593</t>
+          <t>2.510869278617837</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>14.54062445132147</t>
+          <t>14.599855081038044</t>
         </is>
       </c>
     </row>
@@ -9598,7 +9598,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>15.97461228453971</t>
+          <t>16.07483934485834</t>
         </is>
       </c>
     </row>
@@ -9620,7 +9620,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>3.1413098524373995</t>
+          <t>3.061625664573515</t>
         </is>
       </c>
     </row>
@@ -9708,7 +9708,7 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>2.4793509244930414</t>
+          <t>2.461086931352713</t>
         </is>
       </c>
     </row>
@@ -9752,7 +9752,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>10.43461700022867</t>
+          <t>10.34395522708624</t>
         </is>
       </c>
     </row>
@@ -9774,7 +9774,7 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>37.42191907350624</t>
+          <t>46.94934283707943</t>
         </is>
       </c>
     </row>
@@ -9906,7 +9906,7 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>4.561831213565177</t>
+          <t>6.402952440250246</t>
         </is>
       </c>
     </row>
@@ -10016,7 +10016,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>47.10887006162139</t>
+          <t>46.92291292125338</t>
         </is>
       </c>
     </row>
@@ -10038,7 +10038,7 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>10.14218540797087</t>
+          <t>9.771501636130038</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10060,7 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>2.66339067097403</t>
+          <t>2.389230026287074</t>
         </is>
       </c>
     </row>
@@ -10192,7 +10192,7 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>13.377146527766854</t>
+          <t>13.769500968376036</t>
         </is>
       </c>
     </row>
@@ -10214,7 +10214,7 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>18.09009631692509</t>
+          <t>15.89812255279805</t>
         </is>
       </c>
     </row>
@@ -10236,7 +10236,7 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>16.45839441379634</t>
+          <t>16.076761729563827</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Buy Beast Gohan copies
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.42615297536145</t>
+          <t>6.50629812370353</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3.8335765264910067</t>
+          <t>3.820029699286002</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.291131823734859</t>
+          <t>5.308012939886482</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.4023146244803508</t>
+          <t>0.37288312075800534</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2.5456953734455294</t>
+          <t>2.500548572828365</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1.042863680477415</t>
+          <t>1.0047008131259638</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10.045772744925927</t>
+          <t>10.09280428168829</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3.6750935308707695</t>
+          <t>3.7647119084402885</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2.171610549545049</t>
+          <t>2.049002408355414</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>5.760255102103324</t>
+          <t>4.8707714080187134</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>5.164020106730408</t>
+          <t>5.1248353898633985</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>1.6491434275130008</t>
+          <t>1.669276727776249</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>3.421139930603008</t>
+          <t>3.3807372224404304</t>
         </is>
       </c>
     </row>
@@ -1409,12 +1409,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>26.378606852534734</t>
+          <t>10.56598564364404</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>6.525070821703425</t>
+          <t>6.486706452554311</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2.4946506172752607</t>
+          <t>2.5162193558399446</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.6551612017372871</t>
+          <t>0.6364143980533206</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.36122478174114847</t>
+          <t>0.34577904470346404</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>3.3092461724134523</t>
+          <t>3.3660467426911325</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.5440489916117015</t>
+          <t>0.5255700483687927</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>5.4830915226996755</t>
+          <t>3.5434152329344926</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.28227250415058386</t>
+          <t>0.27139048083418055</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>1.2222152949848708</t>
+          <t>1.2080959505300584</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>3.4507533896822378</t>
+          <t>3.2537146127145085</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>0.5734752047820725</t>
+          <t>0.5510855935534409</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>4.915952651400691</t>
+          <t>5.147915549676676</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>4.07895519495651</t>
+          <t>4.210829913721223</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>1.4293344891211035</t>
+          <t>1.4044254366429247</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.2739844070723887</t>
+          <t>0.26676438026069516</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>4.187885473237749</t>
+          <t>4.302815575810051</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1.8323893543282135</t>
+          <t>1.6751027782628762</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.787071958357862</t>
+          <t>2.733018700644969</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.2315808430948247</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>6.228009284928434</t>
+          <t>5.775148758822553</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>1.0064448021279162</t>
+          <t>1.0023872501712248</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>0.7148690982234334</t>
+          <t>0.6894086679415352</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>0.27059843448680887</t>
+          <t>0.2618339301868602</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>0.22759246151469548</t>
+          <t>0.22098448949347266</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>0.2218289183146394</t>
+          <t>0.2155974206943565</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>6.479559374358537</t>
+          <t>6.407427502453423</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>0.2363752595965174</t>
+          <t>0.22000819456148113</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>1.1869894707907374</t>
+          <t>1.1446056315761142</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.2831307895481918</t>
+          <t>0.2631985056419568</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>2.2526445222047458</t>
+          <t>2.1909791018051936</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>0.697452980617661</t>
+          <t>0.669499356514482</t>
         </is>
       </c>
     </row>
@@ -6188,7 +6188,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>0.20406420795604063</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>1.2269391912561094</t>
+          <t>1.2017886418064379</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.8237077486622641</t>
+          <t>1.7728316212051343</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.9130618617888904</t>
+          <t>0.8865416110424111</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.5046382062327719</t>
+          <t>0.4762182716319718</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>1.415401457863526</t>
+          <t>1.3459352255208303</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>4.15500567941239</t>
+          <t>3.9698017485872583</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>13.69424222519893</t>
+          <t>13.302815957583691</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>12.936232197600923</t>
+          <t>12.717734904993634</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>1.0359228708185535</t>
+          <t>1.0026059267128795</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>1.5155708917567594</t>
+          <t>1.507768181103991</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>2.1976402625292804</t>
+          <t>2.0678751146127627</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>9.87862832132172</t>
+          <t>9.64023411225122</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>16.897474363627268</t>
+          <t>17.14457417283218</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>8.902779739225354</t>
+          <t>8.76280521373368</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>0.9696405247681229</t>
+          <t>0.9210279361392871</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>0.3363556919912636</t>
+          <t>0.3220764622142367</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>9.583256182213562</t>
+          <t>9.25397153834698</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>3.3221467538306406</t>
+          <t>3.1412134893653914</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>14.731965342242683</t>
+          <t>14.833200618667382</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>1.338853834689929</t>
+          <t>1.284531081068161</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>6.069158648410628</t>
+          <t>5.885514812355384</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>6.168635979486111</t>
+          <t>5.909646224369787</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>3.83956455307981</t>
+          <t>3.7719589676200442</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>0.775049198170643</t>
+          <t>0.7430655793817662</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>6.825339426919342</t>
+          <t>6.749957536909861</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>2.128503620959222</t>
+          <t>2.1597132017247134</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>1.286196856507119</t>
+          <t>1.332670442363417</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>2.192114851256761</t>
+          <t>2.141847547276079</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>20.40199745693254</t>
+          <t>20.532541978561213</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>4.747004414353853</t>
+          <t>4.7229196750035385</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>28.327318130090784</t>
+          <t>27.96191851288087</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>0.48445665772482194</t>
+          <t>0.45767787021238093</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.6549000642264231</t>
+          <t>0.6086022366928662</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>20.331271797015404</t>
+          <t>21.174326884024964</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>34.87960522860293</t>
+          <t>36.122396904432655</t>
         </is>
       </c>
     </row>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>14.78858184090546</t>
+          <t>14.81571190601685</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>3.692631680723639</t>
+          <t>3.6001540415107707</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>3.234671240899309</t>
+          <t>2.270560833930396</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>9.817740380418144</t>
+          <t>10.29910176100357</t>
         </is>
       </c>
     </row>
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>5.923119974603203</t>
+          <t>5.853451382194352</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>8.238620545367597</t>
+          <t>8.030999234286531</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>0.8995522045103117</t>
+          <t>0.8812199991118153</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9444,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>1.7486953926685231</t>
+          <t>1.3989187759885482</t>
         </is>
       </c>
     </row>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>14.413734536074273</t>
+          <t>14.357247389356521</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>2.4625650487410176</t>
+          <t>2.305059465215974</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>14.768974715486479</t>
+          <t>15.09423551739844</t>
         </is>
       </c>
     </row>
@@ -9598,7 +9598,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>15.61766031403959</t>
+          <t>15.16108102752405</t>
         </is>
       </c>
     </row>
@@ -9620,7 +9620,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>3.0089947735980087</t>
+          <t>2.8227637540510884</t>
         </is>
       </c>
     </row>
@@ -9708,7 +9708,7 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>2.3978857132816422</t>
+          <t>2.32527717381633</t>
         </is>
       </c>
     </row>
@@ -9752,7 +9752,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>10.09085633586806</t>
+          <t>9.738563412711196</t>
         </is>
       </c>
     </row>
@@ -9774,7 +9774,7 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>46.49257034709279</t>
+          <t>44.829107071332</t>
         </is>
       </c>
     </row>
@@ -9906,7 +9906,7 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>6.254476273804688</t>
+          <t>6.120719777042568</t>
         </is>
       </c>
     </row>
@@ -10016,7 +10016,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>45.92158381916685</t>
+          <t>45.48565474710946</t>
         </is>
       </c>
     </row>
@@ -10038,7 +10038,7 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>9.50337235124281</t>
+          <t>9.155166158495684</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10060,7 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>2.293932364730086</t>
+          <t>2.106053891054453</t>
         </is>
       </c>
     </row>
@@ -10192,7 +10192,7 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>13.951443255578354</t>
+          <t>14.52526626239721</t>
         </is>
       </c>
     </row>
@@ -10214,7 +10214,7 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>15.36495582148302</t>
+          <t>14.68880936651485</t>
         </is>
       </c>
     </row>
@@ -10236,7 +10236,7 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>16.23546510025362</t>
+          <t>16.952557022349154</t>
         </is>
       </c>
     </row>
@@ -10258,7 +10258,7 @@
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>68.42421726234998</t>
+          <t>68.77515314466874</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add EZAs and Majin Kuu
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3.6398810171913603</t>
+          <t>4.466472600671301</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2.9075357712304686</t>
+          <t>3.3514384452412265</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>3.6762604704494857</t>
+          <t>4.533627908267188</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.2435953859484799</t>
+          <t>0.2930186431141339</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1.6368128395644845</t>
+          <t>1.9773242136529865</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>6.481921045393251</t>
+          <t>7.873231988734098</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2.3427806541190304</t>
+          <t>2.87077635711918</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.5208579246008234</t>
+          <t>1.700577841853358</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>5.211417549523055</t>
+          <t>5.546551989335376</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>3.4043797654692343</t>
+          <t>4.179825235863951</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>1.078632835661727</t>
+          <t>1.2903544730889507</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2.170984800424069</t>
+          <t>2.648668570148782</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>10.797557518585647</t>
+          <t>10.73436377849643</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>4.675207713739483</t>
+          <t>5.495760345972292</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2.396190685182994</t>
+          <t>2.668906846887444</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.4017974285145941</t>
+          <t>0.49439595648473145</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.2561291962766023</t>
+          <t>0.29059505630253235</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2.9203706729510515</t>
+          <t>3.1925462588229294</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.4172413558420799</t>
+          <t>0.45809166177549265</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>2.9821425362611507</t>
+          <t>3.472241768507491</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.207536133524335</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>0.7508020083518118</t>
+          <t>0.9101466944066381</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>1.9316725454976897</t>
+          <t>2.34333895431961</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>6.858463096673472</t>
+          <t>6.240890448270542</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>4.7874548967035055</t>
+          <t>4.741089868924704</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>0.8724174166762576</t>
+          <t>1.0657716097705539</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.20216786241533133</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>2.6989278060858366</t>
+          <t>3.2914091077864027</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1.2453034168225101</t>
+          <t>1.4428539891696008</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.279331562015056</t>
+          <t>2.404718281356613</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>6.691972758794009</t>
+          <t>6.518181497519635</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>1.0202038140282639</t>
+          <t>1.046519975382438</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>0.42591925624548765</t>
+          <t>0.522543714566837</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>0.20473463598726038</t>
+          <t>0.24844164572693295</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>2.8805854944093134</t>
+          <t>3.3843772020567826</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>0.6638835190267827</t>
+          <t>0.8185003114266763</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.23257889246026192</t>
+          <t>0.24611833527861388</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>1.4457232653914054</t>
+          <t>1.7685615169063635</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>0.438445811247858</t>
+          <t>0.5217332099676044</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.1274653842174829</t>
+          <t>1.370468758781921</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.6513598233271973</t>
+          <t>0.741480717074015</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.42317035995244384</t>
+          <t>0.44323690750919387</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>0.997731095591797</t>
+          <t>1.1775773668495604</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>2.3101817120121506</t>
+          <t>2.858447029403092</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>2.2230939340300315</t>
+          <t>2.7956152001785526</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>3.268911700880242</t>
+          <t>3.89120620767153</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>0.7310232548772905</t>
+          <t>0.8487182980058131</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>0.9830518219966571</t>
+          <t>1.198880550857906</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>1.6945082754133947</t>
+          <t>1.8678134329504443</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>6.0713967780659575</t>
+          <t>7.488548093605437</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>10.80969259189834</t>
+          <t>10.416528970764688</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>5.721302955327908</t>
+          <t>7.052577717344332</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>0.59071155900973</t>
+          <t>0.7108595616645838</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>0.20759023408254906</t>
+          <t>0.2454945818494938</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>4.463748691492391</t>
+          <t>5.466893199908068</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>1.9595332394002103</t>
+          <t>2.420693899945471</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>14.266356756853819</t>
+          <t>14.741001879122123</t>
         </is>
       </c>
     </row>
@@ -7992,7 +7992,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>5.745055486062067</t>
+          <t>7.428256983547752</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>4.489380556676227</t>
+          <t>4.988781765119781</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>4.134050607010536</t>
+          <t>4.978645170453265</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>2.4623776148158214</t>
+          <t>2.9796683607062313</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>0.5064227911703552</t>
+          <t>0.5855201419645022</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>4.747534767716421</t>
+          <t>5.667653656465009</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>2.2918670355201414</t>
+          <t>2.34306839091866</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>1.174480490551852</t>
+          <t>1.189998191904056</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>0.34736287874891936</t>
+          <t>0.4287999408239891</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>15.480177925821788</t>
+          <t>17.78980442939843</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>1.6556706795416432</t>
+          <t>1.0956631759465267</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>7.464323762752208</t>
+          <t>7.605289990076173</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>0.3759649647274439</t>
+          <t>0.4143285517885209</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.5537156623428492</t>
+          <t>0.5758558905221705</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>24.609908598226973</t>
+          <t>24.050312549064614</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>36.54918215559326</t>
+          <t>38.24398183829709</t>
         </is>
       </c>
     </row>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>10.924791816993443</t>
+          <t>12.811288081129234</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>2.089470261021128</t>
+          <t>2.5781436438955017</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>1.2661916395954158</t>
+          <t>1.4490655056065287</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>15.397655341040087</t>
+          <t>13.980914770199886</t>
         </is>
       </c>
     </row>
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>3.7817166974121617</t>
+          <t>4.658835642673839</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>5.884127837114169</t>
+          <t>6.640837979360156</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>0.68382207617559</t>
+          <t>0.789330583937073</t>
         </is>
       </c>
     </row>
@@ -9422,7 +9422,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>0.2636261319337816</t>
+          <t>0.31583743927483265</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9444,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>2.676861673144785</t>
+          <t>2.073264877282327</t>
         </is>
       </c>
     </row>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>13.930358730374756</t>
+          <t>14.52114988284984</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>1.512762873730088</t>
+          <t>1.859303560038776</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>13.908053351786407</t>
+          <t>15.065554557977755</t>
         </is>
       </c>
     </row>
@@ -9598,7 +9598,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>2.9184246520820896</t>
+          <t>3.58932297121196</t>
         </is>
       </c>
     </row>
@@ -9620,7 +9620,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>1.7860272674584443</t>
+          <t>2.198403480015154</t>
         </is>
       </c>
     </row>
@@ -9708,7 +9708,7 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>1.4326413319116025</t>
+          <t>1.6981128015170555</t>
         </is>
       </c>
     </row>
@@ -9752,7 +9752,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>1.3800472991305295</t>
+          <t>1.6954954178526496</t>
         </is>
       </c>
     </row>
@@ -9774,7 +9774,7 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>32.79162973418425</t>
+          <t>39.35271158179698</t>
         </is>
       </c>
     </row>
@@ -9906,7 +9906,7 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>4.685943036389515</t>
+          <t>5.388575141667327</t>
         </is>
       </c>
     </row>
@@ -10016,7 +10016,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>15.078765633309137</t>
+          <t>14.327230195809541</t>
         </is>
       </c>
     </row>
@@ -10038,7 +10038,7 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>3.972788337536712</t>
+          <t>4.873961476226842</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10060,7 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>1.827947129323935</t>
+          <t>1.926828384509411</t>
         </is>
       </c>
     </row>
@@ -10192,7 +10192,7 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>16.84381272270938</t>
+          <t>16.549226962144566</t>
         </is>
       </c>
     </row>
@@ -10214,7 +10214,7 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>10.37333103961539</t>
+          <t>12.14948586478016</t>
         </is>
       </c>
     </row>
@@ -10236,7 +10236,7 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>17.901185283044157</t>
+          <t>16.713985910408397</t>
         </is>
       </c>
     </row>
@@ -10258,7 +10258,7 @@
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>54.19605495627985</t>
+          <t>61.22361562241233</t>
         </is>
       </c>
     </row>
@@ -10302,7 +10302,7 @@
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t>10.033838166927339</t>
+          <t>11.665354373515996</t>
         </is>
       </c>
     </row>
@@ -10324,7 +10324,7 @@
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>41.89917280411432</t>
+          <t>43.53643062634067</t>
         </is>
       </c>
     </row>
@@ -10346,7 +10346,7 @@
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>29.089950076458823</t>
+          <t>25.55847411871501</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Fan Meet up banner
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D453"/>
+  <dimension ref="A1:D456"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3.6189084256432587</t>
+          <t>4.30982261817819</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2.935161679303848</t>
+          <t>3.347846263839125</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>3.492925085325443</t>
+          <t>4.237128636961418</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.2433723058740319</t>
+          <t>0.2869830875193282</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1.6056230483694518</t>
+          <t>1.915879972691015</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>4.749738047705847</t>
+          <t>4.3090482917999315</t>
         </is>
       </c>
     </row>
@@ -947,12 +947,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>11.467187820820207</t>
+          <t>2.2892604207703915</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>1.8181299415073662</t>
+          <t>2.184619160501915</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2.258848217992341</t>
+          <t>2.697676941163399</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.5208579246008234</t>
+          <t>1.6350296745026545</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>5.21524632971217</t>
+          <t>5.528824232904632</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>3.2003028446175654</t>
+          <t>3.800229258082414</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>1.03463105737264</t>
+          <t>1.2044497537344423</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2.18537054968613</t>
+          <t>2.592566705794681</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>10.821867344147087</t>
+          <t>10.789091190132895</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>4.685478722667127</t>
+          <t>5.411044592162347</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2.394912618383143</t>
+          <t>2.654217567956063</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.3957657798228859</t>
+          <t>0.47555922500819997</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.2534869348722403</t>
+          <t>0.28066083054268276</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2.9495516612093695</t>
+          <t>3.211803060341289</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.41145081970204783</t>
+          <t>0.44194241223509834</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>2.650094784396126</t>
+          <t>2.9806476029400923</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.20101105163865388</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>0.7604495023841481</t>
+          <t>0.9021480193585703</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>1.873422833727022</t>
+          <t>2.24792284293784</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>7.036894630079938</t>
+          <t>6.502620730847667</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>4.755079979698225</t>
+          <t>4.7546985407939495</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>0.8810727817673423</t>
+          <t>1.039795768584446</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>2.735781942450912</t>
+          <t>3.232516750339026</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1.180205105536102</t>
+          <t>1.3328620571762622</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.219168256749705</t>
+          <t>2.285829654121476</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>6.719692008053329</t>
+          <t>6.548220703254913</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>1.0119584012834508</t>
+          <t>1.056370441484205</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>0.43065669104558624</t>
+          <t>0.5133843197934596</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>0.2047768956777576</t>
+          <t>0.2417261700627087</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>2.904887681418238</t>
+          <t>3.3602643779963657</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>0.6331031443487983</t>
+          <t>0.7672426521811196</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.22921519719153993</t>
+          <t>0.23776948608738446</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>1.4681268061528976</t>
+          <t>1.74510183889338</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>0.4479233203297479</t>
+          <t>0.523523433385809</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.1403472547818734</t>
+          <t>1.3404492311628557</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.6430214654581548</t>
+          <t>0.7105922285285162</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.41510463292129124</t>
+          <t>0.4254590798801524</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>0.9888949955580807</t>
+          <t>1.125419323875216</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>2.3130852266200304</t>
+          <t>2.8257499431752393</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>2.326213208977097</t>
+          <t>2.745896588911024</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>1.0687089394868927</t>
+          <t>1.281449273752191</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>0.7127017977139133</t>
+          <t>0.801754150987608</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>1.2461457974838952</t>
+          <t>1.31393530461445</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>1.6259409549620552</t>
+          <t>1.7510670673769635</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>6.046619564236102</t>
+          <t>7.229276335711776</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>10.721274547450335</t>
+          <t>10.33674347651268</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>0.5745703450702223</t>
+          <t>0.6769461640028774</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>0.20089330998291954</t>
+          <t>0.23266742317394762</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>4.315767929725151</t>
+          <t>5.162700461837169</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>1.9774759936733464</t>
+          <t>2.3840079659203894</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>14.370096394889025</t>
+          <t>14.956589555022411</t>
         </is>
       </c>
     </row>
@@ -7992,7 +7992,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>5.470742320493845</t>
+          <t>6.405049459017242</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>4.434445408046249</t>
+          <t>4.789564589755713</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>4.055538562667838</t>
+          <t>4.741406491520565</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>2.4719518495059702</t>
+          <t>2.9432453123150175</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>0.5126524395391558</t>
+          <t>0.570482488235323</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>4.70871445926052</t>
+          <t>5.562552750224889</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>2.276390457106295</t>
+          <t>2.350066513259172</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>1.160186562987866</t>
+          <t>1.167512756851789</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>0.34580027823312953</t>
+          <t>0.41646147842361003</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>15.722231523410581</t>
+          <t>17.82541396792793</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>1.6305999156221986</t>
+          <t>1.1251831607925027</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>7.529434397016729</t>
+          <t>7.726280528542965</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>0.366467590914896</t>
+          <t>0.3927103495842241</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.5379814653016577</t>
+          <t>0.551380716091207</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>24.635553194605855</t>
+          <t>24.23625629002064</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>28.933492787274403</t>
+          <t>33.510157004355</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>1.3754571055697669</t>
+          <t>1.6786570626328785</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>1.203739612436104</t>
+          <t>1.29726117645653</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>15.08507428810308</t>
+          <t>13.779317755205625</t>
         </is>
       </c>
     </row>
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>3.7382002161607435</t>
+          <t>4.475382539221986</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>5.83724611124511</t>
+          <t>6.391963162153277</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>0.6637039662338919</t>
+          <t>0.7457077900390243</t>
         </is>
       </c>
     </row>
@@ -9422,7 +9422,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>0.2547082762548154</t>
+          <t>0.2971321431385361</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9444,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>2.6216562666622707</t>
+          <t>2.086961482338836</t>
         </is>
       </c>
     </row>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>14.082222665876841</t>
+          <t>14.709392218948096</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>1.4484441630987184</t>
+          <t>1.7400769528151092</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>14.042980039558373</t>
+          <t>15.093580989180651</t>
         </is>
       </c>
     </row>
@@ -9598,7 +9598,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>2.894153070303096</t>
+          <t>3.4934163623209393</t>
         </is>
       </c>
     </row>
@@ -9620,7 +9620,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>1.7665789363048745</t>
+          <t>2.1309610618887755</t>
         </is>
       </c>
     </row>
@@ -9708,7 +9708,7 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>1.3943182301751031</t>
+          <t>1.615262749127865</t>
         </is>
       </c>
     </row>
@@ -9752,7 +9752,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>1.393832548035311</t>
+          <t>1.6589590783032904</t>
         </is>
       </c>
     </row>
@@ -9774,7 +9774,7 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>32.57537779901678</t>
+          <t>38.42139402188072</t>
         </is>
       </c>
     </row>
@@ -9906,7 +9906,7 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>4.525917284752323</t>
+          <t>5.184064748411103</t>
         </is>
       </c>
     </row>
@@ -10016,7 +10016,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>15.199652986887967</t>
+          <t>14.340037224514765</t>
         </is>
       </c>
     </row>
@@ -10038,7 +10038,7 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>3.9152160841542365</t>
+          <t>4.66831932921339</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10060,7 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>1.7997417864253242</t>
+          <t>1.903145031492121</t>
         </is>
       </c>
     </row>
@@ -10192,7 +10192,7 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>16.912469623791957</t>
+          <t>16.85710178996068</t>
         </is>
       </c>
     </row>
@@ -10214,7 +10214,7 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>9.768363973311201</t>
+          <t>11.18917450967932</t>
         </is>
       </c>
     </row>
@@ -10236,7 +10236,7 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>17.759923925012153</t>
+          <t>16.845507121255295</t>
         </is>
       </c>
     </row>
@@ -10258,7 +10258,7 @@
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>53.38652648099045</t>
+          <t>59.7259804551319</t>
         </is>
       </c>
     </row>
@@ -10302,7 +10302,7 @@
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t>10.249531281582659</t>
+          <t>11.413042588328892</t>
         </is>
       </c>
     </row>
@@ -10324,7 +10324,7 @@
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>35.03947874395172</t>
+          <t>35.36957375262423</t>
         </is>
       </c>
     </row>
@@ -10346,7 +10346,7 @@
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>21.810157205100126</t>
+          <t>19.38866486693088</t>
         </is>
       </c>
     </row>
@@ -10368,7 +10368,7 @@
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t>11.724064056963833</t>
+          <t>12.438408696593985</t>
         </is>
       </c>
     </row>
@@ -10389,6 +10389,72 @@
         </is>
       </c>
       <c r="D453" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="1" t="inlineStr">
+        <is>
+          <t>453</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>F2P_PHY_Tamagami_3</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="1" t="inlineStr">
+        <is>
+          <t>454</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>F2P_TEQ_Tamagami_2</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="1" t="inlineStr">
+        <is>
+          <t>455</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>F2P_AGL_Tamagami_1</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>

</xml_diff>

<commit_message>
11th Anni Part II summons
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D456"/>
+  <dimension ref="A1:D460"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.30982261817819</t>
+          <t>4.28755028044265</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3.347846263839125</t>
+          <t>3.23867066363952</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>4.237128636961418</t>
+          <t>3.7941030743331177</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.2869830875193282</t>
+          <t>0.25803028104965187</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1.915879972691015</t>
+          <t>1.825673014980635</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>4.3090482917999315</t>
+          <t>4.69754621821748</t>
         </is>
       </c>
     </row>
@@ -947,12 +947,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2.2892604207703915</t>
+          <t>9.099419200086134</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2.184619160501915</t>
+          <t>2.1222673789034645</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2.697676941163399</t>
+          <t>2.3019642961449804</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.6350296745026545</t>
+          <t>1.5596898075731822</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>5.528824232904632</t>
+          <t>5.569624501252605</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>3.800229258082414</t>
+          <t>3.8105502863629974</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>1.2044497537344423</t>
+          <t>1.165865245830375</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2.592566705794681</t>
+          <t>2.5813499247359495</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>10.789091190132895</t>
+          <t>11.131526226866951</t>
         </is>
       </c>
     </row>
@@ -1431,12 +1431,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>1.7334031858765866</t>
+          <t>9.755494402027226</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>5.411044592162347</t>
+          <t>5.333842942247284</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2.654217567956063</t>
+          <t>2.6714441933556685</t>
         </is>
       </c>
     </row>
@@ -1541,12 +1541,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0.47555922500819997</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.28066083054268276</t>
+          <t>0.2471842372372613</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>3.211803060341289</t>
+          <t>3.200203135008799</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.44194241223509834</t>
+          <t>0.4199633666376798</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>2.9806476029400923</t>
+          <t>2.8301279313505274</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.20101105163865388</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>0.9021480193585703</t>
+          <t>0.887459202221322</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>2.24792284293784</t>
+          <t>1.9732509734463628</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>6.502620730847667</t>
+          <t>6.5342470249340705</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>4.7546985407939495</t>
+          <t>4.786881156613128</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>1.039795768584446</t>
+          <t>1.017050323776138</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>3.232516750339026</t>
+          <t>3.026164078380308</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1.3328620571762622</t>
+          <t>1.258366014764205</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.285829654121476</t>
+          <t>2.193954426258119</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>6.548220703254913</t>
+          <t>6.62007289158727</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>1.056370441484205</t>
+          <t>1.021571957992336</t>
         </is>
       </c>
     </row>
@@ -5523,12 +5523,12 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>0.5133843197934596</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -5550,7 +5550,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>0.2417261700627087</t>
+          <t>0.23376534078408717</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>3.3602643779963657</t>
+          <t>3.2588736371990237</t>
         </is>
       </c>
     </row>
@@ -5875,12 +5875,12 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.7381527920952418</t>
+          <t>0.24909239792527116</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>0.7672426521811196</t>
+          <t>0.7365781034955258</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>0.23776948608738446</t>
+          <t>0.21397956056319323</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>1.74510183889338</t>
+          <t>1.6931976473612917</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>0.523523433385809</t>
+          <t>0.46703934523814006</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.3404492311628557</t>
+          <t>1.311957233125776</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.7105922285285162</t>
+          <t>0.690516873543308</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.4254590798801524</t>
+          <t>0.38849075935245597</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>1.125419323875216</t>
+          <t>1.0609466799148697</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>2.8257499431752393</t>
+          <t>2.586290116982299</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>2.745896588911024</t>
+          <t>2.5903373006673425</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>1.281449273752191</t>
+          <t>1.4637885642892794</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>0.801754150987608</t>
+          <t>0.7472078987193504</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>1.31393530461445</t>
+          <t>1.0166121967654327</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>1.7510670673769635</t>
+          <t>1.6007638354151146</t>
         </is>
       </c>
     </row>
@@ -7613,12 +7613,12 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>7.229276335711776</t>
+          <t>11.756464036470842</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>10.33674347651268</t>
+          <t>10.789891098437124</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>0.6769461640028774</t>
+          <t>0.6263326217526188</t>
         </is>
       </c>
     </row>
@@ -7789,12 +7789,12 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>0.23266742317394762</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>5.162700461837169</t>
+          <t>4.747161788227508</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>2.3840079659203894</t>
+          <t>2.1362568690624997</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>14.956589555022411</t>
+          <t>15.029954829926254</t>
         </is>
       </c>
     </row>
@@ -7992,7 +7992,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>6.405049459017242</t>
+          <t>6.311048972625623</t>
         </is>
       </c>
     </row>
@@ -8141,12 +8141,12 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>4.789564589755713</t>
+          <t>1.1375846640129748</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>4.741406491520565</t>
+          <t>4.416019046183307</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>2.9432453123150175</t>
+          <t>2.8032849122671983</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>0.570482488235323</t>
+          <t>0.5440008877531799</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>5.562552750224889</t>
+          <t>5.418856670201446</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>2.350066513259172</t>
+          <t>2.3507265321933843</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>1.167512756851789</t>
+          <t>1.614436412577731</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>0.41646147842361003</t>
+          <t>0.40006593917028965</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>17.82541396792793</t>
+          <t>17.904350163030273</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>1.1251831607925027</t>
+          <t>1.1689395545288193</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>7.726280528542965</t>
+          <t>7.750529398587055</t>
         </is>
       </c>
     </row>
@@ -8713,12 +8713,12 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>0.3927103495842241</t>
+          <t>0.5708613748923799</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.551380716091207</t>
+          <t>0.5010732042623538</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>24.23625629002064</t>
+          <t>24.89183805428351</t>
         </is>
       </c>
     </row>
@@ -8955,12 +8955,12 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>33.510157004355</t>
+          <t>18.563091902572403</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>1.6786570626328785</t>
+          <t>1.5622062754168293</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>1.29726117645653</t>
+          <t>1.2587634343869318</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>13.779317755205625</t>
+          <t>14.363465644931807</t>
         </is>
       </c>
     </row>
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>4.475382539221986</t>
+          <t>4.020939838343255</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>6.391963162153277</t>
+          <t>6.239121339594775</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>0.7457077900390243</t>
+          <t>0.7197825109570961</t>
         </is>
       </c>
     </row>
@@ -9422,7 +9422,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>0.2971321431385361</t>
+          <t>0.2867382291064562</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9444,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>2.086961482338836</t>
+          <t>2.258221930320474</t>
         </is>
       </c>
     </row>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>14.709392218948096</t>
+          <t>14.791545502479098</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>1.7400769528151092</t>
+          <t>1.549425182390425</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>15.093580989180651</t>
+          <t>14.932224285756327</t>
         </is>
       </c>
     </row>
@@ -9598,7 +9598,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>3.4934163623209393</t>
+          <t>3.2754877884620015</t>
         </is>
       </c>
     </row>
@@ -9620,7 +9620,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>2.1309610618887755</t>
+          <t>1.901263463652948</t>
         </is>
       </c>
     </row>
@@ -9708,7 +9708,7 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>1.615262749127865</t>
+          <t>1.5322314294068957</t>
         </is>
       </c>
     </row>
@@ -9752,7 +9752,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>1.6589590783032904</t>
+          <t>1.5955682060351801</t>
         </is>
       </c>
     </row>
@@ -9774,7 +9774,7 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>38.42139402188072</t>
+          <t>36.30101614655761</t>
         </is>
       </c>
     </row>
@@ -9906,7 +9906,7 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>5.184064748411103</t>
+          <t>5.043588295419466</t>
         </is>
       </c>
     </row>
@@ -10016,7 +10016,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>14.340037224514765</t>
+          <t>15.020261512899685</t>
         </is>
       </c>
     </row>
@@ -10038,7 +10038,7 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>4.66831932921339</t>
+          <t>4.470701308412828</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10060,7 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>1.903145031492121</t>
+          <t>1.6374786555429828</t>
         </is>
       </c>
     </row>
@@ -10192,7 +10192,7 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>16.85710178996068</t>
+          <t>17.12935671532616</t>
         </is>
       </c>
     </row>
@@ -10214,7 +10214,7 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>11.18917450967932</t>
+          <t>10.29851455434736</t>
         </is>
       </c>
     </row>
@@ -10236,7 +10236,7 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>16.845507121255295</t>
+          <t>17.2520602584068</t>
         </is>
       </c>
     </row>
@@ -10258,7 +10258,7 @@
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>59.7259804551319</t>
+          <t>59.86137130224857</t>
         </is>
       </c>
     </row>
@@ -10302,7 +10302,7 @@
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t>11.413042588328892</t>
+          <t>11.201634982349042</t>
         </is>
       </c>
     </row>
@@ -10324,7 +10324,7 @@
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>35.36957375262423</t>
+          <t>34.81275163420027</t>
         </is>
       </c>
     </row>
@@ -10346,7 +10346,7 @@
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>19.38866486693088</t>
+          <t>20.558452271595513</t>
         </is>
       </c>
     </row>
@@ -10368,7 +10368,7 @@
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t>12.438408696593985</t>
+          <t>12.643766929864436</t>
         </is>
       </c>
     </row>
@@ -10457,6 +10457,94 @@
       <c r="D456" t="inlineStr">
         <is>
           <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="1" t="inlineStr">
+        <is>
+          <t>456</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>DF_INT_SSGSS_Vegeta</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>7.197052361782508</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="1" t="inlineStr">
+        <is>
+          <t>457</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>BU_AGL_Ledgic</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>13.15035559753548</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="1" t="inlineStr">
+        <is>
+          <t>458</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>DFLR_INT_SS4_Vegeta_Goku</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>5.546617136646006</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="1" t="inlineStr">
+        <is>
+          <t>459</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>CLR_PHY_UI_Goku_SSGSSE_Vegeta</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>3.6166851286845945</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Buy copy of Kai Goku
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D460"/>
+  <dimension ref="A1:D463"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.952314620980141</t>
+          <t>4.5373933773505595</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3.4558250301612117</t>
+          <t>3.366373122324899</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>4.485238087100072</t>
+          <t>1.4211486170404626</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.23901434692247872</t>
+          <t>0.25201120920720244</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2.3547873114782463</t>
+          <t>2.401842303864301</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>4.56192391490669</t>
+          <t>5.836567035783441</t>
         </is>
       </c>
     </row>
@@ -947,12 +947,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>8.839017265404578</t>
+          <t>6.439003772009604</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2.1594169393842595</t>
+          <t>1.9925460074912045</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2.9478745582627894</t>
+          <t>3.1197839532069302</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.6666666666666665</t>
+          <t>1.8733149685941985</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>6.057904066606328</t>
+          <t>7.654281685776174</t>
         </is>
       </c>
     </row>
@@ -1277,12 +1277,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>26.793366278564722</t>
+          <t>12.713426375035983</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>3.454872006895405</t>
+          <t>1.3696775056958161</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>1.3110398933830278</t>
+          <t>0.8098016813458584</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2.693059565912403</t>
+          <t>2.9100403513602586</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>11.131571221058953</t>
+          <t>8.240460137777417</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>4.475514274157544</t>
+          <t>5.528785109137439</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2.2269268599825813</t>
+          <t>1.6004455008951826</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>3.557516755073614</t>
+          <t>3.3990425664866493</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.4337603705916653</t>
+          <t>0.4595994185994283</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>3.493579379601613</t>
+          <t>1.4888564619077667</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>0.33340624724744394</t>
+          <t>0.46151494387686953</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>0.8592337042894796</t>
+          <t>0.8693991018659801</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>1.6549776853234575</t>
+          <t>1.0783846467002933</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>6.476756114397293</t>
+          <t>6.375169835743822</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>5.629191584400591</t>
+          <t>10.59390656474744</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>1.1003956633055718</t>
+          <t>1.5876438765312355</t>
         </is>
       </c>
     </row>
@@ -3917,7 +3917,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>2.99890425908716</t>
+          <t>2.911933849128296</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>1.4089238748332131</t>
+          <t>1.5828207520481072</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2.076289377051222</t>
+          <t>2.290062990128732</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>6.840421513633402</t>
+          <t>6.84578237294366</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>0.9807638791040604</t>
+          <t>0.907196294641416</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>4.391507851617629</t>
+          <t>4.018700902749259</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.2403011173814012</t>
+          <t>0.2875955488858465</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>0.7390308294774428</t>
+          <t>0.6721988674794598</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>1.5658129358579322</t>
+          <t>1.3882903356541638</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>0.4246226676617728</t>
+          <t>0.44096811358460114</t>
         </is>
       </c>
     </row>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>1.3792583770458149</t>
+          <t>1.414651804613345</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>0.71840368679843</t>
+          <t>0.7646782960405871</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.3669132510680256</t>
+          <t>0.40811243561810584</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>0.9990984383625267</t>
+          <t>0.20022325014331877</t>
         </is>
       </c>
     </row>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>2.860041787855309</t>
+          <t>1.9179916722303698</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>2.798000371567052</t>
+          <t>1.9767612683001383</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>1.4986182763762983</t>
+          <t>1.40534255544455</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>0.5493395544672325</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>1.4766824489204282</t>
+          <t>1.4526053396976915</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>1.3547169796604352</t>
+          <t>1.3222021125024392</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>10.840331846097772</t>
+          <t>3.259997177909449</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>10.184394489600678</t>
+          <t>9.944456345415064</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>0.6234167440361564</t>
+          <t>0.6427303889872878</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>4.601581717834051</t>
+          <t>3.437550436612261</t>
         </is>
       </c>
     </row>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>1.9827343964380617</t>
+          <t>2.2591889730482</t>
         </is>
       </c>
     </row>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>13.70839455575554</t>
+          <t>13.580382838207804</t>
         </is>
       </c>
     </row>
@@ -7992,7 +7992,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>6.52910194903757</t>
+          <t>3.910527149987851</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>1.1849363641921355</t>
+          <t>1.1956489868592035</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>4.011772167512062</t>
+          <t>2.686511932085389</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>2.849232232671369</t>
+          <t>2.2502294799688087</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>0.563103163986796</t>
+          <t>0.7841851967875364</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8322,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>5.639125386177021</t>
+          <t>5.396138440578857</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>4.012180009516243</t>
+          <t>3.684921183483098</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>1.557445099496081</t>
+          <t>2.274751695723469</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>0.4129512819912602</t>
+          <t>0.40410123804115017</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>18.026192195771937</t>
+          <t>11.376205793723948</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>1.0197857985061631</t>
+          <t>0.9371551433523136</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>7.908897344514294</t>
+          <t>9.425555253086095</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>0.5441218868840588</t>
+          <t>0.2540746158083268</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.4505442357153466</t>
+          <t>0.37522150874562854</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>25.835186114695226</t>
+          <t>21.065993706081237</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>18.69804525575301</t>
+          <t>13.806791466707342</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>1.4805535444795028</t>
+          <t>1.3188034479569666</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>1.7524906584082793</t>
+          <t>1.5938272176711499</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>14.941924586360429</t>
+          <t>15.502743218200175</t>
         </is>
       </c>
     </row>
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>3.654591517749436</t>
+          <t>1.2935127414785499</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>5.941883371270137</t>
+          <t>6.340654279812104</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>0.7381494706441623</t>
+          <t>0.7443776285559229</t>
         </is>
       </c>
     </row>
@@ -9417,12 +9417,12 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>0.3341980140784644</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9444,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>2.140669487954284</t>
+          <t>2.012828243440964</t>
         </is>
       </c>
     </row>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>14.319069651766263</t>
+          <t>13.572055476622399</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>1.430926449609314</t>
+          <t>0.5421105686698535</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>14.596493570951088</t>
+          <t>11.117194272307806</t>
         </is>
       </c>
     </row>
@@ -9598,7 +9598,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>3.654704020379169</t>
+          <t>3.0984460862991003</t>
         </is>
       </c>
     </row>
@@ -9620,7 +9620,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>1.735665651178464</t>
+          <t>1.2434106247437178</t>
         </is>
       </c>
     </row>
@@ -9708,7 +9708,7 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>1.8068785235449636</t>
+          <t>1.8164132643089328</t>
         </is>
       </c>
     </row>
@@ -9752,7 +9752,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>1.7054856849236</t>
+          <t>1.7243745890478088</t>
         </is>
       </c>
     </row>
@@ -9774,7 +9774,7 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>34.58123421150158</t>
+          <t>18.94415563383503</t>
         </is>
       </c>
     </row>
@@ -9906,7 +9906,7 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>3.258070053958848</t>
+          <t>3.3235164260973233</t>
         </is>
       </c>
     </row>
@@ -10016,7 +10016,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>13.061941185080272</t>
+          <t>5.1139398853772775</t>
         </is>
       </c>
     </row>
@@ -10038,7 +10038,7 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>4.183979927484203</t>
+          <t>3.6372851195674443</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10060,7 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>1.379184056810845</t>
+          <t>0.6829415694635803</t>
         </is>
       </c>
     </row>
@@ -10192,7 +10192,7 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>17.540517895605312</t>
+          <t>14.32505588848148</t>
         </is>
       </c>
     </row>
@@ -10214,7 +10214,7 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>10.63456096563458</t>
+          <t>4.531112033504467</t>
         </is>
       </c>
     </row>
@@ -10236,7 +10236,7 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>17.212470622612564</t>
+          <t>18.884953747907993</t>
         </is>
       </c>
     </row>
@@ -10258,7 +10258,7 @@
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>12.39381756151565</t>
+          <t>13.923699052962933</t>
         </is>
       </c>
     </row>
@@ -10302,7 +10302,7 @@
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t>13.929388200328614</t>
+          <t>11.003232888903842</t>
         </is>
       </c>
     </row>
@@ -10324,7 +10324,7 @@
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>33.51480947617925</t>
+          <t>19.314597826013333</t>
         </is>
       </c>
     </row>
@@ -10346,7 +10346,7 @@
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>19.709106453454027</t>
+          <t>31.048056670846755</t>
         </is>
       </c>
     </row>
@@ -10368,7 +10368,7 @@
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t>11.884599361585714</t>
+          <t>12.0862108482079</t>
         </is>
       </c>
     </row>
@@ -10478,7 +10478,7 @@
       </c>
       <c r="D457" t="inlineStr">
         <is>
-          <t>6.88605698422062</t>
+          <t>7.953030322261773</t>
         </is>
       </c>
     </row>
@@ -10500,7 +10500,7 @@
       </c>
       <c r="D458" t="inlineStr">
         <is>
-          <t>12.74744831472148</t>
+          <t>13.00694348007828</t>
         </is>
       </c>
     </row>
@@ -10522,7 +10522,7 @@
       </c>
       <c r="D459" t="inlineStr">
         <is>
-          <t>5.739560661181159</t>
+          <t>8.29142668706406</t>
         </is>
       </c>
     </row>
@@ -10544,7 +10544,73 @@
       </c>
       <c r="D460" t="inlineStr">
         <is>
-          <t>2.3359047727832234</t>
+          <t>1.9625362295311817</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="1" t="inlineStr">
+        <is>
+          <t>460</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>DF_INT_UI_Goku</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="1" t="inlineStr">
+        <is>
+          <t>461</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>BU_STR_Yakon</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>21.21216525592952</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="1" t="inlineStr">
+        <is>
+          <t>462</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>DF_TEQ_Dabura</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>36.47121351709307</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Beast Gohan and skip summons
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D476"/>
+  <dimension ref="A1:D478"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.2905632293825318</t>
+          <t>0.31650924155502724</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.2456671490844652</t>
+          <t>0.2684108139209787</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.3882823136363554</t>
+          <t>0.4229542081406337</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.1396882309080298</t>
+          <t>0.15216177254368723</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.3882823136363554</t>
+          <t>0.4229542081406337</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0.05986638467486991</t>
+          <t>0.06521218823300882</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.3882823136363554</t>
+          <t>0.4229542081406337</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0.1789925395520899</t>
+          <t>0.19497578223518347</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.339747024431811</t>
+          <t>0.3700849321230546</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>0.6705035083585429</t>
+          <t>0.7303765082096987</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>0.2651432340024182</t>
+          <t>0.2888193529370156</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>0.16284245599102326</t>
+          <t>0.17738356759114152</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.07828648739361879</t>
+          <t>0.08527712471263962</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0.15908594040145085</t>
+          <t>0.1732916117622093</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>0.35788108522797163</t>
+          <t>0.3898382844006383</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>0.2416183522347084</t>
+          <t>0.2631938032011029</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.2416183522347084</t>
+          <t>0.2631938032011029</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0.2416183522347084</t>
+          <t>0.2631938032011029</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0.2416183522347084</t>
+          <t>0.2631938032011029</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.09454631174401633</t>
+          <t>0.10298887951347505</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>0.2416183522347084</t>
+          <t>0.2631938032011029</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>0.2416183522347084</t>
+          <t>0.2631938032011029</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>0.2416183522347084</t>
+          <t>0.2631938032011029</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.09454631174401633</t>
+          <t>0.10298887951347505</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0.2416183522347084</t>
+          <t>0.2631938032011029</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>0.24248711305964277</t>
+          <t>0.26414014052801454</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.32331615074619036</t>
+          <t>0.3521868540373527</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>0.18610566398974085</t>
+          <t>0.20272407724701882</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>0.08838107800080604</t>
+          <t>0.09627311764567184</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>0.05811264587650635</t>
+          <t>0.06330184831100545</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>0.037877604857488305</t>
+          <t>0.04125990756243079</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>0.16284245599102326</t>
+          <t>0.17738356759114152</t>
         </is>
       </c>
     </row>
@@ -2844,7 +2844,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>0.09578621547979183</t>
+          <t>0.10433950117281408</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>0.29800155927046346</t>
+          <t>0.3246117814265327</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>0.10303081162407458</t>
+          <t>0.11223100773361382</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>0.10646005472205765</t>
+          <t>0.11596646708391407</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>0.1396882309080298</t>
+          <t>0.15216177254368723</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>0.11354415974898012</t>
+          <t>0.12368315137990094</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3240,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>0.1490440766108807</t>
+          <t>0.16235305391747973</t>
         </is>
       </c>
     </row>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>0.11774949899894238</t>
+          <t>0.12826400883841577</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>0.15139221299864017</t>
+          <t>0.16491086850653458</t>
         </is>
       </c>
     </row>
@@ -3741,12 +3741,12 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>1.2342857142857142</t>
+          <t>0.36</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>0.12452709830679934</t>
+          <t>0.13564681780929738</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>0.2235011694528476</t>
+          <t>0.2434588360698995</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>0.09</t>
+          <t>0.09129706352621231</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>0.07359343687433899</t>
+          <t>0.08016500552400986</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>0.05966417985069664</t>
+          <t>0.06499192741172781</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>0.05302864680048362</t>
+          <t>0.05776387058740311</t>
         </is>
       </c>
     </row>
@@ -4428,7 +4428,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>0.17433793762951907</t>
+          <t>0.18990554493301634</t>
         </is>
       </c>
     </row>
@@ -4494,7 +4494,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>0.15139221299864017</t>
+          <t>0.16491086850653458</t>
         </is>
       </c>
     </row>
@@ -4912,7 +4912,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>0.05479363455676222</t>
+          <t>0.05968646394954596</t>
         </is>
       </c>
     </row>
@@ -4934,7 +4934,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>0.044156062124603386</t>
+          <t>0.048099003314405926</t>
         </is>
       </c>
     </row>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>0.15139221299864017</t>
+          <t>0.16491086850653458</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.3567025226470033</t>
+          <t>0.38855448139011944</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>0.054280818663674416</t>
+          <t>0.05912785586371383</t>
         </is>
       </c>
     </row>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>0.02129201094441152</t>
+          <t>0.02319329341678281</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>0.1277520656664691</t>
+          <t>0.13915976050069684</t>
         </is>
       </c>
     </row>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>0.06641445243029298</t>
+          <t>0.07234496949829193</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>0.04519872457061606</t>
+          <t>0.04923477090855979</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>0.05811264587650635</t>
+          <t>0.06330184831100542</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.04981083932271973</t>
+          <t>0.054258727123718944</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>0.04519872457061606</t>
+          <t>0.04923477090855979</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>0.1509986775252493</t>
+          <t>0.16448219205469083</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>0.05046407099954673</t>
+          <t>0.05497028950217818</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>0.09672280274913124</t>
+          <t>0.10535972154584153</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.06728542799939564</t>
+          <t>0.07329371933623759</t>
         </is>
       </c>
     </row>
@@ -7244,7 +7244,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>0.03784805324966005</t>
+          <t>0.04122771712663364</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>0.1634133783229912</t>
+          <t>0.178005470764031</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>0.026095495797872934</t>
+          <t>0.028425708237546546</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.030417158492016448</t>
+          <t>0.03313327630968972</t>
         </is>
       </c>
     </row>
@@ -9356,7 +9356,7 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>0.02767268851262207</t>
+          <t>0.03014373729095496</t>
         </is>
       </c>
     </row>
@@ -9532,7 +9532,7 @@
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>0.02020138925732709</t>
+          <t>0.022005284033296428</t>
         </is>
       </c>
     </row>
@@ -10897,6 +10897,50 @@
       <c r="D476" t="inlineStr">
         <is>
           <t>5.22</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="1" t="inlineStr">
+        <is>
+          <t>476</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>BU_INT_Super_Hero_Piccolo</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>3.28</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="1" t="inlineStr">
+        <is>
+          <t>477</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>DFLR_TEQ_Beast_Gohan</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>0.9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cell Max Banner and EZAs
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D478"/>
+  <dimension ref="A1:D479"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.325608465711452</t>
+          <t>0.48000000000000004</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.2761272715822972</t>
+          <t>0.2820067946412112</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.43511358500074243</t>
+          <t>0.44437837200131264</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.15653622325359873</t>
+          <t>0.15986931791281475</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.43511358500074243</t>
+          <t>0.44437837200131264</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0.06708695282297088</t>
+          <t>0.06851542196263488</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.43511358500074243</t>
+          <t>0.44437837200131264</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0.20058107937884925</t>
+          <t>0.204852012396917</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.38072438687564975</t>
+          <t>0.3888310755011487</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>0.7513738716172739</t>
+          <t>0.7673727259815107</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>0.29712252923662635</t>
+          <t>0.48000000000000004</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>0.18248311171581919</t>
+          <t>0.18636868830898726</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.08772872982016633</t>
+          <t>0.08959672021079738</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0.17827351754197582</t>
+          <t>0.18206946008388936</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>0.40104562203504607</t>
+          <t>0.4095850066779309</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>0.27076027867001096</t>
+          <t>0.27652552341659453</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.27076027867001096</t>
+          <t>0.27652552341659453</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0.27076027867001096</t>
+          <t>0.27652552341659453</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0.27076027867001096</t>
+          <t>0.27652552341659453</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.10594967426217819</t>
+          <t>0.10820563959779786</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>0.27076027867001096</t>
+          <t>0.27652552341659453</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>0.27076027867001096</t>
+          <t>0.27652552341659453</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>0.27076027867001096</t>
+          <t>0.27652552341659453</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.10594967426217819</t>
+          <t>0.10820563959779786</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0.27076027867001096</t>
+          <t>0.27652552341659453</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>0.2717338219496551</t>
+          <t>0.27751979615960803</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.3623117625995402</t>
+          <t>0.37002639487947736</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>0.20855212767522185</t>
+          <t>0.21299278663884252</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>0.09904084307887545</t>
+          <t>0.1011497000466052</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>0.06512169314229041</t>
+          <t>0.0665083163985576</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>0.042446075605232336</t>
+          <t>0.04334987144854509</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>0.18248311171581919</t>
+          <t>0.18636868830898726</t>
         </is>
       </c>
     </row>
@@ -2844,7 +2844,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>0.10733912451675343</t>
+          <t>0.10962467514021583</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>0.3339439429410107</t>
+          <t>0.34105454488067155</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>0.11545750150565132</t>
+          <t>0.11791591511520583</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>0.11930035039626517</t>
+          <t>0.1218405890227215</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>0.15653622325359873</t>
+          <t>0.15986931791281475</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>0.12723887921030957</t>
+          <t>0.1299481513514513</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3240,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>0.16702049055477125</t>
+          <t>0.17057682463181012</t>
         </is>
       </c>
     </row>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>0.13195143029217285</t>
+          <t>0.1347610458459495</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>0.16965183894707944</t>
+          <t>0.17326420180193505</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>0.139546485304908</t>
+          <t>0.14251782085405199</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>0.25045795720575803</t>
+          <t>0.25579090866050364</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>0.09392173395215925</t>
+          <t>0.09592159074768887</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>0.08246964393260808</t>
+          <t>0.08422565365371844</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>0.06686035979294974</t>
+          <t>0.06828400413230566</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>0.059424505847325275</t>
+          <t>0.06068982002796312</t>
         </is>
       </c>
     </row>
@@ -4428,7 +4428,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>0.19536507942687123</t>
+          <t>0.1995249491956728</t>
         </is>
       </c>
     </row>
@@ -4494,7 +4494,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>0.16965183894707944</t>
+          <t>0.17326420180193505</t>
         </is>
       </c>
     </row>
@@ -4912,7 +4912,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>0.06140237123842324</t>
+          <t>0.06270979971334194</t>
         </is>
       </c>
     </row>
@@ -4934,7 +4934,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>0.04948178635956484</t>
+          <t>0.05053539219223106</t>
         </is>
       </c>
     </row>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>0.16965183894707944</t>
+          <t>0.17326420180193505</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.3997249113775086</t>
+          <t>0.40823617439111487</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>0.06082770390527305</t>
+          <t>0.06212289610299575</t>
         </is>
       </c>
     </row>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>0.02386007007925303</t>
+          <t>0.024368117804544304</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>0.14316042047551816</t>
+          <t>0.1462087068272658</t>
         </is>
       </c>
     </row>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>0.07442479216261758</t>
+          <t>0.07600950445549438</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>0.05065020577733697</t>
+          <t>0.05172869053221146</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>0.06512169314229038</t>
+          <t>0.06650831639855759</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.05581859412196318</t>
+          <t>0.05700712834162079</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>0.05065020577733697</t>
+          <t>0.05172869053221146</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>0.16921083861139988</t>
+          <t>0.1728138113338439</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>0.0565506129823598</t>
+          <t>0.05775473393397835</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>0.10838867488285628</t>
+          <t>0.11069657337345852</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.07540081730981306</t>
+          <t>0.07700631191197115</t>
         </is>
       </c>
     </row>
@@ -7244,7 +7244,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>0.04241295973676985</t>
+          <t>0.04331605045048376</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>0.18312289378648083</t>
+          <t>0.18702209313199636</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>0.029242909940055437</t>
+          <t>0.029865573403599133</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.03408581439893289</t>
+          <t>0.03481159686363472</t>
         </is>
       </c>
     </row>
@@ -9356,7 +9356,7 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>0.031010330067757323</t>
+          <t>0.03167062685645599</t>
         </is>
       </c>
     </row>
@@ -9532,7 +9532,7 @@
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>0.02263790698945723</t>
+          <t>0.02311993143922404</t>
         </is>
       </c>
     </row>
@@ -10941,6 +10941,28 @@
       <c r="D478" t="inlineStr">
         <is>
           <t>0.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="1" t="inlineStr">
+        <is>
+          <t>478</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>CLR_AGL_Cell_Max</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>2.24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daima SS3 mini summons
</commit_message>
<xml_diff>
--- a/SummonRating.xlsx
+++ b/SummonRating.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D479"/>
+  <dimension ref="A1:D481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.2820067946412112</t>
+          <t>0.2950307580082668</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.44437837200131264</t>
+          <t>0.4649011670120507</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.15986931791281475</t>
+          <t>0.16725258732184334</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.44437837200131264</t>
+          <t>0.4649011670120507</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0.06851542196263488</t>
+          <t>0.07167968028079</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.44437837200131264</t>
+          <t>0.4649011670120507</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0.204852012396917</t>
+          <t>0.21431272453514566</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.3888310755011487</t>
+          <t>0.4067885211355446</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>0.24</t>
+          <t>0.41142857142857137</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>0.7673727259815107</t>
+          <t>0.8028124191448479</t>
         </is>
       </c>
     </row>
@@ -1365,12 +1365,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>0.13714285714285715</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>0.18636868830898726</t>
+          <t>0.19497578223518347</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0.08959672021079738</t>
+          <t>0.09373457938301474</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>0.18206946008388936</t>
+          <t>0.19047800208873375</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>0.4095850066779309</t>
+          <t>0.42850093432235303</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>0.27652552341659453</t>
+          <t>0.2892963443878255</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0.27652552341659453</t>
+          <t>0.2892963443878255</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0.27652552341659453</t>
+          <t>0.2892963443878255</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0.27652552341659453</t>
+          <t>0.2892963443878255</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0.10820563959779786</t>
+          <t>0.11320291736914909</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>0.27652552341659453</t>
+          <t>0.2892963443878255</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>0.27652552341659453</t>
+          <t>0.2892963443878255</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>0.27652552341659453</t>
+          <t>0.2892963443878255</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>0.10820563959779786</t>
+          <t>0.11320291736914909</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>0.27652552341659453</t>
+          <t>0.2892963443878255</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>0.27751979615960803</t>
+          <t>0.2903365357825449</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>0.37002639487947736</t>
+          <t>0.38711538104339327</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>0.21299278663884252</t>
+          <t>0.2228294654116382</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>0.1011497000466052</t>
+          <t>0.10582111227151876</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>0.0665083163985576</t>
+          <t>0.06957988025034845</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>0.04334987144854509</t>
+          <t>0.04535190525922233</t>
         </is>
       </c>
     </row>
@@ -2663,12 +2663,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>0.030000000000000002</t>
+          <t>0.02</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>0.18636868830898726</t>
+          <t>0.19497578223518347</t>
         </is>
       </c>
     </row>
@@ -2844,7 +2844,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>0.10962467514021583</t>
+          <t>0.11468748844926398</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>0.34105454488067155</t>
+          <t>0.35680551961993245</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>0.11791591511520583</t>
+          <t>0.1233616440410182</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>0.1218405890227215</t>
+          <t>0.12746757176996806</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>0.15986931791281475</t>
+          <t>0.16725258732184334</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>0.1299481513514513</t>
+          <t>0.13594956690234655</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3240,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>0.17057682463181012</t>
+          <t>0.1784546004779553</t>
         </is>
       </c>
     </row>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>0.1347610458459495</t>
+          <t>0.14098473604687786</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>0.17326420180193505</t>
+          <t>0.18126608920312876</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>0.14251782085405199</t>
+          <t>0.14909974339360382</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>0.25579090866050364</t>
+          <t>0.26760413971494934</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>0.09592159074768887</t>
+          <t>0.100351552393106</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>0.08422565365371844</t>
+          <t>0.08811546002929871</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>0.06828400413230566</t>
+          <t>0.07143757484504855</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>0.06068982002796312</t>
+          <t>0.06349266736291126</t>
         </is>
       </c>
     </row>
@@ -4428,7 +4428,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>0.1995249491956728</t>
+          <t>0.20873964075104537</t>
         </is>
       </c>
     </row>
@@ -4494,7 +4494,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>0.17326420180193505</t>
+          <t>0.18126608920312876</t>
         </is>
       </c>
     </row>
@@ -4912,7 +4912,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>0.06270979971334194</t>
+          <t>0.06560593608218744</t>
         </is>
       </c>
     </row>
@@ -4934,7 +4934,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>0.05053539219223106</t>
+          <t>0.05286927601757922</t>
         </is>
       </c>
     </row>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>0.17326420180193505</t>
+          <t>0.18126608920312876</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>0.40823617439111487</t>
+          <t>0.4270898087056399</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>0.06212289610299575</t>
+          <t>0.06499192741172781</t>
         </is>
       </c>
     </row>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>0.024368117804544304</t>
+          <t>0.02549351435399361</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>0.1462087068272658</t>
+          <t>0.15296108612396167</t>
         </is>
       </c>
     </row>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>0.07600950445549438</t>
+          <t>0.07951986314325533</t>
         </is>
       </c>
     </row>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>0.05172869053221146</t>
+          <t>0.05411768463915989</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>0.06650831639855759</t>
+          <t>0.06957988025034842</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>0.05700712834162079</t>
+          <t>0.059639897357441504</t>
         </is>
       </c>
     </row>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>0.05172869053221146</t>
+          <t>0.05411768463915989</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>0.1728138113338439</t>
+          <t>0.18079489828246423</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>0.05775473393397835</t>
+          <t>0.06042202973437622</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>0.11069657337345852</t>
+          <t>0.11580889032422109</t>
         </is>
       </c>
     </row>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>0.07700631191197115</t>
+          <t>0.08056270631250163</t>
         </is>
       </c>
     </row>
@@ -7244,7 +7244,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>0.04331605045048376</t>
+          <t>0.04531652230078216</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>0.18702209313199636</t>
+          <t>0.19565936335408485</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>0.029865573403599133</t>
+          <t>0.031244859794338237</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>0.03481159686363472</t>
+          <t>0.036419306219990864</t>
         </is>
       </c>
     </row>
@@ -9356,7 +9356,7 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>0.03167062685645599</t>
+          <t>0.03313327630968972</t>
         </is>
       </c>
     </row>
@@ -9532,7 +9532,7 @@
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>0.02311993143922404</t>
+          <t>0.024187682804918557</t>
         </is>
       </c>
     </row>
@@ -9769,12 +9769,12 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>1.9600000000000002</t>
+          <t>1.68</t>
         </is>
       </c>
     </row>
@@ -10963,6 +10963,50 @@
       <c r="D479" t="inlineStr">
         <is>
           <t>2.24</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="1" t="inlineStr">
+        <is>
+          <t>479</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>BU_AGL_Supreme_Kai_DAIMA</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>0.56</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="1" t="inlineStr">
+        <is>
+          <t>480</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>DF_PHY_SS3_Goku_Mini_DAIMA</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>5.22</t>
         </is>
       </c>
     </row>

</xml_diff>